<commit_message>
Actualización automática hashcode mié jul 28 02:23:51 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>6b5bef8bc5d42f9d30b95d561587e88f</t>
+    <t>d1207b34dd146200462e7eda16475e81</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -827,7 +827,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>1ccd1de32dbe005c6c1543b97ed022a1</t>
+    <t>0b9fdb77c2306ca15ea4882915c5cf03</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -857,7 +857,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>dc9a77fb31c24e9e863f6dda3027d276</t>
+    <t>4f59027b01f2608e46116dcf1e940da8</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>c2ba8bf17373c5f0cff1fce454cec82a</t>
+    <t>708e959fcd99233532b4e728b8ea2a45</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>54b0228258c692d7ac30c1cc315ffe1d</t>
+    <t>fa4da00ea6ea210b37afd666b7934289</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>7fa8cb2d6ddce7331b6da5a3bda30a3d</t>
+    <t>0d31be08e5da513f79cba3aad4e612db</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>b0ca006d6efc4a6a7f3e9e1e6ab99e9f</t>
+    <t>12aa2afe1312739cd170cfbbf6db4bca</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -2831,7 +2831,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>9f4900f2d329a3f8851e5ab2be6b0083</t>
+    <t>b405e7a5ca5f41363a4f948ad66e67e7</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2933,7 +2933,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>b06f4c56633310a66fe340ec26e8c64e</t>
+    <t>77c5e8202b4f1481937ffc3459066017</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3074,7 +3074,7 @@
     <t>03-030012TM</t>
   </si>
   <si>
-    <t>f2d7d4cbab759cdd14b8052ce5ef9dce</t>
+    <t>a40b31c1cb95200afe4345b7d66118f2</t>
   </si>
   <si>
     <t>01-080101-010089A</t>
@@ -4250,7 +4250,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>685853aadf29d8720ad77666b2bcd08a</t>
+    <t>97bddfc05a36601dd4f26294d424c8d5</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4265,7 +4265,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>c7b676b6fb3551cc5ef82efa3330934d</t>
+    <t>808d4c295a30aa62eac19de0f31ed5b2</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue jul 29 03:57:36 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -65,7 +65,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>1df51009c1b5367256f79b4c97a9aee7</t>
+    <t>ed9acce598ab85c41b400614a877078e</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -101,7 +101,7 @@
     <t>05-050207TP</t>
   </si>
   <si>
-    <t>09088a9949ad1a8f49e48e974ac83087</t>
+    <t>059e8f1eba321846fc43151850338435</t>
   </si>
   <si>
     <t>915-150012A</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>53601e0421ef0b80d2334b97bd351763</t>
+    <t>e4680b930d22d7d95a2e1aff9717d877</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -152,7 +152,7 @@
     <t>05-050316TC</t>
   </si>
   <si>
-    <t>27ea83e59e475359c7067824c461be37</t>
+    <t>95bc9b548276ae6f60dc29ef1264f8ed</t>
   </si>
   <si>
     <t>03-030059TP</t>
@@ -206,7 +206,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>cf0dc0e7bccb941d33745a261424c664</t>
+    <t>dce0b1f1d6ed8ddf2e03e86f90a23704</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -647,7 +647,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>25fbfe6bc6a3bd0a2084d71b2d872320</t>
+    <t>b314e5a1fa25c9d6ab436413067e54de</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -662,7 +662,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>4b993743580714c27f04099bacdaa06f</t>
+    <t>1a3f1505868feb8a19f6cbcdfc804738</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -680,7 +680,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>58f664ec13664584ee1ece5d81b44762</t>
+    <t>8926a7b4d2655f02eaa2160e49ef96ad</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -716,7 +716,7 @@
     <t>05-050312TP</t>
   </si>
   <si>
-    <t>fbec840e02f535bdf0b4b1cd69c2a46a</t>
+    <t>e57b169cf0d8d4048e0a76ea4204c296</t>
   </si>
   <si>
     <t>05-0709-070954TC</t>
@@ -731,7 +731,7 @@
     <t>05-050312TC</t>
   </si>
   <si>
-    <t>a435f31ba0bbe2506f40ac6402765640</t>
+    <t>5ad1bafd7c04cb5e92e04db29180a46e</t>
   </si>
   <si>
     <t>03-030055TP</t>
@@ -851,7 +851,7 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>d0df0a98d510e632eb5b028bbf2aba2d</t>
+    <t>2ca64185bfd6830fb10cf73cef34f560</t>
   </si>
   <si>
     <t>05-050007TP</t>
@@ -866,7 +866,7 @@
     <t>05-050308A</t>
   </si>
   <si>
-    <t>2b0269c464b59fe3dd3489ae566592a3</t>
+    <t>5ebc226671fdbd07110f027c3fd35fd4</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -899,7 +899,7 @@
     <t>05-050203TC</t>
   </si>
   <si>
-    <t>69e4cd9089eff13849e48dca5d55da53</t>
+    <t>57702b7921554deff2cd45ddaff45c4b</t>
   </si>
   <si>
     <t>01-110304-11030404A</t>
@@ -926,7 +926,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>82426963d2aca61c392b118ba5129933</t>
+    <t>9bfd60431b45d499946ababbedf265a1</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -953,7 +953,7 @@
     <t>05-050303TC</t>
   </si>
   <si>
-    <t>c861d4fd025db76c7afc46ce10a49f3f</t>
+    <t>4a357f852fdc44460a200c3a02cc839d</t>
   </si>
   <si>
     <t>01-010010TP</t>
@@ -971,7 +971,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>3b78150ff1fc474be866da618f4a7754</t>
+    <t>e8cf2322e0111a167c83cdbea9f3e3dd</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1013,7 +1013,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>0fa317cd20a5b49aad28226bf6df9533</t>
+    <t>38b9da908bdd75aafe2d3c826c744706</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1055,7 +1055,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>bd9f44647569b5e2f4c5ad711528b41a</t>
+    <t>b4022141fd796266c0e0b82f212f99c3</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1064,7 +1064,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>220fbe3e9aaef97d6c55ff34f5c02ce1</t>
+    <t>eccdb284fe64b1be028c8b68764282f5</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1133,7 +1133,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>bc91d4b0be812322444314f5443b41bc</t>
+    <t>f77883a5a8ff0fe4b0d11b07edf654ba</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1208,13 +1208,13 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>2e5855dc59a3d101c8e3dae40a359c00</t>
+    <t>57fc0dac869fb3f0d141891a6c9a10c8</t>
   </si>
   <si>
     <t>05-050304A</t>
   </si>
   <si>
-    <t>57ef2d6c399be2220cb6bf4e701a20f6</t>
+    <t>8b43d6eb180c63a16e926b8faf7aee0c</t>
   </si>
   <si>
     <t>05-050009TP</t>
@@ -1238,7 +1238,7 @@
     <t>05-050205TC</t>
   </si>
   <si>
-    <t>c4030331425f6bf729588605a470eb2c</t>
+    <t>1bb755195f22abb90b20e6847658bffb</t>
   </si>
   <si>
     <t>04-040014TM</t>
@@ -1307,7 +1307,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>78e8e5b4d35bc1dd3ceb6a351506c4bc</t>
+    <t>786ced3b59d255ed903db148049874c1</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1466,7 +1466,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>c60c197cb24578b07b6a78579336d15a</t>
+    <t>f68caf7517eec411d056e39f6a6bf8e9</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1496,7 +1496,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>6fb5b1881add52977736c6f8a650d8e7</t>
+    <t>853400072a9a923bb317833eb8e1029d</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1565,7 +1565,7 @@
     <t>05-050310TC</t>
   </si>
   <si>
-    <t>8f8bebfa3bf1f47dff51f2df564f140d</t>
+    <t>0ce4e02808b8b9e5627f74e5a070f157</t>
   </si>
   <si>
     <t>04-040004A</t>
@@ -1613,7 +1613,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>d91d562d5a99603c1c4c517bd16bc4d2</t>
+    <t>3d60a2d43a3866ef20089508a1ad4cca</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1748,7 +1748,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>9957746ca62d480b301fca0d3984ec02</t>
+    <t>e2f0a39e1ed7d8ae2482944dfdb5b15e</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -1769,7 +1769,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>eb4717392d96cb5d186e478cf51f188e</t>
+    <t>d9ddd5c3b6ddaab06f18a11561b69053</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -1793,7 +1793,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>d5a53b38dbb69a247d63cd2d60e28603</t>
+    <t>99e0624f512a37ca64da29d7ceea58e7</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -1901,7 +1901,7 @@
     <t>03-030070TC</t>
   </si>
   <si>
-    <t>884ca1dc8b42bf2cf75c1180c6035b0c</t>
+    <t>8d62e228cacd1180e9dc5effcf95158e</t>
   </si>
   <si>
     <t>05-0709-070906ATP</t>
@@ -1955,7 +1955,7 @@
     <t>03-030070TP</t>
   </si>
   <si>
-    <t>90954109c5d442f2adf8575dd44df35d</t>
+    <t>b144c9348c1ba9f4281b4caf0324bbcf</t>
   </si>
   <si>
     <t>01-080101-010084TC</t>
@@ -2165,7 +2165,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>9e126b63abb9a0b3dd5452a74c4fb13b</t>
+    <t>db02905784f29aa7e098ab09aa487438</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>0841f66eec1f7caf51680bed6f5054c6</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2348,7 +2348,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>102a560568012b479f3fa0a2bfad807a</t>
+    <t>2765c8f1c87dca50e2ff17335bb53c94</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2420,7 +2420,7 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>baf84d1cbe510866799112cbfcd7709b</t>
+    <t>6a52edd308d0914ca301e2258cd0169c</t>
   </si>
   <si>
     <t>05-050313A</t>
@@ -2519,7 +2519,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>6bef42abac4de6cc7407d8d26f62065a</t>
+    <t>7cae69c40117095f8c69f95634c88089</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2531,7 +2531,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>830064ea44c0d05c93a59723f7118ea2</t>
+    <t>d7c9eb3bb1ebb4a091388333d7bd2a92</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2612,7 +2612,7 @@
     <t>05-050208TC</t>
   </si>
   <si>
-    <t>d1484942ef08d715b335040b3a5e7c24</t>
+    <t>fab33c8231a9280e35833755f1a2078d</t>
   </si>
   <si>
     <t>03-030039A</t>
@@ -2657,13 +2657,13 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>af1498cfb98edd0fd3304919bc590619</t>
+    <t>4082473e455ea2efcc317070f655c008</t>
   </si>
   <si>
     <t>05-050311A</t>
   </si>
   <si>
-    <t>a72749e8a01d69815f877c9d567e2fd3</t>
+    <t>67ab01d296e75654c21f4739000e956c</t>
   </si>
   <si>
     <t>05-050208TP</t>
@@ -2693,7 +2693,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>067ca15bdc2bb75fdda992d4b749a669</t>
+    <t>2cfe0f1373d2ec03ad6aa6b88c28f516</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -2732,13 +2732,13 @@
     <t>05-050317TC</t>
   </si>
   <si>
-    <t>6c1aa9bb02a7b3c0cdde7e4b3fc07dbf</t>
+    <t>4bd2f562bbbac4f175d158a4b2977ab2</t>
   </si>
   <si>
     <t>05-050312A</t>
   </si>
   <si>
-    <t>e36cfc8d647d2ba777e89889eb5fd238</t>
+    <t>a89528d3176a4dbcfe7c017e954a5ab5</t>
   </si>
   <si>
     <t>05-050009A</t>
@@ -2750,7 +2750,7 @@
     <t>05-050203A</t>
   </si>
   <si>
-    <t>bcb473d3636ec9820ddc03661f7e42a7</t>
+    <t>c56df910e4fed527df2ddd7eb4892484</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -2789,7 +2789,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>d798c3c15221dcec831d881a939029c2</t>
+    <t>6d93fcf9e0612fa89a7a361894e88df5</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -2900,7 +2900,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>bfc8fc8f5e86b6db53dd5586d2a06e43</t>
+    <t>053e9979a929718be152a7b44a18f23b</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -2915,7 +2915,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>6dc98ce9ec631a34dbe0d8e750d5b178</t>
+    <t>7f53db899963dee22e9ba6497c61010b</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -2951,7 +2951,7 @@
     <t>03-030012A</t>
   </si>
   <si>
-    <t>c5c7c649b1403b6bd1a0e26b62810927</t>
+    <t>56c8d45a7d37b859645830d7ec698895</t>
   </si>
   <si>
     <t>03-030045TC</t>
@@ -2990,7 +2990,7 @@
     <t>05-050308TC</t>
   </si>
   <si>
-    <t>f6d27ccd73a65f0bdc5b05a571214f90</t>
+    <t>63ebd04f7f4961c0d42926a65412ba4a</t>
   </si>
   <si>
     <t>02-020002TC</t>
@@ -3008,7 +3008,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>b76fa55681ab244c650ea7ba30d7b660</t>
+    <t>fa298e244c4126c3d7361f58970d83c5</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3026,7 +3026,7 @@
     <t>03-030012TC</t>
   </si>
   <si>
-    <t>642e93137d04f203e5c272c3f7981b54</t>
+    <t>eb90b19323a5859efa320578d58c13a6</t>
   </si>
   <si>
     <t>03-030058TC</t>
@@ -3044,7 +3044,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>f19590d68f24b9b672fd3c539aab8343</t>
+    <t>6f945d891b1b07a146ded54fbb93459b</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3098,7 +3098,7 @@
     <t>03-030012TP</t>
   </si>
   <si>
-    <t>56b4e83a6888967e55ee50b24f18dba8</t>
+    <t>68cebef0e28dc8122bf6c530043b3209</t>
   </si>
   <si>
     <t>03-030058TM</t>
@@ -3116,7 +3116,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>ba39438bc23efc7a39321ed0bae1a377</t>
+    <t>8f584d73c1d2ae49a61f6dfe4800c4ef</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3275,7 +3275,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>14d050b2269d173538aed8d132a1567b</t>
+    <t>e161a2fa2ee9400f268f365465bde9d9</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3329,7 +3329,7 @@
     <t>05-050204TC</t>
   </si>
   <si>
-    <t>a2f2c89d8e61151db8e5d62a41e3d34c</t>
+    <t>61bfb6dfbb9345ec8f1be50c3d1d8590</t>
   </si>
   <si>
     <t>04-040015TM</t>
@@ -3365,7 +3365,7 @@
     <t>05-050302TC</t>
   </si>
   <si>
-    <t>6da39242dc3e342481be3b884dfb17d8</t>
+    <t>8681f7b889429514746ff6849c36e77e</t>
   </si>
   <si>
     <t>01-110304-11030403TP</t>
@@ -3518,7 +3518,7 @@
     <t>05-050317A</t>
   </si>
   <si>
-    <t>79ec90319fcd89f911fb8849489458d2</t>
+    <t>fca18a2901952950103d43ab77236f8c</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -3584,7 +3584,7 @@
     <t>05-050206TP</t>
   </si>
   <si>
-    <t>5451fc92aae3e5333e1e9e215b99d53d</t>
+    <t>52e22e2e5aa4e0749a78e40333915b33</t>
   </si>
   <si>
     <t>01-010068TM</t>
@@ -3608,7 +3608,7 @@
     <t>05-050206TC</t>
   </si>
   <si>
-    <t>ea6c1a53ffac560a970a1f9ab1584e81</t>
+    <t>2cad2a7bf53ea3238fa8405eecf65ea3</t>
   </si>
   <si>
     <t>04-040013TM</t>
@@ -3692,7 +3692,7 @@
     <t>05-050304TC</t>
   </si>
   <si>
-    <t>e7280d7791813b01dc8a9941481ce44d</t>
+    <t>09c2ea614878074519969e3138174001</t>
   </si>
   <si>
     <t>03-030043TP</t>
@@ -3704,13 +3704,13 @@
     <t>05-050206A</t>
   </si>
   <si>
-    <t>f96b1ebfe6616e0b52a80aaed3ce7e80</t>
+    <t>6be39dc7d3f370598bac8b3e04944505</t>
   </si>
   <si>
     <t>05-050315A</t>
   </si>
   <si>
-    <t>69e752efebe41c5f6e6b78c9585d5f64</t>
+    <t>ea364ee5492aec3427b2f883e19dea73</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -3773,7 +3773,7 @@
     <t>05-050304TP</t>
   </si>
   <si>
-    <t>363a4038010308db052655fb866438e4</t>
+    <t>0c351ffaffde51c6347d401a693f8eee</t>
   </si>
   <si>
     <t>04-040002TP</t>
@@ -3821,7 +3821,7 @@
     <t>05-050315TC</t>
   </si>
   <si>
-    <t>952382d47d10bd78b5a7cebabbc8493e</t>
+    <t>4f3388340ea7f4a2af6d438266c16a79</t>
   </si>
   <si>
     <t>01-010046TM</t>
@@ -3836,7 +3836,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>00befa18721ee13a08f8b9160e59350c</t>
+    <t>1dfdd5679f7ee319e320d406aa4ca709</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -3860,7 +3860,7 @@
     <t>05-050207A</t>
   </si>
   <si>
-    <t>c9d8ad33e3779fce70cd4c812e3a58e9</t>
+    <t>d9f4f2892bdd8d80380caf4dcc428307</t>
   </si>
   <si>
     <t>02-020006TM</t>
@@ -3911,7 +3911,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>9c12e2aaa7853b75756fbbc3d8715c29</t>
+    <t>44e3088d57e75072827ee3ee130b7943</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -3983,7 +3983,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>97f9a506bab813cf629d1c01b94a73cb</t>
+    <t>05089a667705b6ff52f21f0a6990ad9b</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4004,7 +4004,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>1251070858590fb23d481929357c7bbd</t>
+    <t>41bf80ef7c81b0a5661624678ccde1ca</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4109,7 +4109,7 @@
     <t>03-030071A</t>
   </si>
   <si>
-    <t>a55cd841ae22817e9d8e75e6235c48a7</t>
+    <t>bc215835c85ba728793c88004710b458</t>
   </si>
   <si>
     <t>915-150010TP</t>
@@ -4133,7 +4133,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>e8813c180153e8e2f7458d7d4691e535</t>
+    <t>b0c2a18df112b9f277fecaa6a1e00eb7</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4175,7 +4175,7 @@
     <t>03-030070A</t>
   </si>
   <si>
-    <t>13a58843e6c5aa259a24eb42e4c67fbc</t>
+    <t>2ef08e05d9da3935517d358309018e8d</t>
   </si>
   <si>
     <t>03-02010301-030083TM</t>
@@ -4286,7 +4286,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>1434c9f69be3cb90e050bb47d6d9121f</t>
+    <t>7f3c93123e6807038cd5a33a137219fe</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>
@@ -4343,7 +4343,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>e25302e57621436b50037185e826bdbf</t>
+    <t>9ac516dcbe0b313e4b36eb8426ea47b9</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4370,7 +4370,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>58589a08c5d5c3408b928146f58a5795</t>
+    <t>1affb1ed2822a12b159e8df078bf0975</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -4469,13 +4469,13 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>8f893dcb52b1e47d448c2b51b718df3e</t>
+    <t>6ca08574d86ae3aa9d7e5c47c265b84a</t>
   </si>
   <si>
     <t>05-050002A</t>
   </si>
   <si>
-    <t>58fbeb8b4138f0d93bf09bb62d1abeda</t>
+    <t>42ae2ecbbe95475185886ba7eb9ed1f7</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4505,7 +4505,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>4ab28706ee1ae6eb91108014bebc7fe6</t>
+    <t>4674a84d8a29ca83aa949ac49fbfc93a</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -4532,7 +4532,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>46c088441dbb7bf6222b524c5aeedd6c</t>
+    <t>6f6df58ed26c3b04d4a1451cd1752a17</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4640,7 +4640,7 @@
     <t>03-030071TC</t>
   </si>
   <si>
-    <t>402455665a127b9c85bbd42f906ecf74</t>
+    <t>4a30d67ce0a5cdc8693422460434cffe</t>
   </si>
   <si>
     <t>915-150014TC</t>
@@ -4688,7 +4688,7 @@
     <t>03-030071TP</t>
   </si>
   <si>
-    <t>ab434232503911719a501da4bb02d3c9</t>
+    <t>1ce9255c51d6bdec0678e73941c7577d</t>
   </si>
   <si>
     <t>915-150003TP</t>
@@ -4736,7 +4736,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>f3f6811874ecdc67316e05785138873c</t>
+    <t>f39c13e6a0c461b855c0c6328d15b4d7</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -4871,7 +4871,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>f793cf1af20f3a85061e0db0c3134e3b</t>
+    <t>e64797a2cb3edeb4ee2d3a9ac5c7bd75</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie jul 30 05:29:44 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>0841f66eec1f7caf51680bed6f5054c6</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2669,7 +2669,7 @@
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>cbe53266bb0cce4d0fe1a366ae1aa4da</t>
+    <t>6e7a711ccd7d38b00285bd320bf93cfa</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -3338,7 +3338,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>76119c28981c4dbf23c59f7a8cfc6fd9</t>
+    <t>197c0b9cfac61b90cfd77d9e3b15133c</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3512,7 +3512,7 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>5894348331bb6e1528cc7c651402a1b7</t>
+    <t>85cdec942922fd1be3bcf4d0623befca</t>
   </si>
   <si>
     <t>05-050317A</t>
@@ -4325,7 +4325,7 @@
     <t>05-050202TC</t>
   </si>
   <si>
-    <t>656faa7679774432e51d07f4641ddc9d</t>
+    <t>ec29680cb56f42a64a35dbc3449c2575</t>
   </si>
   <si>
     <t>03-030062TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode lun ago  2 06:14:24 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1457,7 +1457,7 @@
     <t>05-050003TM</t>
   </si>
   <si>
-    <t>5479388ebbf116e5c648f81165e5b532</t>
+    <t>a996d4ebbf0fd8d2ceecd7b76c1e4798</t>
   </si>
   <si>
     <t>01-010025TM</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>0841f66eec1f7caf51680bed6f5054c6</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié ago  4 00:58:01 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>d1207b34dd146200462e7eda16475e81</t>
+    <t>408047ce987223fba9f85e8d7dda986f</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -533,7 +533,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>4a75f014e6cf8b2a6884a8454b7d349c</t>
+    <t>57287b73631d1dd0760a97d7f3caac2e</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -584,7 +584,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>30587d204d5fa418df4b30ce24416406</t>
+    <t>6de338d5b96f4c93b6ec4bb89b59161e</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -827,7 +827,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>0b9fdb77c2306ca15ea4882915c5cf03</t>
+    <t>84f9177b78615335c74de6904e2acd32</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -857,7 +857,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>4f59027b01f2608e46116dcf1e940da8</t>
+    <t>ab0ea17fae2aec0703ccc1e868a613be</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1478,7 +1478,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>949da19d905f5c0164705cdbf138b039</t>
+    <t>3e99b032c7ffd9082e7b4646ae3134b8</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>0841f66eec1f7caf51680bed6f5054c6</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2426,7 +2426,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>b5e4fb67b34969403b416ddbb15a1d24</t>
+    <t>1e9f650233b1837146e626f3c41edea3</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2831,7 +2831,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>b405e7a5ca5f41363a4f948ad66e67e7</t>
+    <t>568f02ee5c11b452a06580198ae3fcfd</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2933,7 +2933,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>77c5e8202b4f1481937ffc3459066017</t>
+    <t>df33604063d2187b012a3a687c78f6f7</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3440,7 +3440,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>9f8ae3fc79ca25eb516e02c7d8e9e1ed</t>
+    <t>3c97d05e668859254bf07149cb1a8d06</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3467,7 +3467,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>25bb50cf2142c3c1efc9273f65308156</t>
+    <t>ed84dfdffacedeec79d20a683308511e</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4040,7 +4040,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>e8973709aee26ae01b8b5a785784a646</t>
+    <t>90c03a7dd9cf250bec609eba72199372</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4250,7 +4250,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>97bddfc05a36601dd4f26294d424c8d5</t>
+    <t>ad6e173e9e187d4df9db4e9e93687c24</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4265,7 +4265,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>808d4c295a30aa62eac19de0f31ed5b2</t>
+    <t>3a4d48d91fc07d0a8fd7f12c5d10e8e5</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue ago  5 02:29:13 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -179,7 +179,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>0c865616e57da7ff865bf8e20b4bcf2f</t>
+    <t>a6ed462f4b3da22413d958a0e0aa216f</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -647,7 +647,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>b314e5a1fa25c9d6ab436413067e54de</t>
+    <t>50799c60fdb747d4279d38bd5b03aeb8</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>708e959fcd99233532b4e728b8ea2a45</t>
+    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>fa4da00ea6ea210b37afd666b7934289</t>
+    <t>fe069915e6896d5ed070ddbadaac6446</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>0d31be08e5da513f79cba3aad4e612db</t>
+    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1748,7 +1748,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>e2f0a39e1ed7d8ae2482944dfdb5b15e</t>
+    <t>b0ac4930ec15dbac39af731b9db4768c</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -1769,7 +1769,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>d9ddd5c3b6ddaab06f18a11561b69053</t>
+    <t>2270685ec7d3a5468017dba19d33c2bd</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2612,7 +2612,7 @@
     <t>05-050208TC</t>
   </si>
   <si>
-    <t>fab33c8231a9280e35833755f1a2078d</t>
+    <t>4b1b942b40330cd0cc3ceb2b49128d69</t>
   </si>
   <si>
     <t>03-030039A</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>12aa2afe1312739cd170cfbbf6db4bca</t>
+    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -3116,7 +3116,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>8f584d73c1d2ae49a61f6dfe4800c4ef</t>
+    <t>887e5ce461f76ef5d09805b2e0f0c8c3</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie ago  6 05:02:23 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -65,7 +65,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>ed9acce598ab85c41b400614a877078e</t>
+    <t>bf88958680fd0ad4437263ca6fdb297f</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -101,7 +101,7 @@
     <t>05-050207TP</t>
   </si>
   <si>
-    <t>059e8f1eba321846fc43151850338435</t>
+    <t>3f566850f7e1fb5e14efe24cd9262168</t>
   </si>
   <si>
     <t>915-150012A</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>e4680b930d22d7d95a2e1aff9717d877</t>
+    <t>3be5860e231c20fa27df04eb4ca8cf98</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -152,7 +152,7 @@
     <t>05-050316TC</t>
   </si>
   <si>
-    <t>95bc9b548276ae6f60dc29ef1264f8ed</t>
+    <t>6bf83fd50321eed05183fd05dcc29b85</t>
   </si>
   <si>
     <t>03-030059TP</t>
@@ -206,7 +206,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>dce0b1f1d6ed8ddf2e03e86f90a23704</t>
+    <t>bdfa6c8d82452f12b312fe16aed392ed</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -680,7 +680,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>8926a7b4d2655f02eaa2160e49ef96ad</t>
+    <t>dc47d7dcb14346d6d0beb3cbf823be31</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -716,7 +716,7 @@
     <t>05-050312TP</t>
   </si>
   <si>
-    <t>e57b169cf0d8d4048e0a76ea4204c296</t>
+    <t>9630a8476f259b238c150ab3f99edf8e</t>
   </si>
   <si>
     <t>05-0709-070954TC</t>
@@ -731,7 +731,7 @@
     <t>05-050312TC</t>
   </si>
   <si>
-    <t>5ad1bafd7c04cb5e92e04db29180a46e</t>
+    <t>ff88d21c9f0b469b698693cda95351e9</t>
   </si>
   <si>
     <t>03-030055TP</t>
@@ -851,7 +851,7 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>2ca64185bfd6830fb10cf73cef34f560</t>
+    <t>d54dc554914eb3eb482791129a9f1b55</t>
   </si>
   <si>
     <t>05-050007TP</t>
@@ -866,7 +866,7 @@
     <t>05-050308A</t>
   </si>
   <si>
-    <t>5ebc226671fdbd07110f027c3fd35fd4</t>
+    <t>cc991a52b705db26dc7a0813407aaf1f</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -899,7 +899,7 @@
     <t>05-050203TC</t>
   </si>
   <si>
-    <t>57702b7921554deff2cd45ddaff45c4b</t>
+    <t>460ad78a8776f06c7aa8601798efa385</t>
   </si>
   <si>
     <t>01-110304-11030404A</t>
@@ -926,7 +926,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>9bfd60431b45d499946ababbedf265a1</t>
+    <t>1003d58c916678b64c8fb9bc851634d1</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -953,7 +953,7 @@
     <t>05-050303TC</t>
   </si>
   <si>
-    <t>4a357f852fdc44460a200c3a02cc839d</t>
+    <t>dacbadc0a71781aab84d5510eb2d5a3a</t>
   </si>
   <si>
     <t>01-010010TP</t>
@@ -971,7 +971,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>e8cf2322e0111a167c83cdbea9f3e3dd</t>
+    <t>20690ceb1cad475a5b571ca87e928d06</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1013,7 +1013,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>38b9da908bdd75aafe2d3c826c744706</t>
+    <t>88af5bf5ace7bc9f41425d4f63be1fa2</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1055,7 +1055,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>b4022141fd796266c0e0b82f212f99c3</t>
+    <t>701ed1d847fae8c7ccd569fc1d79d15f</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1064,7 +1064,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>eccdb284fe64b1be028c8b68764282f5</t>
+    <t>77f66364cc88cbdc1a18e276684ad447</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1133,7 +1133,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>f77883a5a8ff0fe4b0d11b07edf654ba</t>
+    <t>149517503b59ddfc3918c862b96b3067</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1208,13 +1208,13 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>57fc0dac869fb3f0d141891a6c9a10c8</t>
+    <t>09dc94ef4f361581164ab3997e67c878</t>
   </si>
   <si>
     <t>05-050304A</t>
   </si>
   <si>
-    <t>8b43d6eb180c63a16e926b8faf7aee0c</t>
+    <t>09420b52977612a4d86a279f940ff25d</t>
   </si>
   <si>
     <t>05-050009TP</t>
@@ -1238,7 +1238,7 @@
     <t>05-050205TC</t>
   </si>
   <si>
-    <t>1bb755195f22abb90b20e6847658bffb</t>
+    <t>add83c8ffd62b5c5fff7be16dae8afaf</t>
   </si>
   <si>
     <t>04-040014TM</t>
@@ -1307,7 +1307,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>786ced3b59d255ed903db148049874c1</t>
+    <t>e0c82a61a67245f79968a744f7b09936</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1466,7 +1466,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>f68caf7517eec411d056e39f6a6bf8e9</t>
+    <t>659242aec416d17e85f02ecbb12330d9</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1496,7 +1496,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>853400072a9a923bb317833eb8e1029d</t>
+    <t>66a9960dc0d88e04f3a96d58130f043c</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1565,7 +1565,7 @@
     <t>05-050310TC</t>
   </si>
   <si>
-    <t>0ce4e02808b8b9e5627f74e5a070f157</t>
+    <t>60115817a4a3be48293379683941555f</t>
   </si>
   <si>
     <t>04-040004A</t>
@@ -1613,7 +1613,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>3d60a2d43a3866ef20089508a1ad4cca</t>
+    <t>4fcc2830cebe5ef789159e5ea8813780</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1793,7 +1793,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>99e0624f512a37ca64da29d7ceea58e7</t>
+    <t>0f1b7e48d003129c49d1a2059acc209b</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2165,7 +2165,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>db02905784f29aa7e098ab09aa487438</t>
+    <t>2e53c6037ada0a5f4509b5c48de7db82</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2348,7 +2348,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>2765c8f1c87dca50e2ff17335bb53c94</t>
+    <t>cd6d4751cda79df64f498f4b24da5db7</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2420,7 +2420,7 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>6a52edd308d0914ca301e2258cd0169c</t>
+    <t>ac412a65c65171b2378eada58b4f3bd5</t>
   </si>
   <si>
     <t>05-050313A</t>
@@ -2519,7 +2519,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>7cae69c40117095f8c69f95634c88089</t>
+    <t>90ab25c4405ead4ee0afe1b9d14f2107</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2531,7 +2531,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>d7c9eb3bb1ebb4a091388333d7bd2a92</t>
+    <t>2d6ceb7203356c3b73893edf9cda7000</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2663,13 +2663,13 @@
     <t>05-050311A</t>
   </si>
   <si>
-    <t>67ab01d296e75654c21f4739000e956c</t>
+    <t>00659defee040ed572c29c341ea04db5</t>
   </si>
   <si>
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>6e7a711ccd7d38b00285bd320bf93cfa</t>
+    <t>1715ab406c35b7c24e90dcbb31ace64b</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -2693,7 +2693,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>2cfe0f1373d2ec03ad6aa6b88c28f516</t>
+    <t>e71bf6219416afaac82fb6bc9f5e2fa3</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -2732,13 +2732,13 @@
     <t>05-050317TC</t>
   </si>
   <si>
-    <t>4bd2f562bbbac4f175d158a4b2977ab2</t>
+    <t>7067f67b2942213b4d4713364e70ae2e</t>
   </si>
   <si>
     <t>05-050312A</t>
   </si>
   <si>
-    <t>a89528d3176a4dbcfe7c017e954a5ab5</t>
+    <t>a9630c418c3f59d6a1b0b360a841ebf0</t>
   </si>
   <si>
     <t>05-050009A</t>
@@ -2750,7 +2750,7 @@
     <t>05-050203A</t>
   </si>
   <si>
-    <t>c56df910e4fed527df2ddd7eb4892484</t>
+    <t>60ddfdefed4769e4fc5a58fc7044c3e5</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -2789,7 +2789,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>6d93fcf9e0612fa89a7a361894e88df5</t>
+    <t>229410bf60ee30df3fa138b86e565bc4</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -2900,7 +2900,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>053e9979a929718be152a7b44a18f23b</t>
+    <t>7f4dc12e25c618f37e507de07c1df792</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -2915,7 +2915,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>7f53db899963dee22e9ba6497c61010b</t>
+    <t>41669038dfc6b535dfbec046e1d33aa1</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -2990,7 +2990,7 @@
     <t>05-050308TC</t>
   </si>
   <si>
-    <t>63ebd04f7f4961c0d42926a65412ba4a</t>
+    <t>c6b34662dbb3d73f48d62ae6dbde660d</t>
   </si>
   <si>
     <t>02-020002TC</t>
@@ -3008,7 +3008,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>fa298e244c4126c3d7361f58970d83c5</t>
+    <t>134162bc7e138f3db345fa90ad9f1a3d</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3044,7 +3044,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>6f945d891b1b07a146ded54fbb93459b</t>
+    <t>e6f48497af448ef49af760d78c76a34e</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3275,7 +3275,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>e161a2fa2ee9400f268f365465bde9d9</t>
+    <t>f27901d9c6928abaa5448bc98fd3c169</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3329,7 +3329,7 @@
     <t>05-050204TC</t>
   </si>
   <si>
-    <t>61bfb6dfbb9345ec8f1be50c3d1d8590</t>
+    <t>29a2a7a244786b74b0f5a6bbb50b99de</t>
   </si>
   <si>
     <t>04-040015TM</t>
@@ -3365,7 +3365,7 @@
     <t>05-050302TC</t>
   </si>
   <si>
-    <t>8681f7b889429514746ff6849c36e77e</t>
+    <t>72c1a8e6f3d566ecac609952c138676c</t>
   </si>
   <si>
     <t>01-110304-11030403TP</t>
@@ -3512,13 +3512,13 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>85cdec942922fd1be3bcf4d0623befca</t>
+    <t>4a0a1f70e7364e195cef4517668fda56</t>
   </si>
   <si>
     <t>05-050317A</t>
   </si>
   <si>
-    <t>fca18a2901952950103d43ab77236f8c</t>
+    <t>8698bccf05cce2f5667bf3d4c8455e29</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -3584,7 +3584,7 @@
     <t>05-050206TP</t>
   </si>
   <si>
-    <t>52e22e2e5aa4e0749a78e40333915b33</t>
+    <t>a6c0778e5c6025b5eca2a3b5364d1036</t>
   </si>
   <si>
     <t>01-010068TM</t>
@@ -3608,7 +3608,7 @@
     <t>05-050206TC</t>
   </si>
   <si>
-    <t>2cad2a7bf53ea3238fa8405eecf65ea3</t>
+    <t>e0fadaae9e7a01f3914884584a6b7517</t>
   </si>
   <si>
     <t>04-040013TM</t>
@@ -3692,7 +3692,7 @@
     <t>05-050304TC</t>
   </si>
   <si>
-    <t>09c2ea614878074519969e3138174001</t>
+    <t>c4fe35ca784828d1893f420a8d6d2832</t>
   </si>
   <si>
     <t>03-030043TP</t>
@@ -3704,13 +3704,13 @@
     <t>05-050206A</t>
   </si>
   <si>
-    <t>6be39dc7d3f370598bac8b3e04944505</t>
+    <t>ef1f7bc09084fe7e760fcd662b2c9eec</t>
   </si>
   <si>
     <t>05-050315A</t>
   </si>
   <si>
-    <t>ea364ee5492aec3427b2f883e19dea73</t>
+    <t>432f2b12e1f6894d2d49d0752077aa1d</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -3773,7 +3773,7 @@
     <t>05-050304TP</t>
   </si>
   <si>
-    <t>0c351ffaffde51c6347d401a693f8eee</t>
+    <t>62150c20d121c8274d6f90ed3903f51d</t>
   </si>
   <si>
     <t>04-040002TP</t>
@@ -3821,7 +3821,7 @@
     <t>05-050315TC</t>
   </si>
   <si>
-    <t>4f3388340ea7f4a2af6d438266c16a79</t>
+    <t>3460c0548689483b7415f521fbf687cb</t>
   </si>
   <si>
     <t>01-010046TM</t>
@@ -3836,7 +3836,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>1dfdd5679f7ee319e320d406aa4ca709</t>
+    <t>5e4ab72ee31126c82067e63326a6968e</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -3860,7 +3860,7 @@
     <t>05-050207A</t>
   </si>
   <si>
-    <t>d9f4f2892bdd8d80380caf4dcc428307</t>
+    <t>8cbba115c0d3741f462453bd485fd304</t>
   </si>
   <si>
     <t>02-020006TM</t>
@@ -3911,7 +3911,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>44e3088d57e75072827ee3ee130b7943</t>
+    <t>d74eb364d395241e4a88ce4dd643a1b4</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -3983,7 +3983,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>05089a667705b6ff52f21f0a6990ad9b</t>
+    <t>e43456585f774ed373438d7ef49f2aa3</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4004,7 +4004,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>41bf80ef7c81b0a5661624678ccde1ca</t>
+    <t>f43b4a6f7cc8bf13c3a92b4b7f8e726d</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4133,7 +4133,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>b0c2a18df112b9f277fecaa6a1e00eb7</t>
+    <t>ea579b3f30efb72eb919c6a56f538c3e</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4325,7 +4325,7 @@
     <t>05-050202TC</t>
   </si>
   <si>
-    <t>ec29680cb56f42a64a35dbc3449c2575</t>
+    <t>58fca060a06c31d35ca37b7b32ae2d13</t>
   </si>
   <si>
     <t>03-030062TP</t>
@@ -4343,7 +4343,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>9ac516dcbe0b313e4b36eb8426ea47b9</t>
+    <t>7522cf9fbb024ae1c150b2151111be09</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4370,7 +4370,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>1affb1ed2822a12b159e8df078bf0975</t>
+    <t>fa838f54022d6a8979ed747fda2cb32f</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -4469,13 +4469,13 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>6ca08574d86ae3aa9d7e5c47c265b84a</t>
+    <t>186b1a836d5aa29ca4cd018da9200e46</t>
   </si>
   <si>
     <t>05-050002A</t>
   </si>
   <si>
-    <t>42ae2ecbbe95475185886ba7eb9ed1f7</t>
+    <t>7509b2ca97b6b009aa96ff8bb2d842d5</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4505,7 +4505,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>4674a84d8a29ca83aa949ac49fbfc93a</t>
+    <t>1a091c654aec82de978d555c663bab50</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -4532,7 +4532,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>6f6df58ed26c3b04d4a1451cd1752a17</t>
+    <t>2a07bf6c6c1eb49dfac0a251abbaf02f</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4736,7 +4736,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>f39c13e6a0c461b855c0c6328d15b4d7</t>
+    <t>ee1b5d5b8ff266973aaea21d50fad9fa</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -4871,7 +4871,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>e64797a2cb3edeb4ee2d3a9ac5c7bd75</t>
+    <t>fa45adef370f900924977faca8daa50d</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb ago  7 03:55:14 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2657,7 +2657,7 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>4082473e455ea2efcc317070f655c008</t>
+    <t>dcedc3bb0496b5514f1f455c2762bfbb</t>
   </si>
   <si>
     <t>05-050311A</t>
@@ -3338,7 +3338,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>197c0b9cfac61b90cfd77d9e3b15133c</t>
+    <t>8e139870df3053cfbb1e578385924988</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -4286,7 +4286,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>7f3c93123e6807038cd5a33a137219fe</t>
+    <t>e54e7c48877447368243eafb48fab8ff</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom ago  8 05:12:18 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -662,7 +662,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>1a3f1505868feb8a19f6cbcdfc804738</t>
+    <t>3f3cb0272d91d93b8d9910216dd98b56</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -1748,7 +1748,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>b0ac4930ec15dbac39af731b9db4768c</t>
+    <t>0e6c865ef608c20883124ef0380127e2</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>0841f66eec1f7caf51680bed6f5054c6</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode lun ago  9 05:43:20 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1748,7 +1748,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>0e6c865ef608c20883124ef0380127e2</t>
+    <t>b0ac4930ec15dbac39af731b9db4768c</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>0841f66eec1f7caf51680bed6f5054c6</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar ago 10 04:48:44 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -827,7 +827,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>84f9177b78615335c74de6904e2acd32</t>
+    <t>14dc6a7115ed8643d0342c17efbddf27</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -857,7 +857,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>ab0ea17fae2aec0703ccc1e868a613be</t>
+    <t>546191a602cd86ccda80feba3dc550d8</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
+    <t>e485342c765c36244fab6a0d410188bb</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>fe069915e6896d5ed070ddbadaac6446</t>
+    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
+    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1307,7 +1307,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>e0c82a61a67245f79968a744f7b09936</t>
+    <t>accee517f3d37c3718bdd35d130fdb09</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1466,7 +1466,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>659242aec416d17e85f02ecbb12330d9</t>
+    <t>d03a41d30eaa290a2df7d86128170fc8</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>0841f66eec1f7caf51680bed6f5054c6</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
+    <t>397f95ff13cb7f56235d92785ac466a5</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -2831,7 +2831,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>568f02ee5c11b452a06580198ae3fcfd</t>
+    <t>bce246d0f326510acf85215689732b93</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2933,7 +2933,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>df33604063d2187b012a3a687c78f6f7</t>
+    <t>c178e29df4f7707ac5dd97e5dfb43e98</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3983,7 +3983,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>e43456585f774ed373438d7ef49f2aa3</t>
+    <t>cb9274c9525c17ea68bb2adb72b918b2</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4250,7 +4250,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ad6e173e9e187d4df9db4e9e93687c24</t>
+    <t>ff983b6dba0a7b6b341e82f792b83e5f</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4265,7 +4265,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>3a4d48d91fc07d0a8fd7f12c5d10e8e5</t>
+    <t>f13308e69a2d1e8b94c4a1516c7a0cc4</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>
@@ -4871,7 +4871,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>fa45adef370f900924977faca8daa50d</t>
+    <t>166e7d248577a16ab1474b1ad6135ff9</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié ago 11 05:19:59 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -827,7 +827,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>14dc6a7115ed8643d0342c17efbddf27</t>
+    <t>84f9177b78615335c74de6904e2acd32</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -857,7 +857,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>546191a602cd86ccda80feba3dc550d8</t>
+    <t>ab0ea17fae2aec0703ccc1e868a613be</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>e485342c765c36244fab6a0d410188bb</t>
+    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
+    <t>fe069915e6896d5ed070ddbadaac6446</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
+    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1307,7 +1307,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>accee517f3d37c3718bdd35d130fdb09</t>
+    <t>e0c82a61a67245f79968a744f7b09936</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1466,7 +1466,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>d03a41d30eaa290a2df7d86128170fc8</t>
+    <t>659242aec416d17e85f02ecbb12330d9</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -2165,7 +2165,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>2e53c6037ada0a5f4509b5c48de7db82</t>
+    <t>222036ac958a83c91ac7ee20641a3bcd</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>0841f66eec1f7caf51680bed6f5054c6</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2348,7 +2348,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>cd6d4751cda79df64f498f4b24da5db7</t>
+    <t>56b006ec8a69efa8ace08d6c37cc8aab</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>397f95ff13cb7f56235d92785ac466a5</t>
+    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -2831,7 +2831,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>bce246d0f326510acf85215689732b93</t>
+    <t>568f02ee5c11b452a06580198ae3fcfd</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2933,7 +2933,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>c178e29df4f7707ac5dd97e5dfb43e98</t>
+    <t>df33604063d2187b012a3a687c78f6f7</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3008,7 +3008,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>134162bc7e138f3db345fa90ad9f1a3d</t>
+    <t>ea84c9018e64e1a60956b7b5ea05c98d</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3983,7 +3983,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>cb9274c9525c17ea68bb2adb72b918b2</t>
+    <t>e43456585f774ed373438d7ef49f2aa3</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4004,7 +4004,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>f43b4a6f7cc8bf13c3a92b4b7f8e726d</t>
+    <t>b0d983bda09391468dcc9b39c3bfbd4b</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4133,7 +4133,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>ea579b3f30efb72eb919c6a56f538c3e</t>
+    <t>98a8d5220c099a28a1f4102ef82c39cb</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4250,7 +4250,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ff983b6dba0a7b6b341e82f792b83e5f</t>
+    <t>ad6e173e9e187d4df9db4e9e93687c24</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4265,7 +4265,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>f13308e69a2d1e8b94c4a1516c7a0cc4</t>
+    <t>3a4d48d91fc07d0a8fd7f12c5d10e8e5</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4475,7 +4475,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>7509b2ca97b6b009aa96ff8bb2d842d5</t>
+    <t>29e2d68caa84824815942fcbb7de8fcb</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4532,7 +4532,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>2a07bf6c6c1eb49dfac0a251abbaf02f</t>
+    <t>26d18c3464dd106a56836bfa4eab269a</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4736,7 +4736,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>ee1b5d5b8ff266973aaea21d50fad9fa</t>
+    <t>4e0e765b29a9b7c15fa8c3babf7ab96b</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -4871,7 +4871,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>166e7d248577a16ab1474b1ad6135ff9</t>
+    <t>fa45adef370f900924977faca8daa50d</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue ago 12 05:38:39 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -827,7 +827,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>84f9177b78615335c74de6904e2acd32</t>
+    <t>14dc6a7115ed8643d0342c17efbddf27</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -857,7 +857,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>ab0ea17fae2aec0703ccc1e868a613be</t>
+    <t>546191a602cd86ccda80feba3dc550d8</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
+    <t>e485342c765c36244fab6a0d410188bb</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>fe069915e6896d5ed070ddbadaac6446</t>
+    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
+    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1307,7 +1307,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>e0c82a61a67245f79968a744f7b09936</t>
+    <t>accee517f3d37c3718bdd35d130fdb09</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1466,7 +1466,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>659242aec416d17e85f02ecbb12330d9</t>
+    <t>d03a41d30eaa290a2df7d86128170fc8</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1769,7 +1769,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>2270685ec7d3a5468017dba19d33c2bd</t>
+    <t>258d3ef813ddad27f7ba8abc6388b27b</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2165,7 +2165,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>222036ac958a83c91ac7ee20641a3bcd</t>
+    <t>2e53c6037ada0a5f4509b5c48de7db82</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>0841f66eec1f7caf51680bed6f5054c6</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2348,7 +2348,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>56b006ec8a69efa8ace08d6c37cc8aab</t>
+    <t>cd6d4751cda79df64f498f4b24da5db7</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
+    <t>397f95ff13cb7f56235d92785ac466a5</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -2831,7 +2831,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>568f02ee5c11b452a06580198ae3fcfd</t>
+    <t>bce246d0f326510acf85215689732b93</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2933,7 +2933,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>df33604063d2187b012a3a687c78f6f7</t>
+    <t>c178e29df4f7707ac5dd97e5dfb43e98</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3008,7 +3008,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>ea84c9018e64e1a60956b7b5ea05c98d</t>
+    <t>134162bc7e138f3db345fa90ad9f1a3d</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3116,7 +3116,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>887e5ce461f76ef5d09805b2e0f0c8c3</t>
+    <t>d07887befe6d56766f32d3ba049af99e</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3983,7 +3983,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>e43456585f774ed373438d7ef49f2aa3</t>
+    <t>cb9274c9525c17ea68bb2adb72b918b2</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4004,7 +4004,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>b0d983bda09391468dcc9b39c3bfbd4b</t>
+    <t>f43b4a6f7cc8bf13c3a92b4b7f8e726d</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4133,7 +4133,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>98a8d5220c099a28a1f4102ef82c39cb</t>
+    <t>ea579b3f30efb72eb919c6a56f538c3e</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4250,7 +4250,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ad6e173e9e187d4df9db4e9e93687c24</t>
+    <t>ff983b6dba0a7b6b341e82f792b83e5f</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4265,7 +4265,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>3a4d48d91fc07d0a8fd7f12c5d10e8e5</t>
+    <t>f13308e69a2d1e8b94c4a1516c7a0cc4</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4475,7 +4475,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>29e2d68caa84824815942fcbb7de8fcb</t>
+    <t>7509b2ca97b6b009aa96ff8bb2d842d5</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4532,7 +4532,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>26d18c3464dd106a56836bfa4eab269a</t>
+    <t>2a07bf6c6c1eb49dfac0a251abbaf02f</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4736,7 +4736,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>4e0e765b29a9b7c15fa8c3babf7ab96b</t>
+    <t>ee1b5d5b8ff266973aaea21d50fad9fa</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -4871,7 +4871,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>fa45adef370f900924977faca8daa50d</t>
+    <t>166e7d248577a16ab1474b1ad6135ff9</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie ago 13 04:46:28 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -827,7 +827,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>14dc6a7115ed8643d0342c17efbddf27</t>
+    <t>84f9177b78615335c74de6904e2acd32</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -857,7 +857,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>546191a602cd86ccda80feba3dc550d8</t>
+    <t>ab0ea17fae2aec0703ccc1e868a613be</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1307,7 +1307,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>accee517f3d37c3718bdd35d130fdb09</t>
+    <t>e0c82a61a67245f79968a744f7b09936</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1466,7 +1466,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>d03a41d30eaa290a2df7d86128170fc8</t>
+    <t>659242aec416d17e85f02ecbb12330d9</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1769,7 +1769,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>258d3ef813ddad27f7ba8abc6388b27b</t>
+    <t>2270685ec7d3a5468017dba19d33c2bd</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2831,7 +2831,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>bce246d0f326510acf85215689732b93</t>
+    <t>568f02ee5c11b452a06580198ae3fcfd</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2933,7 +2933,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>c178e29df4f7707ac5dd97e5dfb43e98</t>
+    <t>df33604063d2187b012a3a687c78f6f7</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3116,7 +3116,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>d07887befe6d56766f32d3ba049af99e</t>
+    <t>887e5ce461f76ef5d09805b2e0f0c8c3</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3983,7 +3983,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>cb9274c9525c17ea68bb2adb72b918b2</t>
+    <t>e43456585f774ed373438d7ef49f2aa3</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4250,7 +4250,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ff983b6dba0a7b6b341e82f792b83e5f</t>
+    <t>ad6e173e9e187d4df9db4e9e93687c24</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4265,7 +4265,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>f13308e69a2d1e8b94c4a1516c7a0cc4</t>
+    <t>3a4d48d91fc07d0a8fd7f12c5d10e8e5</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>
@@ -4871,7 +4871,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>166e7d248577a16ab1474b1ad6135ff9</t>
+    <t>fa45adef370f900924977faca8daa50d</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb ago 14 05:39:22 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>e485342c765c36244fab6a0d410188bb</t>
+    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
+    <t>fe069915e6896d5ed070ddbadaac6446</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
+    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1307,7 +1307,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>e0c82a61a67245f79968a744f7b09936</t>
+    <t>accee517f3d37c3718bdd35d130fdb09</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1466,7 +1466,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>659242aec416d17e85f02ecbb12330d9</t>
+    <t>d03a41d30eaa290a2df7d86128170fc8</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -2165,7 +2165,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>2e53c6037ada0a5f4509b5c48de7db82</t>
+    <t>222036ac958a83c91ac7ee20641a3bcd</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>0841f66eec1f7caf51680bed6f5054c6</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2348,7 +2348,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>cd6d4751cda79df64f498f4b24da5db7</t>
+    <t>56b006ec8a69efa8ace08d6c37cc8aab</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>397f95ff13cb7f56235d92785ac466a5</t>
+    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -3008,7 +3008,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>134162bc7e138f3db345fa90ad9f1a3d</t>
+    <t>ea84c9018e64e1a60956b7b5ea05c98d</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3983,7 +3983,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>e43456585f774ed373438d7ef49f2aa3</t>
+    <t>cb9274c9525c17ea68bb2adb72b918b2</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4004,7 +4004,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>f43b4a6f7cc8bf13c3a92b4b7f8e726d</t>
+    <t>b0d983bda09391468dcc9b39c3bfbd4b</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4133,7 +4133,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>ea579b3f30efb72eb919c6a56f538c3e</t>
+    <t>98a8d5220c099a28a1f4102ef82c39cb</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4475,7 +4475,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>7509b2ca97b6b009aa96ff8bb2d842d5</t>
+    <t>29e2d68caa84824815942fcbb7de8fcb</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4532,7 +4532,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>2a07bf6c6c1eb49dfac0a251abbaf02f</t>
+    <t>26d18c3464dd106a56836bfa4eab269a</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>
@@ -4736,7 +4736,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>ee1b5d5b8ff266973aaea21d50fad9fa</t>
+    <t>4e0e765b29a9b7c15fa8c3babf7ab96b</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -4871,7 +4871,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>fa45adef370f900924977faca8daa50d</t>
+    <t>166e7d248577a16ab1474b1ad6135ff9</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom ago 15 04:36:09 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
+    <t>e485342c765c36244fab6a0d410188bb</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>fe069915e6896d5ed070ddbadaac6446</t>
+    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
+    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1307,7 +1307,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>accee517f3d37c3718bdd35d130fdb09</t>
+    <t>e0c82a61a67245f79968a744f7b09936</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1466,7 +1466,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>d03a41d30eaa290a2df7d86128170fc8</t>
+    <t>659242aec416d17e85f02ecbb12330d9</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1748,7 +1748,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>b0ac4930ec15dbac39af731b9db4768c</t>
+    <t>0e6c865ef608c20883124ef0380127e2</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>0841f66eec1f7caf51680bed6f5054c6</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
+    <t>397f95ff13cb7f56235d92785ac466a5</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -3983,7 +3983,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>cb9274c9525c17ea68bb2adb72b918b2</t>
+    <t>e43456585f774ed373438d7ef49f2aa3</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>
@@ -4871,7 +4871,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>166e7d248577a16ab1474b1ad6135ff9</t>
+    <t>fa45adef370f900924977faca8daa50d</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode lun ago 16 05:38:38 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>e485342c765c36244fab6a0d410188bb</t>
+    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
+    <t>fe069915e6896d5ed070ddbadaac6446</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
+    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1748,7 +1748,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>0e6c865ef608c20883124ef0380127e2</t>
+    <t>b0ac4930ec15dbac39af731b9db4768c</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -2165,7 +2165,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>222036ac958a83c91ac7ee20641a3bcd</t>
+    <t>2e53c6037ada0a5f4509b5c48de7db82</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>0841f66eec1f7caf51680bed6f5054c6</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2348,7 +2348,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>56b006ec8a69efa8ace08d6c37cc8aab</t>
+    <t>cd6d4751cda79df64f498f4b24da5db7</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>397f95ff13cb7f56235d92785ac466a5</t>
+    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -3008,7 +3008,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>ea84c9018e64e1a60956b7b5ea05c98d</t>
+    <t>134162bc7e138f3db345fa90ad9f1a3d</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -4004,7 +4004,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>b0d983bda09391468dcc9b39c3bfbd4b</t>
+    <t>f43b4a6f7cc8bf13c3a92b4b7f8e726d</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4133,7 +4133,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>98a8d5220c099a28a1f4102ef82c39cb</t>
+    <t>ea579b3f30efb72eb919c6a56f538c3e</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4475,7 +4475,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>29e2d68caa84824815942fcbb7de8fcb</t>
+    <t>7509b2ca97b6b009aa96ff8bb2d842d5</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4532,7 +4532,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>26d18c3464dd106a56836bfa4eab269a</t>
+    <t>2a07bf6c6c1eb49dfac0a251abbaf02f</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4736,7 +4736,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>4e0e765b29a9b7c15fa8c3babf7ab96b</t>
+    <t>ee1b5d5b8ff266973aaea21d50fad9fa</t>
   </si>
   <si>
     <t>01-010006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar ago 17 05:35:58 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -827,7 +827,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>84f9177b78615335c74de6904e2acd32</t>
+    <t>14dc6a7115ed8643d0342c17efbddf27</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -857,7 +857,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>ab0ea17fae2aec0703ccc1e868a613be</t>
+    <t>546191a602cd86ccda80feba3dc550d8</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
+    <t>e485342c765c36244fab6a0d410188bb</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>fe069915e6896d5ed070ddbadaac6446</t>
+    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
+    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1457,7 +1457,7 @@
     <t>05-050003TM</t>
   </si>
   <si>
-    <t>a996d4ebbf0fd8d2ceecd7b76c1e4798</t>
+    <t>26a174eb39b463d9fb80104d5dee9319</t>
   </si>
   <si>
     <t>01-010025TM</t>
@@ -1748,7 +1748,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>b0ac4930ec15dbac39af731b9db4768c</t>
+    <t>0e6c865ef608c20883124ef0380127e2</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -1769,7 +1769,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>2270685ec7d3a5468017dba19d33c2bd</t>
+    <t>258d3ef813ddad27f7ba8abc6388b27b</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2165,7 +2165,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>2e53c6037ada0a5f4509b5c48de7db82</t>
+    <t>222036ac958a83c91ac7ee20641a3bcd</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>0841f66eec1f7caf51680bed6f5054c6</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2348,7 +2348,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>cd6d4751cda79df64f498f4b24da5db7</t>
+    <t>56b006ec8a69efa8ace08d6c37cc8aab</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
+    <t>397f95ff13cb7f56235d92785ac466a5</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -2831,7 +2831,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>568f02ee5c11b452a06580198ae3fcfd</t>
+    <t>bce246d0f326510acf85215689732b93</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2933,7 +2933,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>df33604063d2187b012a3a687c78f6f7</t>
+    <t>c178e29df4f7707ac5dd97e5dfb43e98</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3008,7 +3008,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>134162bc7e138f3db345fa90ad9f1a3d</t>
+    <t>ea84c9018e64e1a60956b7b5ea05c98d</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3116,7 +3116,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>887e5ce461f76ef5d09805b2e0f0c8c3</t>
+    <t>d07887befe6d56766f32d3ba049af99e</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -4004,7 +4004,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>f43b4a6f7cc8bf13c3a92b4b7f8e726d</t>
+    <t>b0d983bda09391468dcc9b39c3bfbd4b</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4133,7 +4133,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>ea579b3f30efb72eb919c6a56f538c3e</t>
+    <t>98a8d5220c099a28a1f4102ef82c39cb</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4250,7 +4250,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ad6e173e9e187d4df9db4e9e93687c24</t>
+    <t>ff983b6dba0a7b6b341e82f792b83e5f</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4265,7 +4265,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>3a4d48d91fc07d0a8fd7f12c5d10e8e5</t>
+    <t>f13308e69a2d1e8b94c4a1516c7a0cc4</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4475,7 +4475,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>7509b2ca97b6b009aa96ff8bb2d842d5</t>
+    <t>29e2d68caa84824815942fcbb7de8fcb</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4532,7 +4532,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>2a07bf6c6c1eb49dfac0a251abbaf02f</t>
+    <t>26d18c3464dd106a56836bfa4eab269a</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4736,7 +4736,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>ee1b5d5b8ff266973aaea21d50fad9fa</t>
+    <t>4e0e765b29a9b7c15fa8c3babf7ab96b</t>
   </si>
   <si>
     <t>01-010006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié ago 18 06:22:13 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -827,7 +827,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>14dc6a7115ed8643d0342c17efbddf27</t>
+    <t>84f9177b78615335c74de6904e2acd32</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -857,7 +857,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>546191a602cd86ccda80feba3dc550d8</t>
+    <t>ab0ea17fae2aec0703ccc1e868a613be</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>e485342c765c36244fab6a0d410188bb</t>
+    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
+    <t>fe069915e6896d5ed070ddbadaac6446</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
+    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1748,7 +1748,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>0e6c865ef608c20883124ef0380127e2</t>
+    <t>b0ac4930ec15dbac39af731b9db4768c</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -1769,7 +1769,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>258d3ef813ddad27f7ba8abc6388b27b</t>
+    <t>2270685ec7d3a5468017dba19d33c2bd</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>0841f66eec1f7caf51680bed6f5054c6</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>397f95ff13cb7f56235d92785ac466a5</t>
+    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -2831,7 +2831,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>bce246d0f326510acf85215689732b93</t>
+    <t>568f02ee5c11b452a06580198ae3fcfd</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2933,7 +2933,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>c178e29df4f7707ac5dd97e5dfb43e98</t>
+    <t>df33604063d2187b012a3a687c78f6f7</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3116,7 +3116,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>d07887befe6d56766f32d3ba049af99e</t>
+    <t>887e5ce461f76ef5d09805b2e0f0c8c3</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -4250,7 +4250,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ff983b6dba0a7b6b341e82f792b83e5f</t>
+    <t>ad6e173e9e187d4df9db4e9e93687c24</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4265,7 +4265,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>f13308e69a2d1e8b94c4a1516c7a0cc4</t>
+    <t>3a4d48d91fc07d0a8fd7f12c5d10e8e5</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue ago 19 05:44:32 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1178,7 +1178,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>6afc8b7b89d7b6de5b1f057617bf949e</t>
+    <t>e485342c765c36244fab6a0d410188bb</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1196,7 +1196,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>fe069915e6896d5ed070ddbadaac6446</t>
+    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>3c21b8271b2dc768c843ffbf8ff5324f</t>
+    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1748,7 +1748,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>b0ac4930ec15dbac39af731b9db4768c</t>
+    <t>0e6c865ef608c20883124ef0380127e2</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>0841f66eec1f7caf51680bed6f5054c6</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2744,7 +2744,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>99021a89849f7c14eb47cfe4d4b3107d</t>
+    <t>397f95ff13cb7f56235d92785ac466a5</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie ago 20 01:11:16 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -827,7 +827,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>84f9177b78615335c74de6904e2acd32</t>
+    <t>14dc6a7115ed8643d0342c17efbddf27</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -857,7 +857,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>ab0ea17fae2aec0703ccc1e868a613be</t>
+    <t>546191a602cd86ccda80feba3dc550d8</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -2831,7 +2831,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>568f02ee5c11b452a06580198ae3fcfd</t>
+    <t>bce246d0f326510acf85215689732b93</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2933,7 +2933,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>df33604063d2187b012a3a687c78f6f7</t>
+    <t>c178e29df4f7707ac5dd97e5dfb43e98</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4250,7 +4250,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ad6e173e9e187d4df9db4e9e93687c24</t>
+    <t>ff983b6dba0a7b6b341e82f792b83e5f</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4265,7 +4265,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>3a4d48d91fc07d0a8fd7f12c5d10e8e5</t>
+    <t>f13308e69a2d1e8b94c4a1516c7a0cc4</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4556,7 +4556,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom ago 22 04:48:21 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1769,7 +1769,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>2270685ec7d3a5468017dba19d33c2bd</t>
+    <t>258d3ef813ddad27f7ba8abc6388b27b</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2165,7 +2165,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>222036ac958a83c91ac7ee20641a3bcd</t>
+    <t>2e53c6037ada0a5f4509b5c48de7db82</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2210,7 +2210,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2348,7 +2348,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>56b006ec8a69efa8ace08d6c37cc8aab</t>
+    <t>cd6d4751cda79df64f498f4b24da5db7</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -3008,7 +3008,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>ea84c9018e64e1a60956b7b5ea05c98d</t>
+    <t>134162bc7e138f3db345fa90ad9f1a3d</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3116,7 +3116,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>887e5ce461f76ef5d09805b2e0f0c8c3</t>
+    <t>d07887befe6d56766f32d3ba049af99e</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -4004,7 +4004,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>b0d983bda09391468dcc9b39c3bfbd4b</t>
+    <t>f43b4a6f7cc8bf13c3a92b4b7f8e726d</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4133,7 +4133,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>98a8d5220c099a28a1f4102ef82c39cb</t>
+    <t>ea579b3f30efb72eb919c6a56f538c3e</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4475,7 +4475,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>29e2d68caa84824815942fcbb7de8fcb</t>
+    <t>7509b2ca97b6b009aa96ff8bb2d842d5</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4532,7 +4532,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>26d18c3464dd106a56836bfa4eab269a</t>
+    <t>2a07bf6c6c1eb49dfac0a251abbaf02f</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4736,7 +4736,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>4e0e765b29a9b7c15fa8c3babf7ab96b</t>
+    <t>ee1b5d5b8ff266973aaea21d50fad9fa</t>
   </si>
   <si>
     <t>01-010006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie sep  3 01:18:35 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>408047ce987223fba9f85e8d7dda986f</t>
+    <t>8506888276693576c92158880b2778a0</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -533,7 +533,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>57287b73631d1dd0760a97d7f3caac2e</t>
+    <t>89d8b8363a38e01d7a16c2da40df1f3c</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -590,7 +590,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>6de338d5b96f4c93b6ec4bb89b59161e</t>
+    <t>8cabc50ed25dbd573a6921609a339df7</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -656,7 +656,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>50799c60fdb747d4279d38bd5b03aeb8</t>
+    <t>099acd20269d8221cd4fdb8b77193168</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -836,7 +836,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>14dc6a7115ed8643d0342c17efbddf27</t>
+    <t>50865ddaa756834b155e8a12a9fb6878</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -866,7 +866,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>546191a602cd86ccda80feba3dc550d8</t>
+    <t>76f66f979d0ed127425772edced54f59</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1502,7 +1502,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>3e99b032c7ffd9082e7b4646ae3134b8</t>
+    <t>c6fa7b4bcd9efd33c0b46e83f0d3938d</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2450,7 +2450,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>1e9f650233b1837146e626f3c41edea3</t>
+    <t>a7094538211176a4493642127d720327</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2861,7 +2861,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>bce246d0f326510acf85215689732b93</t>
+    <t>ac6440f27d6bdf0632f1ffe1730f4b3b</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2966,7 +2966,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>c178e29df4f7707ac5dd97e5dfb43e98</t>
+    <t>2b690f85f54ad877602f070b51761aa2</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3473,7 +3473,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>3c97d05e668859254bf07149cb1a8d06</t>
+    <t>9fbc1de2835461ce96e0d065fbdc2ccb</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3500,7 +3500,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>ed84dfdffacedeec79d20a683308511e</t>
+    <t>8b8f45498a8f0607cad6be289853893b</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4073,7 +4073,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>90c03a7dd9cf250bec609eba72199372</t>
+    <t>042d3fe35e65dcec9484c707fdbd953d</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4289,7 +4289,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ff983b6dba0a7b6b341e82f792b83e5f</t>
+    <t>7ae182c84642edc5382f561eaa06598d</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4304,7 +4304,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>f13308e69a2d1e8b94c4a1516c7a0cc4</t>
+    <t>976c8f5e0985ab7716283e7852a946df</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb sep  4 02:00:45 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1202,7 +1202,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>e485342c765c36244fab6a0d410188bb</t>
+    <t>1701cd60c0fd5c809f2a1e98dd85181c</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>f35cd2720c6d6e18ab5e89ca234f5b7e</t>
+    <t>f359acb0bce62ddc8b0b443d3adad72a</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1244,7 +1244,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>588e4b8b4b02f4b3b76a481722da12f3</t>
+    <t>15e2dc221af3fce6b6db0833049ce66f</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1772,7 +1772,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>0e6c865ef608c20883124ef0380127e2</t>
+    <t>16900adb23af8ab043627443199b4fc5</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -1793,7 +1793,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>258d3ef813ddad27f7ba8abc6388b27b</t>
+    <t>b66efb5c6546772060de0ac4cbfd1afa</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2636,7 +2636,7 @@
     <t>05-050208TC</t>
   </si>
   <si>
-    <t>4b1b942b40330cd0cc3ceb2b49128d69</t>
+    <t>988b94643e2660daa15f9c369f70b789</t>
   </si>
   <si>
     <t>03-030039A</t>
@@ -2768,7 +2768,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>397f95ff13cb7f56235d92785ac466a5</t>
+    <t>4f87d9f7a205a1dbbe49e3a094de731b</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -3149,7 +3149,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>d07887befe6d56766f32d3ba049af99e</t>
+    <t>5714d0a0107259283cbc6a8b9eeda9e7</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -4604,7 +4604,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom sep  5 05:22:00 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -65,7 +65,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>bf88958680fd0ad4437263ca6fdb297f</t>
+    <t>af31c33312e9cbdceb91ba1cae619041</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -101,7 +101,7 @@
     <t>05-050207TP</t>
   </si>
   <si>
-    <t>3f566850f7e1fb5e14efe24cd9262168</t>
+    <t>dd7be23b0a967f072967c7d89602e78f</t>
   </si>
   <si>
     <t>915-150012A</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>3be5860e231c20fa27df04eb4ca8cf98</t>
+    <t>825b50c1077bcc44e9142241e49f1cff</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -152,7 +152,7 @@
     <t>05-050316TC</t>
   </si>
   <si>
-    <t>6bf83fd50321eed05183fd05dcc29b85</t>
+    <t>fa8cb3c3b8b756132399d3332953b0bd</t>
   </si>
   <si>
     <t>03-030059TP</t>
@@ -179,7 +179,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>a6ed462f4b3da22413d958a0e0aa216f</t>
+    <t>e7c2c0aef67605ee2a88d1c598b2683f</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -206,7 +206,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>bdfa6c8d82452f12b312fe16aed392ed</t>
+    <t>9969a07157b2257f0fd8700132780393</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -689,7 +689,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>dc47d7dcb14346d6d0beb3cbf823be31</t>
+    <t>01a7a415f0359063e9a59e03cafd8e98</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -725,7 +725,7 @@
     <t>05-050312TP</t>
   </si>
   <si>
-    <t>9630a8476f259b238c150ab3f99edf8e</t>
+    <t>9480db809a06505fe676dccf85bf1d75</t>
   </si>
   <si>
     <t>05-0709-070954TC</t>
@@ -740,7 +740,7 @@
     <t>05-050312TC</t>
   </si>
   <si>
-    <t>ff88d21c9f0b469b698693cda95351e9</t>
+    <t>0e5cabff8af1d5481b7c3e17d8c96c98</t>
   </si>
   <si>
     <t>03-030055TP</t>
@@ -860,7 +860,7 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>d54dc554914eb3eb482791129a9f1b55</t>
+    <t>12d24d38c646234d7d05cda9ca8b8076</t>
   </si>
   <si>
     <t>05-050007TP</t>
@@ -875,7 +875,7 @@
     <t>05-050308A</t>
   </si>
   <si>
-    <t>cc991a52b705db26dc7a0813407aaf1f</t>
+    <t>5fa90ebdbc289531432d123ecba8a9cd</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -917,7 +917,7 @@
     <t>05-050203TC</t>
   </si>
   <si>
-    <t>460ad78a8776f06c7aa8601798efa385</t>
+    <t>26b3c81df830df1b8eab5101e091d8b5</t>
   </si>
   <si>
     <t>01-110304-11030404A</t>
@@ -947,7 +947,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>1003d58c916678b64c8fb9bc851634d1</t>
+    <t>56c15d873c55652037efa85c0e61256c</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -974,7 +974,7 @@
     <t>05-050303TC</t>
   </si>
   <si>
-    <t>dacbadc0a71781aab84d5510eb2d5a3a</t>
+    <t>2f3b2814347a9ffef04fc451a611e891</t>
   </si>
   <si>
     <t>01-010010TP</t>
@@ -992,7 +992,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>20690ceb1cad475a5b571ca87e928d06</t>
+    <t>800d717efa91ff5a59b84a895bd97196</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1037,7 +1037,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>88af5bf5ace7bc9f41425d4f63be1fa2</t>
+    <t>5c5ae8f115b3f8982c041013f59312e9</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1079,7 +1079,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>701ed1d847fae8c7ccd569fc1d79d15f</t>
+    <t>e5cb158eb7c88f78f46fce5df8aa9b39</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1088,7 +1088,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>77f66364cc88cbdc1a18e276684ad447</t>
+    <t>9bcfbfdd1d28207dd0d0df4d04d0a876</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1157,7 +1157,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>149517503b59ddfc3918c862b96b3067</t>
+    <t>f1ac35b69c56c41e4086c6b0275d1479</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1232,13 +1232,13 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>09dc94ef4f361581164ab3997e67c878</t>
+    <t>2537c24366e2e12fd3cb2e61066ec412</t>
   </si>
   <si>
     <t>05-050304A</t>
   </si>
   <si>
-    <t>09420b52977612a4d86a279f940ff25d</t>
+    <t>f5123e7de2b78d32a70a6953346246ce</t>
   </si>
   <si>
     <t>05-050009TP</t>
@@ -1262,7 +1262,7 @@
     <t>05-050205TC</t>
   </si>
   <si>
-    <t>add83c8ffd62b5c5fff7be16dae8afaf</t>
+    <t>b70d5a3413a2be3ab3b58ac3e96bd586</t>
   </si>
   <si>
     <t>04-040014TM</t>
@@ -1331,7 +1331,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>e0c82a61a67245f79968a744f7b09936</t>
+    <t>bd0c190fdc6ad6858e7db26ed0e1a31c</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1490,7 +1490,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>659242aec416d17e85f02ecbb12330d9</t>
+    <t>36c11d492334114e57cd2f6887dc8b58</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1520,7 +1520,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>66a9960dc0d88e04f3a96d58130f043c</t>
+    <t>9f1c93a1b6c164b4b600c0f09e89154f</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1589,7 +1589,7 @@
     <t>05-050310TC</t>
   </si>
   <si>
-    <t>60115817a4a3be48293379683941555f</t>
+    <t>25e887e5583f35372283f28e92d27333</t>
   </si>
   <si>
     <t>04-040004A</t>
@@ -1637,7 +1637,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>4fcc2830cebe5ef789159e5ea8813780</t>
+    <t>a36c23993dcd2e15a775968f6ac17b5b</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1817,7 +1817,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>0f1b7e48d003129c49d1a2059acc209b</t>
+    <t>29364419b881cb3062a9df4ab7349651</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2189,7 +2189,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>2e53c6037ada0a5f4509b5c48de7db82</t>
+    <t>e1f70a292fb3beb643a4f3e43fe7ee57</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2372,7 +2372,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>cd6d4751cda79df64f498f4b24da5db7</t>
+    <t>868e881d8cfa61e7418a181b49c7601e</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2444,7 +2444,7 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>ac412a65c65171b2378eada58b4f3bd5</t>
+    <t>7e11d9dbca5e14a6169d3edcd00a5c32</t>
   </si>
   <si>
     <t>05-050313A</t>
@@ -2543,7 +2543,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>90ab25c4405ead4ee0afe1b9d14f2107</t>
+    <t>57d4113904f1dc0c137b2728c40d233c</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2555,7 +2555,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>2d6ceb7203356c3b73893edf9cda7000</t>
+    <t>73feff9b9fc889606338dd4511865eac</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2687,7 +2687,7 @@
     <t>05-050311A</t>
   </si>
   <si>
-    <t>00659defee040ed572c29c341ea04db5</t>
+    <t>f79c33d32f08b5ff0aa0bd9fcef6dc2c</t>
   </si>
   <si>
     <t>05-050208TP</t>
@@ -2717,7 +2717,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>e71bf6219416afaac82fb6bc9f5e2fa3</t>
+    <t>e6f7e6ed8a816ffab3bd6a1833ee032c</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -2756,13 +2756,13 @@
     <t>05-050317TC</t>
   </si>
   <si>
-    <t>7067f67b2942213b4d4713364e70ae2e</t>
+    <t>391af302ebda2244cf8770442ea1af07</t>
   </si>
   <si>
     <t>05-050312A</t>
   </si>
   <si>
-    <t>a9630c418c3f59d6a1b0b360a841ebf0</t>
+    <t>3091490aa5b60503358cb85f6a8240cb</t>
   </si>
   <si>
     <t>05-050009A</t>
@@ -2774,7 +2774,7 @@
     <t>05-050203A</t>
   </si>
   <si>
-    <t>60ddfdefed4769e4fc5a58fc7044c3e5</t>
+    <t>3b6268853f1fa8bd68839f0ef7b0f77b</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -2813,7 +2813,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>229410bf60ee30df3fa138b86e565bc4</t>
+    <t>b490a8599bb44f03e16e699f50a3053b</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -2930,7 +2930,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>7f4dc12e25c618f37e507de07c1df792</t>
+    <t>eb6dfa8ffd370531febde8b59adcfd16</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -2948,7 +2948,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>41669038dfc6b535dfbec046e1d33aa1</t>
+    <t>d4bebbf518230ca2aa990ad2dc7e13ac</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3023,7 +3023,7 @@
     <t>05-050308TC</t>
   </si>
   <si>
-    <t>c6b34662dbb3d73f48d62ae6dbde660d</t>
+    <t>a967e55f38ad4dd7eb150b3d0c03f0e5</t>
   </si>
   <si>
     <t>02-020002TC</t>
@@ -3041,7 +3041,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>134162bc7e138f3db345fa90ad9f1a3d</t>
+    <t>0b9c566e0f5b6d1080d7457b397c03ca</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3077,7 +3077,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>e6f48497af448ef49af760d78c76a34e</t>
+    <t>66c801a01056005954e9d18be923ab21</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3308,7 +3308,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>f27901d9c6928abaa5448bc98fd3c169</t>
+    <t>69506d8e29770012b06f21a3ef06de36</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3362,7 +3362,7 @@
     <t>05-050204TC</t>
   </si>
   <si>
-    <t>29a2a7a244786b74b0f5a6bbb50b99de</t>
+    <t>c34def8415f15a56ed6c596d8adda356</t>
   </si>
   <si>
     <t>04-040015TM</t>
@@ -3371,7 +3371,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>8e139870df3053cfbb1e578385924988</t>
+    <t>f868f002b4016f6d6646129be2c2a6c1</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3545,13 +3545,13 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>4a0a1f70e7364e195cef4517668fda56</t>
+    <t>01659c7eafacf6dee84b8f9830f0152d</t>
   </si>
   <si>
     <t>05-050317A</t>
   </si>
   <si>
-    <t>8698bccf05cce2f5667bf3d4c8455e29</t>
+    <t>005c764de734828fc6bdbbb991f36770</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -3617,7 +3617,7 @@
     <t>05-050206TP</t>
   </si>
   <si>
-    <t>a6c0778e5c6025b5eca2a3b5364d1036</t>
+    <t>1411adebe1166b57dc7540f57ea16da0</t>
   </si>
   <si>
     <t>01-010068TM</t>
@@ -3641,7 +3641,7 @@
     <t>05-050206TC</t>
   </si>
   <si>
-    <t>e0fadaae9e7a01f3914884584a6b7517</t>
+    <t>49e6e8f9ed06e3212c670b1732af6eb3</t>
   </si>
   <si>
     <t>04-040013TM</t>
@@ -3725,7 +3725,7 @@
     <t>05-050304TC</t>
   </si>
   <si>
-    <t>c4fe35ca784828d1893f420a8d6d2832</t>
+    <t>799fbc74ee8253704912777ac54737ec</t>
   </si>
   <si>
     <t>03-030043TP</t>
@@ -3737,13 +3737,13 @@
     <t>05-050206A</t>
   </si>
   <si>
-    <t>ef1f7bc09084fe7e760fcd662b2c9eec</t>
+    <t>4ba2893dda91c9e205f8b0fa258cb7bd</t>
   </si>
   <si>
     <t>05-050315A</t>
   </si>
   <si>
-    <t>432f2b12e1f6894d2d49d0752077aa1d</t>
+    <t>4398dab51214844ae1f69721217b712f</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -3806,7 +3806,7 @@
     <t>05-050304TP</t>
   </si>
   <si>
-    <t>62150c20d121c8274d6f90ed3903f51d</t>
+    <t>69d13b3f4c7e12d5e837a43427a48a49</t>
   </si>
   <si>
     <t>04-040002TP</t>
@@ -3854,7 +3854,7 @@
     <t>05-050315TC</t>
   </si>
   <si>
-    <t>3460c0548689483b7415f521fbf687cb</t>
+    <t>35f22da182aa74db4d971175e1f7ff5a</t>
   </si>
   <si>
     <t>01-010046TM</t>
@@ -3869,7 +3869,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>5e4ab72ee31126c82067e63326a6968e</t>
+    <t>e147113dd5b8c706c06b2aadc32bb7ca</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -3893,7 +3893,7 @@
     <t>05-050207A</t>
   </si>
   <si>
-    <t>8cbba115c0d3741f462453bd485fd304</t>
+    <t>85e573f71f103e1bfc01a51dc4c1008f</t>
   </si>
   <si>
     <t>02-020006TM</t>
@@ -3944,7 +3944,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>d74eb364d395241e4a88ce4dd643a1b4</t>
+    <t>ec8bb2e90a05f054616078e7212bfab6</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4016,7 +4016,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>e43456585f774ed373438d7ef49f2aa3</t>
+    <t>5775b0c75e8855e415257f666150defd</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4037,7 +4037,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>f43b4a6f7cc8bf13c3a92b4b7f8e726d</t>
+    <t>03c66e267ded994d8dd5ddacb499fc1a</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4166,7 +4166,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>ea579b3f30efb72eb919c6a56f538c3e</t>
+    <t>0c1b8c3533265996ed8fa48d76099afa</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4373,7 +4373,7 @@
     <t>05-050202TC</t>
   </si>
   <si>
-    <t>58fca060a06c31d35ca37b7b32ae2d13</t>
+    <t>c84e23c3a8123f8e8bd33e3e35b003a0</t>
   </si>
   <si>
     <t>03-030062TP</t>
@@ -4391,7 +4391,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>7522cf9fbb024ae1c150b2151111be09</t>
+    <t>6ec8c0785f7b16239d4d000394e0bda0</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4418,7 +4418,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>fa838f54022d6a8979ed747fda2cb32f</t>
+    <t>59cda5b7f2ce6783165a8ae08efc6d92</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -4517,13 +4517,13 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>186b1a836d5aa29ca4cd018da9200e46</t>
+    <t>e4b2856774cbae42b1d120f2d9c0b332</t>
   </si>
   <si>
     <t>05-050002A</t>
   </si>
   <si>
-    <t>7509b2ca97b6b009aa96ff8bb2d842d5</t>
+    <t>7433bb1f821af1563b08782cd69ad453</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4553,7 +4553,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>1a091c654aec82de978d555c663bab50</t>
+    <t>ab7e9aa4427c9f9a8cf59a7b8ea39ae3</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -4580,7 +4580,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>2a07bf6c6c1eb49dfac0a251abbaf02f</t>
+    <t>9411a4c89dba8c34f087a4e12eb198f5</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4784,7 +4784,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>ee1b5d5b8ff266973aaea21d50fad9fa</t>
+    <t>59aef8db0712138bd6b475a7301a320e</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -4919,7 +4919,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>fa45adef370f900924977faca8daa50d</t>
+    <t>6a698cf8d62f24a329f480cae1e2141b</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode lun sep  6 04:13:45 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2681,7 +2681,7 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>dcedc3bb0496b5514f1f455c2762bfbb</t>
+    <t>921218d33f5bba627e2f373ae40219c2</t>
   </si>
   <si>
     <t>05-050311A</t>
@@ -2693,7 +2693,7 @@
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>1715ab406c35b7c24e90dcbb31ace64b</t>
+    <t>136907f84a1695f8305181af3522d5f1</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -3398,7 +3398,7 @@
     <t>05-050302TC</t>
   </si>
   <si>
-    <t>72c1a8e6f3d566ecac609952c138676c</t>
+    <t>7e066dfe45567d280d6a3ffbbf63c728</t>
   </si>
   <si>
     <t>01-110304-11030403TP</t>
@@ -4325,7 +4325,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>e54e7c48877447368243eafb48fab8ff</t>
+    <t>4ab8df049d5c4d0984ad02982e7e6850</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié sep  8 05:45:38 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -671,7 +671,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>3f3cb0272d91d93b8d9910216dd98b56</t>
+    <t>9b99ed5dfc22d6e656c41522c8d8880a</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>eac6d56063697c4696c84438a0564182</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -4604,7 +4604,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode lun sep 13 05:28:20 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -4604,7 +4604,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar oct  5 00:52:32 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>8506888276693576c92158880b2778a0</t>
+    <t>2ae1f19395183ed5b2388788b0763313</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -179,7 +179,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>e7c2c0aef67605ee2a88d1c598b2683f</t>
+    <t>3ab600f8362b7bcfde638b88e63a8edf</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -533,7 +533,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>89d8b8363a38e01d7a16c2da40df1f3c</t>
+    <t>981e561710c6392271f58d6d5de82ad8</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -590,7 +590,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>8cabc50ed25dbd573a6921609a339df7</t>
+    <t>005015f0be3db5f7e4cd377d5bae9a3d</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -1502,7 +1502,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>c6fa7b4bcd9efd33c0b46e83f0d3938d</t>
+    <t>473e2b694ed3b18268ad2c4e1f834416</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2450,7 +2450,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>a7094538211176a4493642127d720327</t>
+    <t>ed22506af71d0901f2e012d947ce109b</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -3371,7 +3371,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>f868f002b4016f6d6646129be2c2a6c1</t>
+    <t>83753fff470acdb2d7675839e5d94a25</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3473,7 +3473,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>9fbc1de2835461ce96e0d065fbdc2ccb</t>
+    <t>3509aa1997c3bcfb51b1a748dbd724ac</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3500,7 +3500,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>8b8f45498a8f0607cad6be289853893b</t>
+    <t>e7360a55096f740ab6e9aa80791956d2</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4073,7 +4073,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>042d3fe35e65dcec9484c707fdbd953d</t>
+    <t>44bb8b5c0ae4d1268d9bac033e211aee</t>
   </si>
   <si>
     <t>03-030062TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié oct  6 01:14:37 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -836,7 +836,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>50865ddaa756834b155e8a12a9fb6878</t>
+    <t>79c6fc1430a3f9e4f6e6c36542af1e17</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -866,7 +866,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>76f66f979d0ed127425772edced54f59</t>
+    <t>92b314f412ebbd43548831cc6d68d234</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2861,7 +2861,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>ac6440f27d6bdf0632f1ffe1730f4b3b</t>
+    <t>259e27a37f0d7f6eb129a5b2bc1816cf</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2966,7 +2966,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>2b690f85f54ad877602f070b51761aa2</t>
+    <t>a5bbea05ff12d3a39e488a47ddf51a4b</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4289,7 +4289,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>7ae182c84642edc5382f561eaa06598d</t>
+    <t>071ce4cf140698ffa659ba39f35e03c6</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4304,7 +4304,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>976c8f5e0985ab7716283e7852a946df</t>
+    <t>be3e17f9107a367b7bb00230db9b8e17</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue oct  7 04:37:03 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -101,7 +101,7 @@
     <t>05-050207TP</t>
   </si>
   <si>
-    <t>dd7be23b0a967f072967c7d89602e78f</t>
+    <t>6823801810e55ff4c050f38a91e4ee75</t>
   </si>
   <si>
     <t>915-150012A</t>
@@ -152,7 +152,7 @@
     <t>05-050316TC</t>
   </si>
   <si>
-    <t>fa8cb3c3b8b756132399d3332953b0bd</t>
+    <t>3962fd7b709886f150bd31bb3b07ca9e</t>
   </si>
   <si>
     <t>03-030059TP</t>
@@ -206,7 +206,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>9969a07157b2257f0fd8700132780393</t>
+    <t>e5cfcd4b711511c2aa6cacf2c915a266</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -656,7 +656,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>099acd20269d8221cd4fdb8b77193168</t>
+    <t>d7dc2244dcc7fecc58c0c3f61dbc3c9c</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -671,7 +671,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>9b99ed5dfc22d6e656c41522c8d8880a</t>
+    <t>ffc1acb4f56a9e3a2b0a163ba14a7197</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -725,7 +725,7 @@
     <t>05-050312TP</t>
   </si>
   <si>
-    <t>9480db809a06505fe676dccf85bf1d75</t>
+    <t>506c015a866fcfd78105d0dad33e5604</t>
   </si>
   <si>
     <t>05-0709-070954TC</t>
@@ -875,7 +875,7 @@
     <t>05-050308A</t>
   </si>
   <si>
-    <t>5fa90ebdbc289531432d123ecba8a9cd</t>
+    <t>ec4833957306512adf3cd6b652995fbb</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -974,7 +974,7 @@
     <t>05-050303TC</t>
   </si>
   <si>
-    <t>2f3b2814347a9ffef04fc451a611e891</t>
+    <t>df06acf56eb967b330d5b4c870ed029f</t>
   </si>
   <si>
     <t>01-010010TP</t>
@@ -1037,7 +1037,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>5c5ae8f115b3f8982c041013f59312e9</t>
+    <t>451d116ee64b5aa6bf3d70e50dc98460</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1079,7 +1079,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>e5cb158eb7c88f78f46fce5df8aa9b39</t>
+    <t>7c81ed8327f94681ddb71d7a034dd2ae</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1157,7 +1157,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>f1ac35b69c56c41e4086c6b0275d1479</t>
+    <t>f148727e7d1763d473f4e7d50a0d0537</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1202,7 +1202,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>1701cd60c0fd5c809f2a1e98dd85181c</t>
+    <t>0f0b95fa16b5e960960f40a05e998b7d</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1220,7 +1220,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>f359acb0bce62ddc8b0b443d3adad72a</t>
+    <t>ea9fa2a2d873e401a1d888c0f6376dc2</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1232,7 +1232,7 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>2537c24366e2e12fd3cb2e61066ec412</t>
+    <t>3ae556d2c06d358191ed2723760b46e4</t>
   </si>
   <si>
     <t>05-050304A</t>
@@ -1244,7 +1244,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>15e2dc221af3fce6b6db0833049ce66f</t>
+    <t>4b3e211c526bd74d156e50d353f2766a</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1262,7 +1262,7 @@
     <t>05-050205TC</t>
   </si>
   <si>
-    <t>b70d5a3413a2be3ab3b58ac3e96bd586</t>
+    <t>e3be78c7f7ac4ae739d60ebbe7e4cdc0</t>
   </si>
   <si>
     <t>04-040014TM</t>
@@ -1772,7 +1772,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>16900adb23af8ab043627443199b4fc5</t>
+    <t>c501e142b73504eb3b4a45e2f070a253</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -1793,7 +1793,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>b66efb5c6546772060de0ac4cbfd1afa</t>
+    <t>11835b3af42c6721df5009cb6446eec7</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2543,7 +2543,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>57d4113904f1dc0c137b2728c40d233c</t>
+    <t>2aad3b51d90da07c415874bee03ca5f1</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2555,7 +2555,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>73feff9b9fc889606338dd4511865eac</t>
+    <t>875fe72072dbc895784a534a5d3e2e28</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2636,7 +2636,7 @@
     <t>05-050208TC</t>
   </si>
   <si>
-    <t>988b94643e2660daa15f9c369f70b789</t>
+    <t>acbe1bd7f6caee304584eab28318db72</t>
   </si>
   <si>
     <t>03-030039A</t>
@@ -2717,7 +2717,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>e6f7e6ed8a816ffab3bd6a1833ee032c</t>
+    <t>d187e98f94589cff4479a0c30e4cbae3</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -2756,19 +2756,19 @@
     <t>05-050317TC</t>
   </si>
   <si>
-    <t>391af302ebda2244cf8770442ea1af07</t>
+    <t>de3989494a8d80f0e897ec548840e892</t>
   </si>
   <si>
     <t>05-050312A</t>
   </si>
   <si>
-    <t>3091490aa5b60503358cb85f6a8240cb</t>
+    <t>85b414f65cb310bc02d3b5a8d2e6aafa</t>
   </si>
   <si>
     <t>05-050009A</t>
   </si>
   <si>
-    <t>4f87d9f7a205a1dbbe49e3a094de731b</t>
+    <t>2ddf8a6cbdefcc7ff12aea3e3911f860</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -2813,7 +2813,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>b490a8599bb44f03e16e699f50a3053b</t>
+    <t>db8b3e160875855515bd36f32b37d052</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -3149,7 +3149,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>5714d0a0107259283cbc6a8b9eeda9e7</t>
+    <t>7c10915904a1cd481a667b799bde08c7</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3398,7 +3398,7 @@
     <t>05-050302TC</t>
   </si>
   <si>
-    <t>7e066dfe45567d280d6a3ffbbf63c728</t>
+    <t>8221a623c2222a4c1107cf2575720ec5</t>
   </si>
   <si>
     <t>01-110304-11030403TP</t>
@@ -3551,7 +3551,7 @@
     <t>05-050317A</t>
   </si>
   <si>
-    <t>005c764de734828fc6bdbbb991f36770</t>
+    <t>1120433771da77469c9c1baa4818b120</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -3743,7 +3743,7 @@
     <t>05-050315A</t>
   </si>
   <si>
-    <t>4398dab51214844ae1f69721217b712f</t>
+    <t>9f197d1576d87a37f72bad3a0091e36e</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -3854,7 +3854,7 @@
     <t>05-050315TC</t>
   </si>
   <si>
-    <t>35f22da182aa74db4d971175e1f7ff5a</t>
+    <t>18b5b6b7843e3a0c6b5e24f7bb284379</t>
   </si>
   <si>
     <t>01-010046TM</t>
@@ -3869,7 +3869,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>e147113dd5b8c706c06b2aadc32bb7ca</t>
+    <t>04737aab45fd06f3fd0b30259466fa71</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -3893,7 +3893,7 @@
     <t>05-050207A</t>
   </si>
   <si>
-    <t>85e573f71f103e1bfc01a51dc4c1008f</t>
+    <t>e9fb843323e7e79fdc96daf231e22da8</t>
   </si>
   <si>
     <t>02-020006TM</t>
@@ -3944,7 +3944,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>ec8bb2e90a05f054616078e7212bfab6</t>
+    <t>2000fef9b593309d512616c5c0518c00</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4517,7 +4517,7 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>e4b2856774cbae42b1d120f2d9c0b332</t>
+    <t>3bbb92af73a72d21d7d114abb9b296f8</t>
   </si>
   <si>
     <t>05-050002A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie oct  8 02:57:17 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -65,7 +65,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>af31c33312e9cbdceb91ba1cae619041</t>
+    <t>a86f172abe92d0af60bb4038d98e03cc</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>825b50c1077bcc44e9142241e49f1cff</t>
+    <t>742299c11e8c8c59bb7b5f603c1a2e6a</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -689,7 +689,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>01a7a415f0359063e9a59e03cafd8e98</t>
+    <t>db7c7e498b94191bfcd16c6c448b1bfe</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -740,7 +740,7 @@
     <t>05-050312TC</t>
   </si>
   <si>
-    <t>0e5cabff8af1d5481b7c3e17d8c96c98</t>
+    <t>4bc214ce4cd72bd503d49b28e9677a7d</t>
   </si>
   <si>
     <t>03-030055TP</t>
@@ -860,7 +860,7 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>12d24d38c646234d7d05cda9ca8b8076</t>
+    <t>6f475003b91ee3cb78018a7d7aa84e9e</t>
   </si>
   <si>
     <t>05-050007TP</t>
@@ -917,7 +917,7 @@
     <t>05-050203TC</t>
   </si>
   <si>
-    <t>26b3c81df830df1b8eab5101e091d8b5</t>
+    <t>6fbc15156804e5c603f7f7383995e795</t>
   </si>
   <si>
     <t>01-110304-11030404A</t>
@@ -947,7 +947,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>56c15d873c55652037efa85c0e61256c</t>
+    <t>3baf8294f342ef57a23dda7f24b84723</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -992,7 +992,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>800d717efa91ff5a59b84a895bd97196</t>
+    <t>61fc802ceecea34bcfdce0bb4d73e14a</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1088,7 +1088,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>9bcfbfdd1d28207dd0d0df4d04d0a876</t>
+    <t>55ee5d6fedc9f640bc37338056a6d408</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1238,7 +1238,7 @@
     <t>05-050304A</t>
   </si>
   <si>
-    <t>f5123e7de2b78d32a70a6953346246ce</t>
+    <t>cbf8650ebfbd315aa407fe5d6cdc6125</t>
   </si>
   <si>
     <t>05-050009TP</t>
@@ -1331,7 +1331,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>bd0c190fdc6ad6858e7db26ed0e1a31c</t>
+    <t>17b8ca1165f6afe47a21d97f4370e838</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1490,7 +1490,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>36c11d492334114e57cd2f6887dc8b58</t>
+    <t>4213e11a1866120908a41b7a6ecab2f4</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1520,7 +1520,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>9f1c93a1b6c164b4b600c0f09e89154f</t>
+    <t>054b87ac6fadadd77b8661668567f1f0</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1589,7 +1589,7 @@
     <t>05-050310TC</t>
   </si>
   <si>
-    <t>25e887e5583f35372283f28e92d27333</t>
+    <t>617afa5dc0b30aa909f7923714c33519</t>
   </si>
   <si>
     <t>04-040004A</t>
@@ -1637,7 +1637,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>a36c23993dcd2e15a775968f6ac17b5b</t>
+    <t>5f246cc1a85f7556167eab5089df9d7e</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1817,7 +1817,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>29364419b881cb3062a9df4ab7349651</t>
+    <t>ef09ea01ea7b15344d6373f9dc7dd6e4</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2189,7 +2189,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>e1f70a292fb3beb643a4f3e43fe7ee57</t>
+    <t>7ba966fe073162d183913402b06c2788</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2372,7 +2372,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>868e881d8cfa61e7418a181b49c7601e</t>
+    <t>f5a87edab6b688b0022e06744f79f6ae</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2444,7 +2444,7 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>7e11d9dbca5e14a6169d3edcd00a5c32</t>
+    <t>470fe079d9166ba4ca5b84ea164d6910</t>
   </si>
   <si>
     <t>05-050313A</t>
@@ -2687,13 +2687,13 @@
     <t>05-050311A</t>
   </si>
   <si>
-    <t>f79c33d32f08b5ff0aa0bd9fcef6dc2c</t>
+    <t>64725d32d6cbf89c19fdb2b51d148b2d</t>
   </si>
   <si>
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>136907f84a1695f8305181af3522d5f1</t>
+    <t>4eedab6b746da735ee74177a709f6dbe</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -2774,7 +2774,7 @@
     <t>05-050203A</t>
   </si>
   <si>
-    <t>3b6268853f1fa8bd68839f0ef7b0f77b</t>
+    <t>812e573b5585b1c6c53c90b7bdc481d5</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -2930,7 +2930,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>eb6dfa8ffd370531febde8b59adcfd16</t>
+    <t>ce7ffbd88adb00583fb4e8593eff66d7</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -2948,7 +2948,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>d4bebbf518230ca2aa990ad2dc7e13ac</t>
+    <t>13f34be79aabcc1359e23da555501037</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3023,7 +3023,7 @@
     <t>05-050308TC</t>
   </si>
   <si>
-    <t>a967e55f38ad4dd7eb150b3d0c03f0e5</t>
+    <t>f8b18eafb45143d6543fd78519b50745</t>
   </si>
   <si>
     <t>02-020002TC</t>
@@ -3041,7 +3041,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>0b9c566e0f5b6d1080d7457b397c03ca</t>
+    <t>16c70f51260e8c5c0939474556b261f3</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3077,7 +3077,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>66c801a01056005954e9d18be923ab21</t>
+    <t>fe25c468e050060b993e21d48d781d5c</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3308,7 +3308,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>69506d8e29770012b06f21a3ef06de36</t>
+    <t>2e5cc65730065762e8d4798d35dbe0ce</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3362,7 +3362,7 @@
     <t>05-050204TC</t>
   </si>
   <si>
-    <t>c34def8415f15a56ed6c596d8adda356</t>
+    <t>6543d552b980d758663d9fdf72dbd8e2</t>
   </si>
   <si>
     <t>04-040015TM</t>
@@ -3545,7 +3545,7 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>01659c7eafacf6dee84b8f9830f0152d</t>
+    <t>32af589514444a64350b4c5fbc8493d6</t>
   </si>
   <si>
     <t>05-050317A</t>
@@ -3617,7 +3617,7 @@
     <t>05-050206TP</t>
   </si>
   <si>
-    <t>1411adebe1166b57dc7540f57ea16da0</t>
+    <t>6d044d451d14db10e2c453db8aa92744</t>
   </si>
   <si>
     <t>01-010068TM</t>
@@ -3641,7 +3641,7 @@
     <t>05-050206TC</t>
   </si>
   <si>
-    <t>49e6e8f9ed06e3212c670b1732af6eb3</t>
+    <t>14a771ce45abc6edbfcd34d40012eac5</t>
   </si>
   <si>
     <t>04-040013TM</t>
@@ -3725,7 +3725,7 @@
     <t>05-050304TC</t>
   </si>
   <si>
-    <t>799fbc74ee8253704912777ac54737ec</t>
+    <t>c6ad7d5b48a7d6eed7c323ac6b15f70a</t>
   </si>
   <si>
     <t>03-030043TP</t>
@@ -3737,7 +3737,7 @@
     <t>05-050206A</t>
   </si>
   <si>
-    <t>4ba2893dda91c9e205f8b0fa258cb7bd</t>
+    <t>0916ccc9bf552a3cd0790ce6e8c6866e</t>
   </si>
   <si>
     <t>05-050315A</t>
@@ -3806,7 +3806,7 @@
     <t>05-050304TP</t>
   </si>
   <si>
-    <t>69d13b3f4c7e12d5e837a43427a48a49</t>
+    <t>315430436be5f0cd7880be6c439ef769</t>
   </si>
   <si>
     <t>04-040002TP</t>
@@ -4016,7 +4016,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>5775b0c75e8855e415257f666150defd</t>
+    <t>ee83d77ea509e0749a780583f558a49d</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4037,7 +4037,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>03c66e267ded994d8dd5ddacb499fc1a</t>
+    <t>7761ed1e94332377519ba1879fb3b0e6</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4166,7 +4166,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>0c1b8c3533265996ed8fa48d76099afa</t>
+    <t>d0c92177875d9b21edc2cdad9dc20843</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4373,7 +4373,7 @@
     <t>05-050202TC</t>
   </si>
   <si>
-    <t>c84e23c3a8123f8e8bd33e3e35b003a0</t>
+    <t>f51180a9ac2797328f08d09b056ea6be</t>
   </si>
   <si>
     <t>03-030062TP</t>
@@ -4391,7 +4391,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>6ec8c0785f7b16239d4d000394e0bda0</t>
+    <t>5ed77c6ae06fb8ef2acdd1d2547f74d8</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4418,7 +4418,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>59cda5b7f2ce6783165a8ae08efc6d92</t>
+    <t>79745fa3e156d88d9fe3840de4c7cbc4</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -4523,7 +4523,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>7433bb1f821af1563b08782cd69ad453</t>
+    <t>9358ae6f70c031b6ae2680958026ad73</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4553,7 +4553,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>ab7e9aa4427c9f9a8cf59a7b8ea39ae3</t>
+    <t>253716e49b083d7a2c7422ea39a44c5d</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -4580,7 +4580,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>9411a4c89dba8c34f087a4e12eb198f5</t>
+    <t>343fcaf6e9e6a1ad265752fa513dc6bf</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4604,7 +4604,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>
@@ -4784,7 +4784,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>59aef8db0712138bd6b475a7301a320e</t>
+    <t>0386ac6b6a8521d246cae9e8aaa264c4</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -4919,7 +4919,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>6a698cf8d62f24a329f480cae1e2141b</t>
+    <t>2509c347b18298d5dd28d09dd89d9bb8</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb oct  9 05:24:00 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2681,7 +2681,7 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>921218d33f5bba627e2f373ae40219c2</t>
+    <t>0469b64bb08b560959c1a4b120224755</t>
   </si>
   <si>
     <t>05-050311A</t>
@@ -4325,7 +4325,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>4ab8df049d5c4d0984ad02982e7e6850</t>
+    <t>a32272aa3859c328aa744788c8f65243</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode lun oct 11 04:49:56 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -4604,7 +4604,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar oct 12 05:27:14 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -4604,7 +4604,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié oct 13 05:39:32 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -4604,7 +4604,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue oct 14 05:56:02 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -4604,7 +4604,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie oct 29 01:33:10 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1472,7 +1472,7 @@
     <t>01-080101-010112TM</t>
   </si>
   <si>
-    <t>8c6e2b75376b8490b816902250befb49</t>
+    <t>0e4158b3be5756e9866cace2776c8db4</t>
   </si>
   <si>
     <t>01-010025TP</t>
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
   </si>
   <si>
     <t>01-010007TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie oct 29 12:51:10 CEST 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1990" uniqueCount="1695">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1990" uniqueCount="1696">
   <si>
     <t>05-050305TM</t>
   </si>
@@ -29,13 +29,13 @@
     <t>01-010050TP</t>
   </si>
   <si>
-    <t>af91f3692b5c2a074c3f4fbe008ebd6f</t>
+    <t>821d617ccb748bee004129e886366b23</t>
   </si>
   <si>
     <t>01-010035A</t>
   </si>
   <si>
-    <t>4a97e7dfbcdd2b1a8476f0dd150a01ef</t>
+    <t>41719c71caba7b1e33163ba72bfe84aa</t>
   </si>
   <si>
     <t>03-030029A</t>
@@ -107,7 +107,7 @@
     <t>915-150012A</t>
   </si>
   <si>
-    <t>09d75f98149a07c4a0583ae9ca10de4d</t>
+    <t>4b44cb446163485ebb0b311da4abdcc6</t>
   </si>
   <si>
     <t>05-050305TP</t>
@@ -119,7 +119,7 @@
     <t>05-0709-070921BTP</t>
   </si>
   <si>
-    <t>4c6f84b27dcccd77f694c10531a70268</t>
+    <t>05b9491f51ef494cb7e34dadbef1270e</t>
   </si>
   <si>
     <t>01-010010A</t>
@@ -173,7 +173,7 @@
     <t>01-010050TC</t>
   </si>
   <si>
-    <t>f701fc6735e33393ae9dfc09dc1f862b</t>
+    <t>0b806737ac696a894d996b6499d5d1a8</t>
   </si>
   <si>
     <t>05-050302A</t>
@@ -188,19 +188,19 @@
     <t>05-0709-070921BTC</t>
   </si>
   <si>
-    <t>5fd184f870d2af27239c7755601859fa</t>
+    <t>5852ad166ec6983e1f7c2f03b75d3bd2</t>
   </si>
   <si>
     <t>03-030004A</t>
   </si>
   <si>
-    <t>6d62a0557ea936e302361742a90bbf2d</t>
+    <t>4f28fb248e974767ac37a0dceefd7331</t>
   </si>
   <si>
     <t>915-150011A</t>
   </si>
   <si>
-    <t>378ab1f948c4e84c7e2344d013d62a55</t>
+    <t>53fe8e276ff06c3fd44492c69d21f244</t>
   </si>
   <si>
     <t>05-050316TP</t>
@@ -212,7 +212,7 @@
     <t>915-150018TP</t>
   </si>
   <si>
-    <t>62e8009b0bb43fe17664e9f2373a6c8c</t>
+    <t>0993f7a58024c6a48ac3ce721114a5c8</t>
   </si>
   <si>
     <t>03-02010301-030102A</t>
@@ -221,7 +221,7 @@
     <t>915-150018TM</t>
   </si>
   <si>
-    <t>39b20a4d3a33d1313cc52833ba6c0bca</t>
+    <t>b45ce4eb58b920538ebcc1d43fc0184b</t>
   </si>
   <si>
     <t>01-010057A</t>
@@ -248,7 +248,7 @@
     <t>05-0709-070908TC</t>
   </si>
   <si>
-    <t>9908c29b7fab4cef9c80ff46dcf03af6</t>
+    <t>5400dab8b05a98ab638b37351beb6afa</t>
   </si>
   <si>
     <t>05-050105A</t>
@@ -278,19 +278,19 @@
     <t>915-150018TC</t>
   </si>
   <si>
-    <t>6a8ff615cdb00a46b4e5c0f541ed124b</t>
+    <t>a56d0a49802668923272ffd81f20ec30</t>
   </si>
   <si>
     <t>915-150007TP</t>
   </si>
   <si>
-    <t>7d576524d3c4fc8fef7b58eb5f8f284d</t>
+    <t>61fbcac4a0e40b79503dbfe09a088dbc</t>
   </si>
   <si>
     <t>01-010063TP</t>
   </si>
   <si>
-    <t>b3f7614824357fe5c8b54b6288c09e92</t>
+    <t>e7f908c55a61b9f4c5f7a987985fd925</t>
   </si>
   <si>
     <t>01-010032A</t>
@@ -302,7 +302,7 @@
     <t>915-150007TM</t>
   </si>
   <si>
-    <t>b367758740bae7360eac1bc8e5e38bc2</t>
+    <t>6c894387e4343caaa722bdb22cc24fb6</t>
   </si>
   <si>
     <t>01-010063TM</t>
@@ -338,7 +338,7 @@
     <t>05-0709-070908TM</t>
   </si>
   <si>
-    <t>67b7c9f494638cfa165a2cb3d182fc27</t>
+    <t>0f2b5a283bbd0fa2e6f4d204e75a45fb</t>
   </si>
   <si>
     <t>03-030026A</t>
@@ -353,7 +353,7 @@
     <t>05-0709-070908TP</t>
   </si>
   <si>
-    <t>4e05305223e360a8e38718a184190ecd</t>
+    <t>c66752fff0d24cd595df16cead8321f4</t>
   </si>
   <si>
     <t>03-030002A</t>
@@ -368,7 +368,7 @@
     <t>915-150007TC</t>
   </si>
   <si>
-    <t>0159658a61ec1e54769b3e111cd5e338</t>
+    <t>49747575b2941f2d7b203570ce685586</t>
   </si>
   <si>
     <t>04-040012TP</t>
@@ -392,7 +392,7 @@
     <t>905-9050607-905060702TM</t>
   </si>
   <si>
-    <t>b0bfef82cb938c7b37b82ac03dd92e02</t>
+    <t>de587608272e7642fea45dc6a4eec7b4</t>
   </si>
   <si>
     <t>01-010055A</t>
@@ -419,7 +419,7 @@
     <t>905-9050607-905060702TP</t>
   </si>
   <si>
-    <t>9d1d568df4a0a88312f112aaa595d6c1</t>
+    <t>3ff638c668f8683b3239757c18b1bd75</t>
   </si>
   <si>
     <t>03-030025A</t>
@@ -431,7 +431,7 @@
     <t>03-030001A</t>
   </si>
   <si>
-    <t>e9080851709b95373d75ab3d52b1eed3</t>
+    <t>508c4b7f803246bcf6e5c5169d743a75</t>
   </si>
   <si>
     <t>05-050307TP</t>
@@ -446,7 +446,7 @@
     <t>905-9050607-905060702TC</t>
   </si>
   <si>
-    <t>bc13665eac829680b6a0efac910209a9</t>
+    <t>3e37fab3289964e163748ae1ae0dc5eb</t>
   </si>
   <si>
     <t>01-010030A</t>
@@ -533,7 +533,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>981e561710c6392271f58d6d5de82ad8</t>
+    <t>a6a4ad04bd595317b0079bb650a01d78</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -575,7 +575,7 @@
     <t>915-150009TM</t>
   </si>
   <si>
-    <t>c90124b7b564c8fd04454539d0804182</t>
+    <t>1a44f6d0f05186195bc181a560434d4d</t>
   </si>
   <si>
     <t>01-010065TM</t>
@@ -590,7 +590,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>005015f0be3db5f7e4cd377d5bae9a3d</t>
+    <t>0fec58aacd6a62d325a1710fbf7dc0cf</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -602,7 +602,7 @@
     <t>915-150009TP</t>
   </si>
   <si>
-    <t>8c9538fa6d11f86766a4e3d63d121b0e</t>
+    <t>d2e7587229c3885463b891d3614cc054</t>
   </si>
   <si>
     <t>04-040021TC</t>
@@ -632,7 +632,7 @@
     <t>915-150009TC</t>
   </si>
   <si>
-    <t>c44933a8687ca715bd1e53da6d63de28</t>
+    <t>99142123935409b93c41af5ec368f9b2</t>
   </si>
   <si>
     <t>04-040010TP</t>
@@ -665,7 +665,7 @@
     <t>04-040014TC</t>
   </si>
   <si>
-    <t>a412ce738c555f504b3c2fc2563a4afe</t>
+    <t>87a5e69893d7f7e018944f9895caf1d9</t>
   </si>
   <si>
     <t>05-050301TC</t>
@@ -695,7 +695,7 @@
     <t>04-040003TP</t>
   </si>
   <si>
-    <t>9e948857ded2a8589cde9e2d0d74f7f7</t>
+    <t>65691ef982935fd3b44ba3dd108cd83f</t>
   </si>
   <si>
     <t>01-010019A</t>
@@ -710,7 +710,7 @@
     <t>04-040003TM</t>
   </si>
   <si>
-    <t>cd96b58e7ba840c9698dfaad67319aad</t>
+    <t>8faa25e5191430c9e9919d991f82646a</t>
   </si>
   <si>
     <t>01-110304-11030403A</t>
@@ -719,7 +719,7 @@
     <t>01-010043TM</t>
   </si>
   <si>
-    <t>b0a11a3971ce3c114ec540c1c518bf4f</t>
+    <t>7880cb33e90d0f0bb0dad5532b72c6d6</t>
   </si>
   <si>
     <t>05-050312TP</t>
@@ -734,7 +734,7 @@
     <t>04-040003TC</t>
   </si>
   <si>
-    <t>11cbe408a34939d2f06c53505a4dfbb8</t>
+    <t>73ad8a2aeacf9e3eeff989980e0e8450</t>
   </si>
   <si>
     <t>05-050312TC</t>
@@ -830,13 +830,13 @@
     <t>01-010043TC</t>
   </si>
   <si>
-    <t>e7b56bcf0d89e5e16dceb6f97a42f1f9</t>
+    <t>4eabe142441c98a110c9ee12d712cfe6</t>
   </si>
   <si>
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>79c6fc1430a3f9e4f6e6c36542af1e17</t>
+    <t>b65a056e377dd16eedcda4f04a751251</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -866,7 +866,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>92b314f412ebbd43548831cc6d68d234</t>
+    <t>26775f8fb4f7818f49d5dc49b38a3129</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1007,7 +1007,7 @@
     <t>05-0709-070906AA</t>
   </si>
   <si>
-    <t>ec1698ab8e6353b5c9c7fcc6b4c8e660</t>
+    <t>1d10f1f6af396db708ccf4ee098150ca</t>
   </si>
   <si>
     <t>01-010067TC</t>
@@ -1061,13 +1061,13 @@
     <t>05-0709-070910TC</t>
   </si>
   <si>
-    <t>b7d2fb4e6114387d8b68a8ec6efef78b</t>
+    <t>8ef4cd605a3cf46667f8182712494327</t>
   </si>
   <si>
     <t>05-0709-070910TM</t>
   </si>
   <si>
-    <t>c7b13c896d79f110af279a23b4fc0266</t>
+    <t>8d7e340b825b66d5861497c1e780ddc2</t>
   </si>
   <si>
     <t>01-010045TP</t>
@@ -1100,7 +1100,7 @@
     <t>05-0709-070906BA</t>
   </si>
   <si>
-    <t>8eb157a8fa1bbe10c34f8a5bf203d4b3</t>
+    <t>90d8ac6682832f94ac5098dfcf75478f</t>
   </si>
   <si>
     <t>01-010056TC</t>
@@ -1163,7 +1163,7 @@
     <t>05-0709-070910TP</t>
   </si>
   <si>
-    <t>bb9ffa8ad25621f081e6aa7a6eb95859</t>
+    <t>3e431fb07fb0f6c9694ec63ca9dc0768</t>
   </si>
   <si>
     <t>01-010045TC</t>
@@ -1214,7 +1214,7 @@
     <t>03-030006A</t>
   </si>
   <si>
-    <t>8db38e28a1f46406c8d92bc388bb0885</t>
+    <t>2449228716b6538cd66d5bc8c14cf808</t>
   </si>
   <si>
     <t>05-050009TM</t>
@@ -1253,7 +1253,7 @@
     <t>04-040014TP</t>
   </si>
   <si>
-    <t>a6aa62789d57a04a889943c1037ac8a7</t>
+    <t>0defa52e30cb2325fa7a2ac126c3721d</t>
   </si>
   <si>
     <t>03-030042TC</t>
@@ -1268,7 +1268,7 @@
     <t>04-040014TM</t>
   </si>
   <si>
-    <t>492d3a39d5a70a93cd6c37e584ad93d6</t>
+    <t>fca3f688af13cc97c5e08c9d3cdb5ec4</t>
   </si>
   <si>
     <t>03-02010301-030089TM</t>
@@ -1298,7 +1298,7 @@
     <t>01-080101-010091TM</t>
   </si>
   <si>
-    <t>19fc0070b6cb6aaf7ebcf6b8d1e992db</t>
+    <t>3485dcb96c4cad67ffca40b22f7a021a</t>
   </si>
   <si>
     <t>01-010058TM</t>
@@ -1400,7 +1400,7 @@
     <t>01-080101-010091TC</t>
   </si>
   <si>
-    <t>4eb30eab2e23b782208c6a5b2be44559</t>
+    <t>6954b707057466638bc105dedcc0ae2b</t>
   </si>
   <si>
     <t>03-030041TP</t>
@@ -1502,7 +1502,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>473e2b694ed3b18268ad2c4e1f834416</t>
+    <t>70a8a24919664930809e813e115083b9</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -1544,7 +1544,7 @@
     <t>915-150011TP</t>
   </si>
   <si>
-    <t>0c26fd91b9125946602969e60614ecb8</t>
+    <t>e854ca8a23b47c0d6e9010f4816e8974</t>
   </si>
   <si>
     <t>01-010014TP</t>
@@ -1571,7 +1571,7 @@
     <t>905-9050607-905060701A</t>
   </si>
   <si>
-    <t>b2a61c1c546004cbbd4486f2e85dab05</t>
+    <t>7e910355cac59aae9cdb5abe67f245c8</t>
   </si>
   <si>
     <t>01-080101-010093TM</t>
@@ -1604,7 +1604,7 @@
     <t>915-150011TC</t>
   </si>
   <si>
-    <t>856b6031b20a0979bfaf8d26d1b23bbe</t>
+    <t>08fee30ea443d574b66bedbbb56d1561</t>
   </si>
   <si>
     <t>03-030008TP</t>
@@ -1619,7 +1619,7 @@
     <t>915-150011TM</t>
   </si>
   <si>
-    <t>903bb20630a8ace4e47ca2fd1a725f41</t>
+    <t>6f20c78dbc6676815780eb9ecb83d509</t>
   </si>
   <si>
     <t>03-030072TP</t>
@@ -1652,7 +1652,7 @@
     <t>01-010049TP</t>
   </si>
   <si>
-    <t>bd28a05aac77a0bd798d2871eedfbe58</t>
+    <t>bfb7a011b20a35d6c9a0d8ffa3efe1ac</t>
   </si>
   <si>
     <t>01-010003TP</t>
@@ -1673,7 +1673,7 @@
     <t>01-010049TM</t>
   </si>
   <si>
-    <t>8154777e2c8ce05773d7088ed02de109</t>
+    <t>e956c7a7df01a3d09562f57bb09129a4</t>
   </si>
   <si>
     <t>01-080101-010082TM</t>
@@ -1685,7 +1685,7 @@
     <t>04-040003A</t>
   </si>
   <si>
-    <t>d743159f8dd21ff896b707521e0082c6</t>
+    <t>7741b7ed09595472064d877c3a04e492</t>
   </si>
   <si>
     <t>03-02010301-030081A</t>
@@ -1712,7 +1712,7 @@
     <t>05-0709-070902TC</t>
   </si>
   <si>
-    <t>b40b1af66372a7b4200f93a3b9a705ab</t>
+    <t>78141aa3ad407c25ee10a705a2793344</t>
   </si>
   <si>
     <t>03-02010301-030097TC</t>
@@ -1727,7 +1727,7 @@
     <t>03-02010301-030097TM</t>
   </si>
   <si>
-    <t>5311dc722c4fc5a1ee66cca5a4ad5f46</t>
+    <t>2634a1798d1a3c6dfbcfd59bb211ad92</t>
   </si>
   <si>
     <t>03-030050TC</t>
@@ -1799,7 +1799,7 @@
     <t>905-9050607-905060702A</t>
   </si>
   <si>
-    <t>e1021bea513ab0537bc4df13105d9737</t>
+    <t>2b7ace009c184cf0272a47b51bbb0c02</t>
   </si>
   <si>
     <t>03-030061TC</t>
@@ -1811,7 +1811,7 @@
     <t>05-0709-070902TP</t>
   </si>
   <si>
-    <t>852dd907a8027478a4daf60cf9088c2c</t>
+    <t>a321218770d54c1ead7b42d941944f6d</t>
   </si>
   <si>
     <t>05-050201TP</t>
@@ -1823,13 +1823,13 @@
     <t>05-0709-070902TM</t>
   </si>
   <si>
-    <t>2db18754cfde08b840d87e01bd99babb</t>
+    <t>7ba26e807a4cb398bb150a7885740e96</t>
   </si>
   <si>
     <t>915-150009A</t>
   </si>
   <si>
-    <t>27162f060b503dd3b03739e69f99cdf5</t>
+    <t>c385735a4c483d51f2ae13a1c253cf21</t>
   </si>
   <si>
     <t>05-050201TM</t>
@@ -1865,19 +1865,19 @@
     <t>05-0709-070906ATC</t>
   </si>
   <si>
-    <t>1d538b85277d28472a82b08c1972ef36</t>
+    <t>d272e12677169965add2053d711e3d48</t>
   </si>
   <si>
     <t>915-150013TP</t>
   </si>
   <si>
-    <t>0bc8bdf73950f50bb65c5e87bf7c5d77</t>
+    <t>7b84711152414e4c246f740725ddb603</t>
   </si>
   <si>
     <t>03-030006TC</t>
   </si>
   <si>
-    <t>67e89ce88d11a78c862620a61b3f2f70</t>
+    <t>0f44e0ea975115699e243e0508f30d3a</t>
   </si>
   <si>
     <t>03-030006TM</t>
@@ -1889,7 +1889,7 @@
     <t>02-020001TC</t>
   </si>
   <si>
-    <t>16e8cb4dbf50ec4e86c7fa64fe380541</t>
+    <t>9591a6121b5000e5a91a52ea1e8530c1</t>
   </si>
   <si>
     <t>01-010016TP</t>
@@ -1919,7 +1919,7 @@
     <t>05-0709-070906ATM</t>
   </si>
   <si>
-    <t>c28618037e25e3704c441d1b6fd012db</t>
+    <t>3dd7fdf4f82e75464d8723fdbaa9d6a8</t>
   </si>
   <si>
     <t>03-030070TC</t>
@@ -1931,19 +1931,19 @@
     <t>05-0709-070906ATP</t>
   </si>
   <si>
-    <t>d2366e3876160ff8d83a9104aaef04fe</t>
+    <t>7342a9f55328567957fa51a1215fe113</t>
   </si>
   <si>
     <t>915-150013TC</t>
   </si>
   <si>
-    <t>06d4b0df2e3daa2e6f3952151324d3c2</t>
+    <t>306a82df144581f68cff1eb662f27375</t>
   </si>
   <si>
     <t>915-150013TM</t>
   </si>
   <si>
-    <t>9e2b479681aec8331992d5e2e269b068</t>
+    <t>291a632eed38372a2118a845060580f8</t>
   </si>
   <si>
     <t>03-030045A</t>
@@ -1955,7 +1955,7 @@
     <t>05-0709-070910A</t>
   </si>
   <si>
-    <t>ca3bc93378cdc336fb1d23bfd0287161</t>
+    <t>4829f40c44dcec27a667170ba36b3818</t>
   </si>
   <si>
     <t>01-010074A</t>
@@ -2009,13 +2009,13 @@
     <t>01-010050A</t>
   </si>
   <si>
-    <t>172db03539e2184365cf33be7505021b</t>
+    <t>8911b65ff0adc6263b52dd7272d2332f</t>
   </si>
   <si>
     <t>02-020001TM</t>
   </si>
   <si>
-    <t>10cb88bbcdcba6564f4634c1c3e628ef</t>
+    <t>10ef3d705ebb46abf3fa5a21b5e047d7</t>
   </si>
   <si>
     <t>01-080101-010084TP</t>
@@ -2039,7 +2039,7 @@
     <t>02-020001TP</t>
   </si>
   <si>
-    <t>1d2a0fad47aed368e039d0d34410fcec</t>
+    <t>b201805672b67168e40e217b6a6ebb82</t>
   </si>
   <si>
     <t>03-02010301-030091TC</t>
@@ -2105,13 +2105,13 @@
     <t>915-150015TP</t>
   </si>
   <si>
-    <t>ca9a0ce7200f67ff0f489c634cd576bf</t>
+    <t>ad1f80c8a38b25554200cea4225df193</t>
   </si>
   <si>
     <t>03-030004TC</t>
   </si>
   <si>
-    <t>ab039e8b28b07cb439eb3fe7f2a6baee</t>
+    <t>0dd543a2b7142033c57bf093f5631b3a</t>
   </si>
   <si>
     <t>01-010018TC</t>
@@ -2129,7 +2129,7 @@
     <t>915-150015TM</t>
   </si>
   <si>
-    <t>aec11b26aac47ff6bdcac8864b6f5cbf</t>
+    <t>72124e51ca8fbad9a299073b8ccbe1a6</t>
   </si>
   <si>
     <t>901-010202-9010102022TC</t>
@@ -2144,7 +2144,7 @@
     <t>03-030004TP</t>
   </si>
   <si>
-    <t>84a1a9aff333a40f7b93ff13f396825b</t>
+    <t>83f377bdb33260c4ca151c226f670d2e</t>
   </si>
   <si>
     <t>03-030004TM</t>
@@ -2153,7 +2153,7 @@
     <t>915-150015TC</t>
   </si>
   <si>
-    <t>363b8da5a43db16b69f56ba299c69d4a</t>
+    <t>1e80b3d0df570694e83ec8c84bcc78ca</t>
   </si>
   <si>
     <t>04-040009TC</t>
@@ -2204,7 +2204,7 @@
     <t>915-150004TP</t>
   </si>
   <si>
-    <t>19796459bde6467c01113b81816d466f</t>
+    <t>ffed5a323c47487b53ac2cadb90868ab</t>
   </si>
   <si>
     <t>01-010060TP</t>
@@ -2225,7 +2225,7 @@
     <t>915-150004TM</t>
   </si>
   <si>
-    <t>2fe5f54c0a0d39a3106d13918c7f78a7</t>
+    <t>b046fedaf21e139c91af0947c19d4c24</t>
   </si>
   <si>
     <t>01-010060TM</t>
@@ -2234,7 +2234,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
+    <t>4d90c661e98736dfc9bc7228ed2a11e5</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2261,7 +2261,7 @@
     <t>915-150004TC</t>
   </si>
   <si>
-    <t>c3d15ba386f49a4a89cff768392ffa95</t>
+    <t>0fa37d4e516c6457cb1d73aacb9154b7</t>
   </si>
   <si>
     <t>03-030040A</t>
@@ -2282,7 +2282,7 @@
     <t>05-0709-070905BTP</t>
   </si>
   <si>
-    <t>c3a6bebf959923ce3ad21b967d0b2062</t>
+    <t>0ace74bd4d5e14e304eb72587aa1e207</t>
   </si>
   <si>
     <t>01-010007TP</t>
@@ -2405,13 +2405,13 @@
     <t>915-150017TP</t>
   </si>
   <si>
-    <t>2882a2cb40dba8d87f6ef93f3dc9b3b3</t>
+    <t>0bf208eae38e5873692b84a66f8fb2ca</t>
   </si>
   <si>
     <t>915-150017TM</t>
   </si>
   <si>
-    <t>ec21d5055c8849c0238a64995935b9ac</t>
+    <t>49281bf4f40ead942888b810674ffdb9</t>
   </si>
   <si>
     <t>01-010023A</t>
@@ -2438,7 +2438,7 @@
     <t>05-0709-070909TC</t>
   </si>
   <si>
-    <t>4e57d31c81b8f0b4e80c3d80a51d4c70</t>
+    <t>b8d747b6a2f4360f473ec24392463b45</t>
   </si>
   <si>
     <t>05-050204A</t>
@@ -2474,7 +2474,7 @@
     <t>915-150017TC</t>
   </si>
   <si>
-    <t>466d1df6ad4f7853fa33b6bca722803d</t>
+    <t>4370bf2a6c612a26ee49dfc30ab5e233</t>
   </si>
   <si>
     <t>01-010009TC</t>
@@ -2549,7 +2549,7 @@
     <t>04-040011TM</t>
   </si>
   <si>
-    <t>9c97e798b02676a3ca40e0f0ef22b628</t>
+    <t>c9509a175aee0e574dc1a10d5352122b</t>
   </si>
   <si>
     <t>05-050314A</t>
@@ -2564,7 +2564,7 @@
     <t>05-0709-070909TM</t>
   </si>
   <si>
-    <t>3dcb045817c3098469dbe3b3069eb83d</t>
+    <t>9f49a98543ca027eb508621e1fb91e3b</t>
   </si>
   <si>
     <t>01-010009TP</t>
@@ -2576,7 +2576,7 @@
     <t>03-030001TC</t>
   </si>
   <si>
-    <t>ac5faa7b24db5e3a4281517c9b86466e</t>
+    <t>b160c7ec0a78a8efefbead291473c70e</t>
   </si>
   <si>
     <t>03-030047TC</t>
@@ -2588,7 +2588,7 @@
     <t>05-0709-070909TP</t>
   </si>
   <si>
-    <t>1651e0a559aaee0fdaf68eecd726d95c</t>
+    <t>f32062aa5e28d6309651fc09b2df374b</t>
   </si>
   <si>
     <t>04-040011TP</t>
@@ -2606,7 +2606,7 @@
     <t>905-9050607-905060701TM</t>
   </si>
   <si>
-    <t>e0e5a8781dbac31946c52f46dcd95db7</t>
+    <t>1c8a64a363632393752b560f5a6a2f10</t>
   </si>
   <si>
     <t>01-010051TP</t>
@@ -2618,7 +2618,7 @@
     <t>905-9050607-905060701TP</t>
   </si>
   <si>
-    <t>1f4766a2be0c799e3c5310f4e0f5c983</t>
+    <t>6c00b36e0eaa8e4dcd941f8ed587f786</t>
   </si>
   <si>
     <t>01-010045A</t>
@@ -2723,7 +2723,7 @@
     <t>905-9050607-905060701TC</t>
   </si>
   <si>
-    <t>caf0902acd5e4ab007abd4dbb31c1a66</t>
+    <t>b6968f3f8506bbe85976337f02c79a14</t>
   </si>
   <si>
     <t>01-010062TC</t>
@@ -2807,7 +2807,7 @@
     <t>05-0709-070903A</t>
   </si>
   <si>
-    <t>935ef81b9fb805a4be34a828255ed1c9</t>
+    <t>4aaa92afb0abaea7fcdadb713098ba12</t>
   </si>
   <si>
     <t>05-050317TP</t>
@@ -2879,7 +2879,7 @@
     <t>05-0709-070902A</t>
   </si>
   <si>
-    <t>b28a09c762509387e269714acae243b2</t>
+    <t>ee108dfa4ade719dfc394066af30f874</t>
   </si>
   <si>
     <t>03-030013A</t>
@@ -2891,7 +2891,7 @@
     <t>01-010064TP</t>
   </si>
   <si>
-    <t>d152e0b7e58e4c0a3b12fbe91d962f80</t>
+    <t>61af9898f6bd8e9b0b8cc5ef77622c3a</t>
   </si>
   <si>
     <t>03-90205-0205_007A</t>
@@ -2906,7 +2906,7 @@
     <t>915-150008TM</t>
   </si>
   <si>
-    <t>32137b737f73b05333e215fb77c16587</t>
+    <t>f85e80bd8c13c6c66f07235d826f385f</t>
   </si>
   <si>
     <t>01-010064TM</t>
@@ -2954,7 +2954,7 @@
     <t>915-150008TP</t>
   </si>
   <si>
-    <t>4c36003fcffd031a25a22fbbe3a1ca63</t>
+    <t>ac8cf6c32ece5e43ac3f79ebad48ed51</t>
   </si>
   <si>
     <t>01-010075TC</t>
@@ -2966,7 +2966,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>a5bbea05ff12d3a39e488a47ddf51a4b</t>
+    <t>579451a92beef97da558af495ebe8606</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -2978,7 +2978,7 @@
     <t>05-0709-070901A</t>
   </si>
   <si>
-    <t>e6ece49d19fe9fdfa605f0790e42ec84</t>
+    <t>b46da07bb323bdbffc5d0cfa704f77e6</t>
   </si>
   <si>
     <t>03-030012A</t>
@@ -2996,7 +2996,7 @@
     <t>915-150008TC</t>
   </si>
   <si>
-    <t>6e672982fa194296a2efa95bac027c65</t>
+    <t>9518f3d56e3f5e0f6059671e877e498d</t>
   </si>
   <si>
     <t>03-02010301-030100TC</t>
@@ -3017,7 +3017,7 @@
     <t>03-030001TM</t>
   </si>
   <si>
-    <t>2f7eb22ff6ad0ca3d69e86974d03036b</t>
+    <t>ead04ed2740ceb084a3f0ce234470464</t>
   </si>
   <si>
     <t>05-050308TC</t>
@@ -3029,7 +3029,7 @@
     <t>02-020002TC</t>
   </si>
   <si>
-    <t>a3ee29141986a4326417d8abaf0d6c3b</t>
+    <t>417016e5a0ec9e73fd288ff16d22d782</t>
   </si>
   <si>
     <t>03-030047TP</t>
@@ -3047,7 +3047,7 @@
     <t>03-030001TP</t>
   </si>
   <si>
-    <t>ce67bdb572db24e4f6a2a30199fbe017</t>
+    <t>c30b13a5f0820e4e3c43214a99090270</t>
   </si>
   <si>
     <t>03-030047TM</t>
@@ -3101,7 +3101,7 @@
     <t>01-010042TM</t>
   </si>
   <si>
-    <t>ed9f4b5680ebb02261d1eb6cc016f9a4</t>
+    <t>842636dc1e868b133495f4c2822e30a8</t>
   </si>
   <si>
     <t>03-030012TM</t>
@@ -3155,7 +3155,7 @@
     <t>01-080101-010089TM</t>
   </si>
   <si>
-    <t>c557d1831e9be763f4fc83df83adf496</t>
+    <t>f6bfb4fdedde97622b8a9058dcdeb57a</t>
   </si>
   <si>
     <t>03-030058A</t>
@@ -3173,7 +3173,7 @@
     <t>02-020002TM</t>
   </si>
   <si>
-    <t>918d0f6d00993ac69e708551f5e7e685</t>
+    <t>93d7e9998659a16749e560d868f6e77a</t>
   </si>
   <si>
     <t>01-010053TC</t>
@@ -3185,7 +3185,7 @@
     <t>02-020002TP</t>
   </si>
   <si>
-    <t>64b83428c51981a8982ff0dc2928eeb6</t>
+    <t>a306edc42f7ab2f4a339be49a216ffcb</t>
   </si>
   <si>
     <t>01-010031TP</t>
@@ -3224,7 +3224,7 @@
     <t>915-150008A</t>
   </si>
   <si>
-    <t>372abfffb38b2dc96240a099ef34c8d4</t>
+    <t>df19891eae88e9c353acb3c0f9238ac6</t>
   </si>
   <si>
     <t>05-0709-070955TP</t>
@@ -3248,7 +3248,7 @@
     <t>01-010042TC</t>
   </si>
   <si>
-    <t>922fbfeb06bc04374c9b8582e84c655d</t>
+    <t>d678389545d7e835d100ebc2f8ed9cca</t>
   </si>
   <si>
     <t>03-030032TC</t>
@@ -3260,7 +3260,7 @@
     <t>03-030032TM</t>
   </si>
   <si>
-    <t>0bab210f526a9fc6401ce27133db8695</t>
+    <t>e921ee20a692464fa072920c7b478c40</t>
   </si>
   <si>
     <t>03-030078TM</t>
@@ -3314,7 +3314,7 @@
     <t>915-150007A</t>
   </si>
   <si>
-    <t>8bf4d4b70def7c3e1618c64e37847534</t>
+    <t>cafd5b65cc2ec420f27ccaa633e56e54</t>
   </si>
   <si>
     <t>05-050204TM</t>
@@ -3578,7 +3578,7 @@
     <t>01-010022TM</t>
   </si>
   <si>
-    <t>656a006cbcf7ec2b05e7d214903ff9f2</t>
+    <t>d906ce77b292c21e5f235b858758d7a8</t>
   </si>
   <si>
     <t>03-030030TP</t>
@@ -3590,7 +3590,7 @@
     <t>01-010002A</t>
   </si>
   <si>
-    <t>35629bd494fb012622aba1a361a71f50</t>
+    <t>169b297b7fff24b881c52844b61284f0</t>
   </si>
   <si>
     <t>01-010026A</t>
@@ -3632,7 +3632,7 @@
     <t>05-0709-070909A</t>
   </si>
   <si>
-    <t>31cfbe580fe6dfa303d681e53f909b80</t>
+    <t>dfc6091f934fc5044cfda2da5a67bfe3</t>
   </si>
   <si>
     <t>05-050206TM</t>
@@ -3647,7 +3647,7 @@
     <t>04-040013TM</t>
   </si>
   <si>
-    <t>d90a7dff71d15179e07e07d8d49cfe8e</t>
+    <t>2fe9e38eb071602504cde8eff31fe52e</t>
   </si>
   <si>
     <t>03-030041TC</t>
@@ -3659,7 +3659,7 @@
     <t>04-040013TP</t>
   </si>
   <si>
-    <t>901335dcb975050b3a06ba2bb478fb2d</t>
+    <t>2677e6917f5f9c5aa9daaa462655b2df</t>
   </si>
   <si>
     <t>01-010011TM</t>
@@ -3710,7 +3710,7 @@
     <t>04-040013TC</t>
   </si>
   <si>
-    <t>5d36b099269766af24b39475fff3e8e3</t>
+    <t>3591178de414aee03e8df5bbfe0638dd</t>
   </si>
   <si>
     <t>01-010011TP</t>
@@ -3755,25 +3755,25 @@
     <t>05-0709-070908A</t>
   </si>
   <si>
-    <t>7392593711ab7bb3250d7e56e6dece16</t>
+    <t>a570bf9870c8beb68d7d03210d5b6f2c</t>
   </si>
   <si>
     <t>01-010022TC</t>
   </si>
   <si>
-    <t>e9d235c08e4c1c94c33f933f84de5cef</t>
+    <t>18fa7188d999ad4ba17761497e898d64</t>
   </si>
   <si>
     <t>01-010049A</t>
   </si>
   <si>
-    <t>cc393fd4da76289572f103c2edfb820d</t>
+    <t>1b165eb937c09f4de7e61b497d3863c7</t>
   </si>
   <si>
     <t>05-0709-070905AA</t>
   </si>
   <si>
-    <t>b63bbf7509084a2b7b03ebc9663565f9</t>
+    <t>6b00962aa51e03e90db15ec9f0d86e8f</t>
   </si>
   <si>
     <t>01-080101-010110TP</t>
@@ -3788,7 +3788,7 @@
     <t>915-150002A</t>
   </si>
   <si>
-    <t>74bc5bcce3784988c2080f7367ac96d1</t>
+    <t>ae9e80c0c022799a39445a2399c8fe6e</t>
   </si>
   <si>
     <t>03-030054TC</t>
@@ -3824,7 +3824,7 @@
     <t>05-0709-070921ATP</t>
   </si>
   <si>
-    <t>ea3f030a8a490b970f7da01d292fecd4</t>
+    <t>74476aad8ebce81639d2b214aaafd947</t>
   </si>
   <si>
     <t>01-010024A</t>
@@ -3881,13 +3881,13 @@
     <t>02-020006TC</t>
   </si>
   <si>
-    <t>2802ab1063279d54146223f696f20eb3</t>
+    <t>863e39fef68f7fa45e955c21edad39b0</t>
   </si>
   <si>
     <t>05-0709-070921ATC</t>
   </si>
   <si>
-    <t>f0e5c24140c9cb41727b2a54e3a260c8</t>
+    <t>deab5c160b3856a617105a2bec99a5e9</t>
   </si>
   <si>
     <t>05-050207A</t>
@@ -3899,7 +3899,7 @@
     <t>02-020006TM</t>
   </si>
   <si>
-    <t>fb6579275369feca2249f6a62946d497</t>
+    <t>6a9b8ebe912b307b25cda9cc6184e098</t>
   </si>
   <si>
     <t>902-0204-02040101BTM</t>
@@ -3920,19 +3920,19 @@
     <t>05-0709-070905BA</t>
   </si>
   <si>
-    <t>6fcb607af1cb60af2252a39f7d1745de</t>
+    <t>265b93a97a6e7762073090ed8bd68ce6</t>
   </si>
   <si>
     <t>02-020006TP</t>
   </si>
   <si>
-    <t>45cce2fdc22e2cfd7fa5302a2e549dab</t>
+    <t>0cbd0f8fba9b7654d2c9e52df7e20192</t>
   </si>
   <si>
     <t>915-150001A</t>
   </si>
   <si>
-    <t>bbb159c371c7188bcb1da38b8b6d591f</t>
+    <t>81d184e5ea89069a9746708c27ba9b3a</t>
   </si>
   <si>
     <t>03-030065TC</t>
@@ -3962,7 +3962,7 @@
     <t>05-0709-070901TC</t>
   </si>
   <si>
-    <t>ed8d0f2e534d224e43bcd71563f0f88b</t>
+    <t>01b6ff12abce8f078560254cddfc1627</t>
   </si>
   <si>
     <t>03-02010301-030096TC</t>
@@ -3971,19 +3971,19 @@
     <t>05-0709-070901TM</t>
   </si>
   <si>
-    <t>a7c1dadd7ec65360b7f5725a4cbe5b52</t>
+    <t>fee68621940ff3e17fd834505ea2331f</t>
   </si>
   <si>
     <t>01-010035TP</t>
   </si>
   <si>
-    <t>edf354052625762b4b29e5510944d1cf</t>
+    <t>6490fabded0eb05a792536ed212a3e3e</t>
   </si>
   <si>
     <t>01-010035TM</t>
   </si>
   <si>
-    <t>e5555af19ade7cb69b3de639b53efbe2</t>
+    <t>9d4902c0a081edff9aa839214ab773dc</t>
   </si>
   <si>
     <t>03-030073A</t>
@@ -4052,13 +4052,13 @@
     <t>05-0709-070901TP</t>
   </si>
   <si>
-    <t>ba34bad9b6e7c800a1ade4e878ae97ca</t>
+    <t>397ba27f653d891ebe59029a6f0dab43</t>
   </si>
   <si>
     <t>01-010035TC</t>
   </si>
   <si>
-    <t>535b9101700329efe947e9ed77b67f67</t>
+    <t>50f3d5dd6de63f6f2ef93eb78f2564ba</t>
   </si>
   <si>
     <t>03-02010301-030097A</t>
@@ -4073,7 +4073,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>44bb8b5c0ae4d1268d9bac033e211aee</t>
+    <t>4c26779b04aeb6357d6d674c0a29a362</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4160,7 +4160,7 @@
     <t>03-030075TC</t>
   </si>
   <si>
-    <t>1dd2ae8d880542e886ef8a0209785ad8</t>
+    <t>108dc20ead86ac9393e968a56ddbf757</t>
   </si>
   <si>
     <t>05-050002TC</t>
@@ -4172,13 +4172,13 @@
     <t>03-030075TP</t>
   </si>
   <si>
-    <t>4275c97ed1a790378ff8d6467314d457</t>
+    <t>6eeff8e5ccfdab36c3b0a066b9bdbb66</t>
   </si>
   <si>
     <t>03-030075TM</t>
   </si>
   <si>
-    <t>8faee9629b60f43f0634f2f8efb568d4</t>
+    <t>c8670ec4e105f8c3246ecc1e391e16c4</t>
   </si>
   <si>
     <t>01-010048TC</t>
@@ -4199,13 +4199,13 @@
     <t>01-010002TM</t>
   </si>
   <si>
-    <t>b1b88d90fa7d6865d68888cf1e30c1b8</t>
+    <t>002835f1d5546c3b330e10097ccbdc55</t>
   </si>
   <si>
     <t>01-010002TP</t>
   </si>
   <si>
-    <t>1b26a4858ebe756a23b4d8e5281c487e</t>
+    <t>0cca9b1731114d9a37c688f6079a9756</t>
   </si>
   <si>
     <t>03-030070A</t>
@@ -4238,7 +4238,7 @@
     <t>05-0709-070903TC</t>
   </si>
   <si>
-    <t>dfb41bc87eb854e2b99e152486144459</t>
+    <t>655ea82c1cd5f1a39de0c488797ceb33</t>
   </si>
   <si>
     <t>01-010037TC</t>
@@ -4277,7 +4277,7 @@
     <t>01-010002TC</t>
   </si>
   <si>
-    <t>2367230e0e9179c07dffed373205d81b</t>
+    <t>a7baf553fd3303b88d87616b23993853</t>
   </si>
   <si>
     <t>03-02010301-030094A</t>
@@ -4310,6 +4310,9 @@
     <t>05-050006TM</t>
   </si>
   <si>
+    <t>f902c0c65af0ce991e7c7e13b50b8236</t>
+  </si>
+  <si>
     <t>05-050104TC</t>
   </si>
   <si>
@@ -4331,7 +4334,7 @@
     <t>05-0709-070903TM</t>
   </si>
   <si>
-    <t>b4e3ba5466c57f698549f42028666b21</t>
+    <t>60bc3633d16921f4896c881995a4e52e</t>
   </si>
   <si>
     <t>03-02010301-030093A</t>
@@ -4349,7 +4352,7 @@
     <t>05-0709-070903TP</t>
   </si>
   <si>
-    <t>d8ef158d83f87a66c3dcaa3efb83d98e</t>
+    <t>e9530b989030d7acff041a50998e3855</t>
   </si>
   <si>
     <t>04-040017TM</t>
@@ -4397,7 +4400,7 @@
     <t>04-040014A</t>
   </si>
   <si>
-    <t>3bbeda48cc454f005a899945f7dbc5cd</t>
+    <t>1b6ed3b3a92747c4d0e386b2f9f87036</t>
   </si>
   <si>
     <t>03-02010301-030092A</t>
@@ -4442,7 +4445,7 @@
     <t>915-150001TP</t>
   </si>
   <si>
-    <t>fb8bdd52c88c645604e93c2f67b8f429</t>
+    <t>0c127b5f0172ed781a509349e6c28409</t>
   </si>
   <si>
     <t>01-010004TP</t>
@@ -4472,7 +4475,7 @@
     <t>04-040013A</t>
   </si>
   <si>
-    <t>97220f71e67f3b425088a394f3a84b22</t>
+    <t>e441fe22d2b6b1f8e98bd23734f91e23</t>
   </si>
   <si>
     <t>03-02010301-030085TM</t>
@@ -4481,7 +4484,7 @@
     <t>915-150001TC</t>
   </si>
   <si>
-    <t>3c8fe25a6d9290e0a1321791ef223075</t>
+    <t>0ee05b216d187cd84b1366bfd9caf193</t>
   </si>
   <si>
     <t>03-02010301-030091A</t>
@@ -4490,7 +4493,7 @@
     <t>915-150001TM</t>
   </si>
   <si>
-    <t>767187267aeb43374fa487d09b04d827</t>
+    <t>d3e31586fc0f238413a108d7c84e733b</t>
   </si>
   <si>
     <t>03-02010301-030092TC</t>
@@ -4508,7 +4511,7 @@
     <t>01-010039TC</t>
   </si>
   <si>
-    <t>7a5683a1bed4ff3e2674c0c7d869e083</t>
+    <t>1f91ba663c5d24d29a8a88b3b45b8af5</t>
   </si>
   <si>
     <t>03-030029TC</t>
@@ -4529,7 +4532,7 @@
     <t>01-010039TM</t>
   </si>
   <si>
-    <t>ef898df150aa366cade8df3324848dbf</t>
+    <t>7cfd5035d1ebc32c5b2e72d83c64bb55</t>
   </si>
   <si>
     <t>01-080101-010084A</t>
@@ -4562,7 +4565,7 @@
     <t>03-030033A</t>
   </si>
   <si>
-    <t>5651ddd7888be309a021eb04eadb21e4</t>
+    <t>15e040aac52534eb1e5fdf489255be7c</t>
   </si>
   <si>
     <t>03-02010301-030102TC</t>
@@ -4616,13 +4619,13 @@
     <t>915-150014TP</t>
   </si>
   <si>
-    <t>ebdec01a6b309e3748d9754a298a2ebb</t>
+    <t>e095021e161529e65617f068d8eacd08</t>
   </si>
   <si>
     <t>05-0709-070906BTC</t>
   </si>
   <si>
-    <t>ff0372bf9239fb61a080e87ed3195bd4</t>
+    <t>948d665e3651e517e7ba26c501a65a10</t>
   </si>
   <si>
     <t>01-010017TC</t>
@@ -4646,7 +4649,7 @@
     <t>915-150014TM</t>
   </si>
   <si>
-    <t>57e6a5c84dd98419a196f687ba7da1cf</t>
+    <t>1ca3c1484e483fc4f4a9f3f57da3afba</t>
   </si>
   <si>
     <t>901-010202-9010102023TC</t>
@@ -4682,7 +4685,7 @@
     <t>05-0709-070906BTM</t>
   </si>
   <si>
-    <t>dab242bab5bc7656d6a1f3e354d7d51e</t>
+    <t>dbee2729cb23d5bd7600ef69e57d464b</t>
   </si>
   <si>
     <t>03-030071TC</t>
@@ -4694,7 +4697,7 @@
     <t>915-150014TC</t>
   </si>
   <si>
-    <t>ec565bb99879f865a731ab258df28300</t>
+    <t>aca0e08bd02ff79f804a3d1d3f23c4ec</t>
   </si>
   <si>
     <t>01-010115TC</t>
@@ -4706,7 +4709,7 @@
     <t>05-0709-070906BTP</t>
   </si>
   <si>
-    <t>602b4fb729c08f06791474bf1a154eb1</t>
+    <t>3ed0674e3f47802436055ef0aee8cd25</t>
   </si>
   <si>
     <t>03-030007TP</t>
@@ -4742,7 +4745,7 @@
     <t>915-150003TP</t>
   </si>
   <si>
-    <t>6c8a48c4793f647ae22e6415d1918f72</t>
+    <t>fce84300477d16728114d72d4f7f8c5f</t>
   </si>
   <si>
     <t>01-080101-010083TC</t>
@@ -4754,7 +4757,7 @@
     <t>05-0709-070905ATC</t>
   </si>
   <si>
-    <t>b2f44d3255fdd42d13a8b4353660a499</t>
+    <t>059a421cbf7df830f6ac6bf08b052994</t>
   </si>
   <si>
     <t>01-010006TC</t>
@@ -4772,7 +4775,7 @@
     <t>915-150003TM</t>
   </si>
   <si>
-    <t>b98caff4d64e24b295aa661bef3da148</t>
+    <t>b7a6d29a9cba82cd87d582fa13a4bd8b</t>
   </si>
   <si>
     <t>01-080101-010083TM</t>
@@ -4823,13 +4826,13 @@
     <t>915-150003TC</t>
   </si>
   <si>
-    <t>cba30d7950a13a0c0967661dd8f1ded3</t>
+    <t>35058e423177b5c2a1d9a3311e909735</t>
   </si>
   <si>
     <t>05-0709-070905ATP</t>
   </si>
   <si>
-    <t>b213c4e2488ad106b7235cb5839dce7a</t>
+    <t>9d0ae80615e37b264f45d02edcddf360</t>
   </si>
   <si>
     <t>03-030018TP</t>
@@ -4880,7 +4883,7 @@
     <t>05-0709-070921AA</t>
   </si>
   <si>
-    <t>95060d6e31bc91f2529e80a514b7f8a5</t>
+    <t>48ceb0bb5e2337ee5eb66697c3577418</t>
   </si>
   <si>
     <t>03-02010301-030094TP</t>
@@ -4898,7 +4901,7 @@
     <t>03-02010301-030094TM</t>
   </si>
   <si>
-    <t>5d277c98d807f951754f80bb69f75730</t>
+    <t>e803f7f4aa3331ae0d7c50f00e3f9fd8</t>
   </si>
   <si>
     <t>03-030077A</t>
@@ -4907,7 +4910,7 @@
     <t>02-020006A</t>
   </si>
   <si>
-    <t>0739e4252751d56b83824b70b671b54d</t>
+    <t>2369ec9edb1081bafb40644aa89da109</t>
   </si>
   <si>
     <t>03-030053A</t>
@@ -4937,7 +4940,7 @@
     <t>05-0709-070921BA</t>
   </si>
   <si>
-    <t>74ae33be2fdccb45346e846d82e80256</t>
+    <t>388219a416373a3bd84b66165eec03cb</t>
   </si>
   <si>
     <t>03-030076A</t>
@@ -4961,7 +4964,7 @@
     <t>915-150016TP</t>
   </si>
   <si>
-    <t>252258ccc0477f771cfa7f7fff6e2847</t>
+    <t>ce1b21339d84c5b978949d033b30414d</t>
   </si>
   <si>
     <t>03-030005TC</t>
@@ -4973,7 +4976,7 @@
     <t>915-150016TM</t>
   </si>
   <si>
-    <t>cddf31685c87ea1f10494c5af2604c98</t>
+    <t>22e4bccc3e21839772d7f2ed46a745fe</t>
   </si>
   <si>
     <t>901-010202-9010102021TC</t>
@@ -5012,7 +5015,7 @@
     <t>915-150016TC</t>
   </si>
   <si>
-    <t>164564ca6182282ff0c3c6b63f6c25c6</t>
+    <t>2a91eeed6df5af4e3324f09910f32329</t>
   </si>
   <si>
     <t>01-080101-010085TC</t>
@@ -11869,12 +11872,12 @@
         <v>1431</v>
       </c>
       <c r="B842" t="s">
-        <v>1</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="843">
       <c r="A843" t="s">
-        <v>1432</v>
+        <v>1433</v>
       </c>
       <c r="B843" t="s">
         <v>1</v>
@@ -11882,15 +11885,15 @@
     </row>
     <row r="844">
       <c r="A844" t="s">
-        <v>1433</v>
+        <v>1434</v>
       </c>
       <c r="B844" t="s">
-        <v>1434</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="845">
       <c r="A845" t="s">
-        <v>1435</v>
+        <v>1436</v>
       </c>
       <c r="B845" t="s">
         <v>1</v>
@@ -11898,23 +11901,23 @@
     </row>
     <row r="846">
       <c r="A846" t="s">
-        <v>1436</v>
+        <v>1437</v>
       </c>
       <c r="B846" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="847">
       <c r="A847" t="s">
-        <v>1438</v>
+        <v>1439</v>
       </c>
       <c r="B847" t="s">
-        <v>1439</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="848">
       <c r="A848" t="s">
-        <v>1440</v>
+        <v>1441</v>
       </c>
       <c r="B848" t="s">
         <v>1</v>
@@ -11922,7 +11925,7 @@
     </row>
     <row r="849">
       <c r="A849" t="s">
-        <v>1441</v>
+        <v>1442</v>
       </c>
       <c r="B849" t="s">
         <v>1</v>
@@ -11930,31 +11933,31 @@
     </row>
     <row r="850">
       <c r="A850" t="s">
-        <v>1442</v>
+        <v>1443</v>
       </c>
       <c r="B850" t="s">
-        <v>1443</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="851">
       <c r="A851" t="s">
-        <v>1444</v>
+        <v>1445</v>
       </c>
       <c r="B851" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="852">
       <c r="A852" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="B852" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="853">
       <c r="A853" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="B853" t="s">
         <v>1</v>
@@ -11962,15 +11965,15 @@
     </row>
     <row r="854">
       <c r="A854" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
       <c r="B854" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="855">
       <c r="A855" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
       <c r="B855" t="s">
         <v>1</v>
@@ -11978,47 +11981,47 @@
     </row>
     <row r="856">
       <c r="A856" t="s">
-        <v>1452</v>
+        <v>1453</v>
       </c>
       <c r="B856" t="s">
-        <v>1453</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="857">
       <c r="A857" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
       <c r="B857" t="s">
-        <v>1455</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="858">
       <c r="A858" t="s">
-        <v>1456</v>
+        <v>1457</v>
       </c>
       <c r="B858" t="s">
-        <v>1457</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="859">
       <c r="A859" t="s">
-        <v>1458</v>
+        <v>1459</v>
       </c>
       <c r="B859" t="s">
-        <v>1459</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="860">
       <c r="A860" t="s">
-        <v>1460</v>
+        <v>1461</v>
       </c>
       <c r="B860" t="s">
-        <v>1461</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="861">
       <c r="A861" t="s">
-        <v>1462</v>
+        <v>1463</v>
       </c>
       <c r="B861" t="s">
         <v>1</v>
@@ -12026,103 +12029,103 @@
     </row>
     <row r="862">
       <c r="A862" t="s">
-        <v>1463</v>
+        <v>1464</v>
       </c>
       <c r="B862" t="s">
-        <v>1464</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="863">
       <c r="A863" t="s">
-        <v>1465</v>
+        <v>1466</v>
       </c>
       <c r="B863" t="s">
-        <v>1466</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="864">
       <c r="A864" t="s">
-        <v>1467</v>
+        <v>1468</v>
       </c>
       <c r="B864" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="865">
       <c r="A865" t="s">
-        <v>1469</v>
+        <v>1470</v>
       </c>
       <c r="B865" t="s">
-        <v>1470</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="866">
       <c r="A866" t="s">
-        <v>1471</v>
+        <v>1472</v>
       </c>
       <c r="B866" t="s">
-        <v>1472</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="867">
       <c r="A867" t="s">
-        <v>1473</v>
+        <v>1474</v>
       </c>
       <c r="B867" t="s">
-        <v>1474</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="868">
       <c r="A868" t="s">
-        <v>1475</v>
+        <v>1476</v>
       </c>
       <c r="B868" t="s">
-        <v>1476</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="869">
       <c r="A869" t="s">
-        <v>1477</v>
+        <v>1478</v>
       </c>
       <c r="B869" t="s">
-        <v>1478</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="870">
       <c r="A870" t="s">
-        <v>1479</v>
+        <v>1480</v>
       </c>
       <c r="B870" t="s">
-        <v>1480</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="871">
       <c r="A871" t="s">
-        <v>1481</v>
+        <v>1482</v>
       </c>
       <c r="B871" t="s">
-        <v>1482</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="872">
       <c r="A872" t="s">
-        <v>1483</v>
+        <v>1484</v>
       </c>
       <c r="B872" t="s">
-        <v>1484</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="873">
       <c r="A873" t="s">
-        <v>1485</v>
+        <v>1486</v>
       </c>
       <c r="B873" t="s">
-        <v>1486</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="874">
       <c r="A874" t="s">
-        <v>1487</v>
+        <v>1488</v>
       </c>
       <c r="B874" t="s">
         <v>1</v>
@@ -12130,15 +12133,15 @@
     </row>
     <row r="875">
       <c r="A875" t="s">
-        <v>1488</v>
+        <v>1489</v>
       </c>
       <c r="B875" t="s">
-        <v>1489</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="876">
       <c r="A876" t="s">
-        <v>1490</v>
+        <v>1491</v>
       </c>
       <c r="B876" t="s">
         <v>1</v>
@@ -12146,15 +12149,15 @@
     </row>
     <row r="877">
       <c r="A877" t="s">
-        <v>1491</v>
+        <v>1492</v>
       </c>
       <c r="B877" t="s">
-        <v>1492</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="878">
       <c r="A878" t="s">
-        <v>1493</v>
+        <v>1494</v>
       </c>
       <c r="B878" t="s">
         <v>1</v>
@@ -12162,15 +12165,15 @@
     </row>
     <row r="879">
       <c r="A879" t="s">
-        <v>1494</v>
+        <v>1495</v>
       </c>
       <c r="B879" t="s">
-        <v>1495</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="880">
       <c r="A880" t="s">
-        <v>1496</v>
+        <v>1497</v>
       </c>
       <c r="B880" t="s">
         <v>75</v>
@@ -12178,15 +12181,15 @@
     </row>
     <row r="881">
       <c r="A881" t="s">
-        <v>1497</v>
+        <v>1498</v>
       </c>
       <c r="B881" t="s">
-        <v>1498</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="882">
       <c r="A882" t="s">
-        <v>1499</v>
+        <v>1500</v>
       </c>
       <c r="B882" t="s">
         <v>1</v>
@@ -12194,39 +12197,39 @@
     </row>
     <row r="883">
       <c r="A883" t="s">
-        <v>1500</v>
+        <v>1501</v>
       </c>
       <c r="B883" t="s">
-        <v>1501</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="884">
       <c r="A884" t="s">
-        <v>1502</v>
+        <v>1503</v>
       </c>
       <c r="B884" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="885">
       <c r="A885" t="s">
-        <v>1504</v>
+        <v>1505</v>
       </c>
       <c r="B885" t="s">
-        <v>1505</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="886">
       <c r="A886" t="s">
-        <v>1506</v>
+        <v>1507</v>
       </c>
       <c r="B886" t="s">
-        <v>1507</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="887">
       <c r="A887" t="s">
-        <v>1508</v>
+        <v>1509</v>
       </c>
       <c r="B887" t="s">
         <v>1</v>
@@ -12234,7 +12237,7 @@
     </row>
     <row r="888">
       <c r="A888" t="s">
-        <v>1509</v>
+        <v>1510</v>
       </c>
       <c r="B888" t="s">
         <v>1</v>
@@ -12242,7 +12245,7 @@
     </row>
     <row r="889">
       <c r="A889" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
       <c r="B889" t="s">
         <v>1</v>
@@ -12250,7 +12253,7 @@
     </row>
     <row r="890">
       <c r="A890" t="s">
-        <v>1511</v>
+        <v>1512</v>
       </c>
       <c r="B890" t="s">
         <v>1</v>
@@ -12258,15 +12261,15 @@
     </row>
     <row r="891">
       <c r="A891" t="s">
-        <v>1512</v>
+        <v>1513</v>
       </c>
       <c r="B891" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="892">
       <c r="A892" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="B892" t="s">
         <v>1</v>
@@ -12274,15 +12277,15 @@
     </row>
     <row r="893">
       <c r="A893" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
       <c r="B893" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="894">
       <c r="A894" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="B894" t="s">
         <v>1</v>
@@ -12290,7 +12293,7 @@
     </row>
     <row r="895">
       <c r="A895" t="s">
-        <v>1518</v>
+        <v>1519</v>
       </c>
       <c r="B895" t="s">
         <v>1</v>
@@ -12298,7 +12301,7 @@
     </row>
     <row r="896">
       <c r="A896" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="B896" t="s">
         <v>1</v>
@@ -12306,7 +12309,7 @@
     </row>
     <row r="897">
       <c r="A897" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="B897" t="s">
         <v>1</v>
@@ -12314,23 +12317,23 @@
     </row>
     <row r="898">
       <c r="A898" t="s">
-        <v>1521</v>
+        <v>1522</v>
       </c>
       <c r="B898" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="899">
       <c r="A899" t="s">
-        <v>1523</v>
+        <v>1524</v>
       </c>
       <c r="B899" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="900">
       <c r="A900" t="s">
-        <v>1525</v>
+        <v>1526</v>
       </c>
       <c r="B900" t="s">
         <v>1</v>
@@ -12338,7 +12341,7 @@
     </row>
     <row r="901">
       <c r="A901" t="s">
-        <v>1526</v>
+        <v>1527</v>
       </c>
       <c r="B901" t="s">
         <v>1</v>
@@ -12346,79 +12349,79 @@
     </row>
     <row r="902">
       <c r="A902" t="s">
-        <v>1527</v>
+        <v>1528</v>
       </c>
       <c r="B902" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="903">
       <c r="A903" t="s">
-        <v>1529</v>
+        <v>1530</v>
       </c>
       <c r="B903" t="s">
-        <v>1530</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="904">
       <c r="A904" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="B904" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="905">
       <c r="A905" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
       <c r="B905" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="906">
       <c r="A906" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="B906" t="s">
-        <v>1536</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="907">
       <c r="A907" t="s">
-        <v>1537</v>
+        <v>1538</v>
       </c>
       <c r="B907" t="s">
-        <v>1538</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="908">
       <c r="A908" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="B908" t="s">
-        <v>1540</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="909">
       <c r="A909" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="B909" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="910">
       <c r="A910" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="B910" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="911">
       <c r="A911" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
       <c r="B911" t="s">
         <v>75</v>
@@ -12426,23 +12429,23 @@
     </row>
     <row r="912">
       <c r="A912" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="B912" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="913">
       <c r="A913" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="B913" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="914">
       <c r="A914" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="B914" t="s">
         <v>1</v>
@@ -12450,199 +12453,199 @@
     </row>
     <row r="915">
       <c r="A915" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="B915" t="s">
-        <v>1552</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="916">
       <c r="A916" t="s">
-        <v>1553</v>
+        <v>1554</v>
       </c>
       <c r="B916" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
     </row>
     <row r="917">
       <c r="A917" t="s">
-        <v>1555</v>
+        <v>1556</v>
       </c>
       <c r="B917" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="918">
       <c r="A918" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="B918" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="919">
       <c r="A919" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="B919" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="920">
       <c r="A920" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="B920" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="921">
       <c r="A921" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="B921" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="922">
       <c r="A922" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="B922" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="923">
       <c r="A923" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="B923" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="924">
       <c r="A924" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="B924" t="s">
-        <v>1570</v>
+        <v>1571</v>
       </c>
     </row>
     <row r="925">
       <c r="A925" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="B925" t="s">
-        <v>1572</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="926">
       <c r="A926" t="s">
-        <v>1573</v>
+        <v>1574</v>
       </c>
       <c r="B926" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="927">
       <c r="A927" t="s">
-        <v>1575</v>
+        <v>1576</v>
       </c>
       <c r="B927" t="s">
-        <v>1576</v>
+        <v>1577</v>
       </c>
     </row>
     <row r="928">
       <c r="A928" t="s">
-        <v>1577</v>
+        <v>1578</v>
       </c>
       <c r="B928" t="s">
-        <v>1578</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="929">
       <c r="A929" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="B929" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="930">
       <c r="A930" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="B930" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="931">
       <c r="A931" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="B931" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="932">
       <c r="A932" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="B932" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="933">
       <c r="A933" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="B933" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="934">
       <c r="A934" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
       <c r="B934" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
     </row>
     <row r="935">
       <c r="A935" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="B935" t="s">
-        <v>1592</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="936">
       <c r="A936" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="B936" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
     </row>
     <row r="937">
       <c r="A937" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
       <c r="B937" t="s">
-        <v>1596</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="938">
       <c r="A938" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="B938" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="939">
       <c r="A939" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="B939" t="s">
         <v>1</v>
@@ -12650,47 +12653,47 @@
     </row>
     <row r="940">
       <c r="A940" t="s">
-        <v>1600</v>
+        <v>1601</v>
       </c>
       <c r="B940" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="941">
       <c r="A941" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="B941" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
     </row>
     <row r="942">
       <c r="A942" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="B942" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="943">
       <c r="A943" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
       <c r="B943" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
     </row>
     <row r="944">
       <c r="A944" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="B944" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="945">
       <c r="A945" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="B945" t="s">
         <v>1</v>
@@ -12698,79 +12701,79 @@
     </row>
     <row r="946">
       <c r="A946" t="s">
-        <v>1611</v>
+        <v>1612</v>
       </c>
       <c r="B946" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="947">
       <c r="A947" t="s">
-        <v>1613</v>
+        <v>1614</v>
       </c>
       <c r="B947" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
     </row>
     <row r="948">
       <c r="A948" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="B948" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="949">
       <c r="A949" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="B949" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="950">
       <c r="A950" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
       <c r="B950" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
     </row>
     <row r="951">
       <c r="A951" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="B951" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="952">
       <c r="A952" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="B952" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="953">
       <c r="A953" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="B953" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
     </row>
     <row r="954">
       <c r="A954" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="B954" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="955">
       <c r="A955" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="B955" t="s">
         <v>1</v>
@@ -12778,31 +12781,31 @@
     </row>
     <row r="956">
       <c r="A956" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="B956" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
     </row>
     <row r="957">
       <c r="A957" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
       <c r="B957" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
     </row>
     <row r="958">
       <c r="A958" t="s">
-        <v>1634</v>
+        <v>1635</v>
       </c>
       <c r="B958" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="959">
       <c r="A959" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="B959" t="s">
         <v>1</v>
@@ -12810,7 +12813,7 @@
     </row>
     <row r="960">
       <c r="A960" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="B960" t="s">
         <v>1</v>
@@ -12818,7 +12821,7 @@
     </row>
     <row r="961">
       <c r="A961" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="B961" t="s">
         <v>75</v>
@@ -12826,7 +12829,7 @@
     </row>
     <row r="962">
       <c r="A962" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
       <c r="B962" t="s">
         <v>75</v>
@@ -12834,15 +12837,15 @@
     </row>
     <row r="963">
       <c r="A963" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="B963" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
     </row>
     <row r="964">
       <c r="A964" t="s">
-        <v>1642</v>
+        <v>1643</v>
       </c>
       <c r="B964" t="s">
         <v>1</v>
@@ -12850,15 +12853,15 @@
     </row>
     <row r="965">
       <c r="A965" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="B965" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
     </row>
     <row r="966">
       <c r="A966" t="s">
-        <v>1645</v>
+        <v>1646</v>
       </c>
       <c r="B966" t="s">
         <v>1</v>
@@ -12866,7 +12869,7 @@
     </row>
     <row r="967">
       <c r="A967" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
       <c r="B967" t="s">
         <v>1</v>
@@ -12874,7 +12877,7 @@
     </row>
     <row r="968">
       <c r="A968" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="B968" t="s">
         <v>1</v>
@@ -12882,31 +12885,31 @@
     </row>
     <row r="969">
       <c r="A969" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
       <c r="B969" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="970">
       <c r="A970" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="B970" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="971">
       <c r="A971" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="B971" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="972">
       <c r="A972" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="B972" t="s">
         <v>75</v>
@@ -12914,15 +12917,15 @@
     </row>
     <row r="973">
       <c r="A973" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="B973" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
     </row>
     <row r="974">
       <c r="A974" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="B974" t="s">
         <v>1</v>
@@ -12930,23 +12933,23 @@
     </row>
     <row r="975">
       <c r="A975" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="B975" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="976">
       <c r="A976" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="B976" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="977">
       <c r="A977" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="B977" t="s">
         <v>1</v>
@@ -12954,7 +12957,7 @@
     </row>
     <row r="978">
       <c r="A978" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="B978" t="s">
         <v>1</v>
@@ -12962,7 +12965,7 @@
     </row>
     <row r="979">
       <c r="A979" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="B979" t="s">
         <v>1386</v>
@@ -12970,23 +12973,23 @@
     </row>
     <row r="980">
       <c r="A980" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="B980" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="981">
       <c r="A981" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="B981" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="982">
       <c r="A982" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="B982" t="s">
         <v>1</v>
@@ -12994,79 +12997,79 @@
     </row>
     <row r="983">
       <c r="A983" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="B983" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="984">
       <c r="A984" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="B984" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="985">
       <c r="A985" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="B985" t="s">
-        <v>1675</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="986">
       <c r="A986" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="B986" t="s">
-        <v>1677</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="987">
       <c r="A987" t="s">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="B987" t="s">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="988">
       <c r="A988" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="B988" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="989">
       <c r="A989" t="s">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="B989" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="990">
       <c r="A990" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="B990" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="991">
       <c r="A991" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="B991" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="992">
       <c r="A992" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="B992" t="s">
         <v>1</v>
@@ -13074,15 +13077,15 @@
     </row>
     <row r="993">
       <c r="A993" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="B993" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="994">
       <c r="A994" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="B994" t="s">
         <v>1</v>
@@ -13090,7 +13093,7 @@
     </row>
     <row r="995">
       <c r="A995" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="B995" t="s">
         <v>1</v>
@@ -13098,10 +13101,10 @@
     </row>
     <row r="996">
       <c r="A996" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="B996" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática hashcode jue nov 18 15:12:29 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -29,13 +29,13 @@
     <t>01-010050TP</t>
   </si>
   <si>
-    <t>821d617ccb748bee004129e886366b23</t>
+    <t>af91f3692b5c2a074c3f4fbe008ebd6f</t>
   </si>
   <si>
     <t>01-010035A</t>
   </si>
   <si>
-    <t>41719c71caba7b1e33163ba72bfe84aa</t>
+    <t>4a97e7dfbcdd2b1a8476f0dd150a01ef</t>
   </si>
   <si>
     <t>03-030029A</t>
@@ -59,7 +59,7 @@
     <t>03-030005A</t>
   </si>
   <si>
-    <t>2af0cb07e0e1f294f110e85e40af40be</t>
+    <t>b9894e60fbfa01ea11b5198f1b3e6816</t>
   </si>
   <si>
     <t>05-050305TC</t>
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>2ae1f19395183ed5b2388788b0763313</t>
+    <t>59de551a125521c3444790c0661399ae</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -107,7 +107,7 @@
     <t>915-150012A</t>
   </si>
   <si>
-    <t>4b44cb446163485ebb0b311da4abdcc6</t>
+    <t>09d75f98149a07c4a0583ae9ca10de4d</t>
   </si>
   <si>
     <t>05-050305TP</t>
@@ -119,7 +119,7 @@
     <t>05-0709-070921BTP</t>
   </si>
   <si>
-    <t>05b9491f51ef494cb7e34dadbef1270e</t>
+    <t>4c6f84b27dcccd77f694c10531a70268</t>
   </si>
   <si>
     <t>01-010010A</t>
@@ -176,7 +176,7 @@
     <t>01-010050TC</t>
   </si>
   <si>
-    <t>0b806737ac696a894d996b6499d5d1a8</t>
+    <t>f701fc6735e33393ae9dfc09dc1f862b</t>
   </si>
   <si>
     <t>05-050302A</t>
@@ -191,19 +191,19 @@
     <t>05-0709-070921BTC</t>
   </si>
   <si>
-    <t>5852ad166ec6983e1f7c2f03b75d3bd2</t>
+    <t>5fd184f870d2af27239c7755601859fa</t>
   </si>
   <si>
     <t>03-030004A</t>
   </si>
   <si>
-    <t>4f28fb248e974767ac37a0dceefd7331</t>
+    <t>6d62a0557ea936e302361742a90bbf2d</t>
   </si>
   <si>
     <t>915-150011A</t>
   </si>
   <si>
-    <t>53fe8e276ff06c3fd44492c69d21f244</t>
+    <t>378ab1f948c4e84c7e2344d013d62a55</t>
   </si>
   <si>
     <t>05-050316TP</t>
@@ -215,7 +215,7 @@
     <t>915-150018TP</t>
   </si>
   <si>
-    <t>0993f7a58024c6a48ac3ce721114a5c8</t>
+    <t>62e8009b0bb43fe17664e9f2373a6c8c</t>
   </si>
   <si>
     <t>03-02010301-030102A</t>
@@ -224,7 +224,7 @@
     <t>915-150018TM</t>
   </si>
   <si>
-    <t>3f22b180f8c5118737028e2efba3aa45</t>
+    <t>39b20a4d3a33d1313cc52833ba6c0bca</t>
   </si>
   <si>
     <t>01-010057A</t>
@@ -251,7 +251,7 @@
     <t>05-0709-070908TC</t>
   </si>
   <si>
-    <t>5400dab8b05a98ab638b37351beb6afa</t>
+    <t>9908c29b7fab4cef9c80ff46dcf03af6</t>
   </si>
   <si>
     <t>05-050105A</t>
@@ -281,19 +281,19 @@
     <t>915-150018TC</t>
   </si>
   <si>
-    <t>a56d0a49802668923272ffd81f20ec30</t>
+    <t>6a8ff615cdb00a46b4e5c0f541ed124b</t>
   </si>
   <si>
     <t>915-150007TP</t>
   </si>
   <si>
-    <t>61fbcac4a0e40b79503dbfe09a088dbc</t>
+    <t>7d576524d3c4fc8fef7b58eb5f8f284d</t>
   </si>
   <si>
     <t>01-010063TP</t>
   </si>
   <si>
-    <t>e7f908c55a61b9f4c5f7a987985fd925</t>
+    <t>b3f7614824357fe5c8b54b6288c09e92</t>
   </si>
   <si>
     <t>01-010032A</t>
@@ -305,7 +305,7 @@
     <t>915-150007TM</t>
   </si>
   <si>
-    <t>6c894387e4343caaa722bdb22cc24fb6</t>
+    <t>b367758740bae7360eac1bc8e5e38bc2</t>
   </si>
   <si>
     <t>01-010063TM</t>
@@ -341,7 +341,7 @@
     <t>05-0709-070908TM</t>
   </si>
   <si>
-    <t>0f2b5a283bbd0fa2e6f4d204e75a45fb</t>
+    <t>67b7c9f494638cfa165a2cb3d182fc27</t>
   </si>
   <si>
     <t>03-030026A</t>
@@ -356,7 +356,7 @@
     <t>05-0709-070908TP</t>
   </si>
   <si>
-    <t>c66752fff0d24cd595df16cead8321f4</t>
+    <t>4e05305223e360a8e38718a184190ecd</t>
   </si>
   <si>
     <t>03-030002A</t>
@@ -371,7 +371,7 @@
     <t>915-150007TC</t>
   </si>
   <si>
-    <t>49747575b2941f2d7b203570ce685586</t>
+    <t>0159658a61ec1e54769b3e111cd5e338</t>
   </si>
   <si>
     <t>04-040012TP</t>
@@ -395,7 +395,7 @@
     <t>905-9050607-905060702TM</t>
   </si>
   <si>
-    <t>de587608272e7642fea45dc6a4eec7b4</t>
+    <t>b0bfef82cb938c7b37b82ac03dd92e02</t>
   </si>
   <si>
     <t>01-010055A</t>
@@ -422,7 +422,7 @@
     <t>905-9050607-905060702TP</t>
   </si>
   <si>
-    <t>3ff638c668f8683b3239757c18b1bd75</t>
+    <t>9d1d568df4a0a88312f112aaa595d6c1</t>
   </si>
   <si>
     <t>03-030025A</t>
@@ -434,7 +434,7 @@
     <t>03-030001A</t>
   </si>
   <si>
-    <t>508c4b7f803246bcf6e5c5169d743a75</t>
+    <t>e9080851709b95373d75ab3d52b1eed3</t>
   </si>
   <si>
     <t>05-050307TP</t>
@@ -449,7 +449,7 @@
     <t>905-9050607-905060702TC</t>
   </si>
   <si>
-    <t>3e37fab3289964e163748ae1ae0dc5eb</t>
+    <t>bc13665eac829680b6a0efac910209a9</t>
   </si>
   <si>
     <t>01-010030A</t>
@@ -536,7 +536,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>a6a4ad04bd595317b0079bb650a01d78</t>
+    <t>dd075c32b83f804ad858b81f767d7141</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -578,7 +578,7 @@
     <t>915-150009TM</t>
   </si>
   <si>
-    <t>1a44f6d0f05186195bc181a560434d4d</t>
+    <t>c90124b7b564c8fd04454539d0804182</t>
   </si>
   <si>
     <t>01-010065TM</t>
@@ -593,7 +593,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>0fec58aacd6a62d325a1710fbf7dc0cf</t>
+    <t>c4164dd3c88981d8c135bbe7faeaf0cf</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -605,7 +605,7 @@
     <t>915-150009TP</t>
   </si>
   <si>
-    <t>d2e7587229c3885463b891d3614cc054</t>
+    <t>8c9538fa6d11f86766a4e3d63d121b0e</t>
   </si>
   <si>
     <t>04-040021TC</t>
@@ -635,7 +635,7 @@
     <t>915-150009TC</t>
   </si>
   <si>
-    <t>99142123935409b93c41af5ec368f9b2</t>
+    <t>c44933a8687ca715bd1e53da6d63de28</t>
   </si>
   <si>
     <t>04-040010TP</t>
@@ -668,7 +668,7 @@
     <t>04-040014TC</t>
   </si>
   <si>
-    <t>87a5e69893d7f7e018944f9895caf1d9</t>
+    <t>a412ce738c555f504b3c2fc2563a4afe</t>
   </si>
   <si>
     <t>05-050301TC</t>
@@ -698,7 +698,7 @@
     <t>04-040003TP</t>
   </si>
   <si>
-    <t>65691ef982935fd3b44ba3dd108cd83f</t>
+    <t>9e948857ded2a8589cde9e2d0d74f7f7</t>
   </si>
   <si>
     <t>01-010019A</t>
@@ -713,7 +713,7 @@
     <t>04-040003TM</t>
   </si>
   <si>
-    <t>8faa25e5191430c9e9919d991f82646a</t>
+    <t>cd96b58e7ba840c9698dfaad67319aad</t>
   </si>
   <si>
     <t>01-110304-11030403A</t>
@@ -722,7 +722,7 @@
     <t>01-010043TM</t>
   </si>
   <si>
-    <t>7880cb33e90d0f0bb0dad5532b72c6d6</t>
+    <t>b0a11a3971ce3c114ec540c1c518bf4f</t>
   </si>
   <si>
     <t>05-050312TP</t>
@@ -737,7 +737,7 @@
     <t>04-040003TC</t>
   </si>
   <si>
-    <t>73ad8a2aeacf9e3eeff989980e0e8450</t>
+    <t>11cbe408a34939d2f06c53505a4dfbb8</t>
   </si>
   <si>
     <t>05-050312TC</t>
@@ -833,13 +833,13 @@
     <t>01-010043TC</t>
   </si>
   <si>
-    <t>4eabe142441c98a110c9ee12d712cfe6</t>
+    <t>e7b56bcf0d89e5e16dceb6f97a42f1f9</t>
   </si>
   <si>
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>b65a056e377dd16eedcda4f04a751251</t>
+    <t>501ff54fe1ec0eb156cb3055e62653e8</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -869,7 +869,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>26775f8fb4f7818f49d5dc49b38a3129</t>
+    <t>8f027885c173037131b7c503d2368195</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1010,7 +1010,7 @@
     <t>05-0709-070906AA</t>
   </si>
   <si>
-    <t>1d10f1f6af396db708ccf4ee098150ca</t>
+    <t>ec1698ab8e6353b5c9c7fcc6b4c8e660</t>
   </si>
   <si>
     <t>01-010067TC</t>
@@ -1064,13 +1064,13 @@
     <t>05-0709-070910TC</t>
   </si>
   <si>
-    <t>8ef4cd605a3cf46667f8182712494327</t>
+    <t>b7d2fb4e6114387d8b68a8ec6efef78b</t>
   </si>
   <si>
     <t>05-0709-070910TM</t>
   </si>
   <si>
-    <t>8d7e340b825b66d5861497c1e780ddc2</t>
+    <t>c7b13c896d79f110af279a23b4fc0266</t>
   </si>
   <si>
     <t>01-010045TP</t>
@@ -1103,7 +1103,7 @@
     <t>05-0709-070906BA</t>
   </si>
   <si>
-    <t>90d8ac6682832f94ac5098dfcf75478f</t>
+    <t>8eb157a8fa1bbe10c34f8a5bf203d4b3</t>
   </si>
   <si>
     <t>01-010056TC</t>
@@ -1166,7 +1166,7 @@
     <t>05-0709-070910TP</t>
   </si>
   <si>
-    <t>3e431fb07fb0f6c9694ec63ca9dc0768</t>
+    <t>bb9ffa8ad25621f081e6aa7a6eb95859</t>
   </si>
   <si>
     <t>01-010045TC</t>
@@ -1217,7 +1217,7 @@
     <t>03-030006A</t>
   </si>
   <si>
-    <t>2449228716b6538cd66d5bc8c14cf808</t>
+    <t>8db38e28a1f46406c8d92bc388bb0885</t>
   </si>
   <si>
     <t>05-050009TM</t>
@@ -1256,7 +1256,7 @@
     <t>04-040014TP</t>
   </si>
   <si>
-    <t>0defa52e30cb2325fa7a2ac126c3721d</t>
+    <t>a6aa62789d57a04a889943c1037ac8a7</t>
   </si>
   <si>
     <t>03-030042TC</t>
@@ -1271,7 +1271,7 @@
     <t>04-040014TM</t>
   </si>
   <si>
-    <t>fca3f688af13cc97c5e08c9d3cdb5ec4</t>
+    <t>492d3a39d5a70a93cd6c37e584ad93d6</t>
   </si>
   <si>
     <t>03-02010301-030089TM</t>
@@ -1301,7 +1301,7 @@
     <t>01-080101-010091TM</t>
   </si>
   <si>
-    <t>3485dcb96c4cad67ffca40b22f7a021a</t>
+    <t>19fc0070b6cb6aaf7ebcf6b8d1e992db</t>
   </si>
   <si>
     <t>01-010058TM</t>
@@ -1403,7 +1403,7 @@
     <t>01-080101-010091TC</t>
   </si>
   <si>
-    <t>6954b707057466638bc105dedcc0ae2b</t>
+    <t>4eb30eab2e23b782208c6a5b2be44559</t>
   </si>
   <si>
     <t>03-030041TP</t>
@@ -1475,7 +1475,7 @@
     <t>01-080101-010112TM</t>
   </si>
   <si>
-    <t>0e4158b3be5756e9866cace2776c8db4</t>
+    <t>8c6e2b75376b8490b816902250befb49</t>
   </si>
   <si>
     <t>01-010025TP</t>
@@ -1505,7 +1505,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>70a8a24919664930809e813e115083b9</t>
+    <t>eaa9458a605631a1d065a462c5e5c008</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -1547,7 +1547,7 @@
     <t>915-150011TP</t>
   </si>
   <si>
-    <t>e854ca8a23b47c0d6e9010f4816e8974</t>
+    <t>0c26fd91b9125946602969e60614ecb8</t>
   </si>
   <si>
     <t>01-010014TP</t>
@@ -1574,7 +1574,7 @@
     <t>905-9050607-905060701A</t>
   </si>
   <si>
-    <t>7e910355cac59aae9cdb5abe67f245c8</t>
+    <t>b2a61c1c546004cbbd4486f2e85dab05</t>
   </si>
   <si>
     <t>01-080101-010093TM</t>
@@ -1607,7 +1607,7 @@
     <t>915-150011TC</t>
   </si>
   <si>
-    <t>08fee30ea443d574b66bedbbb56d1561</t>
+    <t>856b6031b20a0979bfaf8d26d1b23bbe</t>
   </si>
   <si>
     <t>03-030008TP</t>
@@ -1622,7 +1622,7 @@
     <t>915-150011TM</t>
   </si>
   <si>
-    <t>6f20c78dbc6676815780eb9ecb83d509</t>
+    <t>903bb20630a8ace4e47ca2fd1a725f41</t>
   </si>
   <si>
     <t>03-030072TP</t>
@@ -1655,7 +1655,7 @@
     <t>01-010049TP</t>
   </si>
   <si>
-    <t>bfb7a011b20a35d6c9a0d8ffa3efe1ac</t>
+    <t>bd28a05aac77a0bd798d2871eedfbe58</t>
   </si>
   <si>
     <t>01-010003TP</t>
@@ -1676,7 +1676,7 @@
     <t>01-010049TM</t>
   </si>
   <si>
-    <t>e956c7a7df01a3d09562f57bb09129a4</t>
+    <t>8154777e2c8ce05773d7088ed02de109</t>
   </si>
   <si>
     <t>01-080101-010082TM</t>
@@ -1688,7 +1688,7 @@
     <t>04-040003A</t>
   </si>
   <si>
-    <t>7741b7ed09595472064d877c3a04e492</t>
+    <t>d743159f8dd21ff896b707521e0082c6</t>
   </si>
   <si>
     <t>03-02010301-030081A</t>
@@ -1715,7 +1715,7 @@
     <t>05-0709-070902TC</t>
   </si>
   <si>
-    <t>78141aa3ad407c25ee10a705a2793344</t>
+    <t>b40b1af66372a7b4200f93a3b9a705ab</t>
   </si>
   <si>
     <t>03-02010301-030097TC</t>
@@ -1730,7 +1730,7 @@
     <t>03-02010301-030097TM</t>
   </si>
   <si>
-    <t>2634a1798d1a3c6dfbcfd59bb211ad92</t>
+    <t>5311dc722c4fc5a1ee66cca5a4ad5f46</t>
   </si>
   <si>
     <t>03-030050TC</t>
@@ -1802,7 +1802,7 @@
     <t>905-9050607-905060702A</t>
   </si>
   <si>
-    <t>2b7ace009c184cf0272a47b51bbb0c02</t>
+    <t>e1021bea513ab0537bc4df13105d9737</t>
   </si>
   <si>
     <t>03-030061TC</t>
@@ -1814,7 +1814,7 @@
     <t>05-0709-070902TP</t>
   </si>
   <si>
-    <t>a321218770d54c1ead7b42d941944f6d</t>
+    <t>852dd907a8027478a4daf60cf9088c2c</t>
   </si>
   <si>
     <t>05-050201TP</t>
@@ -1826,13 +1826,13 @@
     <t>05-0709-070902TM</t>
   </si>
   <si>
-    <t>7ba26e807a4cb398bb150a7885740e96</t>
+    <t>2db18754cfde08b840d87e01bd99babb</t>
   </si>
   <si>
     <t>915-150009A</t>
   </si>
   <si>
-    <t>c385735a4c483d51f2ae13a1c253cf21</t>
+    <t>27162f060b503dd3b03739e69f99cdf5</t>
   </si>
   <si>
     <t>05-050201TM</t>
@@ -1868,19 +1868,19 @@
     <t>05-0709-070906ATC</t>
   </si>
   <si>
-    <t>d272e12677169965add2053d711e3d48</t>
+    <t>1d538b85277d28472a82b08c1972ef36</t>
   </si>
   <si>
     <t>915-150013TP</t>
   </si>
   <si>
-    <t>7b84711152414e4c246f740725ddb603</t>
+    <t>0bc8bdf73950f50bb65c5e87bf7c5d77</t>
   </si>
   <si>
     <t>03-030006TC</t>
   </si>
   <si>
-    <t>0f44e0ea975115699e243e0508f30d3a</t>
+    <t>67e89ce88d11a78c862620a61b3f2f70</t>
   </si>
   <si>
     <t>03-030006TM</t>
@@ -1892,7 +1892,7 @@
     <t>02-020001TC</t>
   </si>
   <si>
-    <t>9591a6121b5000e5a91a52ea1e8530c1</t>
+    <t>16e8cb4dbf50ec4e86c7fa64fe380541</t>
   </si>
   <si>
     <t>01-010016TP</t>
@@ -1922,7 +1922,7 @@
     <t>05-0709-070906ATM</t>
   </si>
   <si>
-    <t>3dd7fdf4f82e75464d8723fdbaa9d6a8</t>
+    <t>c28618037e25e3704c441d1b6fd012db</t>
   </si>
   <si>
     <t>03-030070TC</t>
@@ -1934,19 +1934,19 @@
     <t>05-0709-070906ATP</t>
   </si>
   <si>
-    <t>7342a9f55328567957fa51a1215fe113</t>
+    <t>d2366e3876160ff8d83a9104aaef04fe</t>
   </si>
   <si>
     <t>915-150013TC</t>
   </si>
   <si>
-    <t>306a82df144581f68cff1eb662f27375</t>
+    <t>06d4b0df2e3daa2e6f3952151324d3c2</t>
   </si>
   <si>
     <t>915-150013TM</t>
   </si>
   <si>
-    <t>291a632eed38372a2118a845060580f8</t>
+    <t>9e2b479681aec8331992d5e2e269b068</t>
   </si>
   <si>
     <t>03-030045A</t>
@@ -1958,7 +1958,7 @@
     <t>05-0709-070910A</t>
   </si>
   <si>
-    <t>4829f40c44dcec27a667170ba36b3818</t>
+    <t>ca3bc93378cdc336fb1d23bfd0287161</t>
   </si>
   <si>
     <t>01-010074A</t>
@@ -2012,13 +2012,13 @@
     <t>01-010050A</t>
   </si>
   <si>
-    <t>8911b65ff0adc6263b52dd7272d2332f</t>
+    <t>172db03539e2184365cf33be7505021b</t>
   </si>
   <si>
     <t>02-020001TM</t>
   </si>
   <si>
-    <t>10ef3d705ebb46abf3fa5a21b5e047d7</t>
+    <t>10cb88bbcdcba6564f4634c1c3e628ef</t>
   </si>
   <si>
     <t>01-080101-010084TP</t>
@@ -2042,7 +2042,7 @@
     <t>02-020001TP</t>
   </si>
   <si>
-    <t>b201805672b67168e40e217b6a6ebb82</t>
+    <t>1d2a0fad47aed368e039d0d34410fcec</t>
   </si>
   <si>
     <t>03-02010301-030091TC</t>
@@ -2108,13 +2108,13 @@
     <t>915-150015TP</t>
   </si>
   <si>
-    <t>ad1f80c8a38b25554200cea4225df193</t>
+    <t>ca9a0ce7200f67ff0f489c634cd576bf</t>
   </si>
   <si>
     <t>03-030004TC</t>
   </si>
   <si>
-    <t>0dd543a2b7142033c57bf093f5631b3a</t>
+    <t>ab039e8b28b07cb439eb3fe7f2a6baee</t>
   </si>
   <si>
     <t>01-010018TC</t>
@@ -2132,7 +2132,7 @@
     <t>915-150015TM</t>
   </si>
   <si>
-    <t>72124e51ca8fbad9a299073b8ccbe1a6</t>
+    <t>aec11b26aac47ff6bdcac8864b6f5cbf</t>
   </si>
   <si>
     <t>901-010202-9010102022TC</t>
@@ -2147,7 +2147,7 @@
     <t>03-030004TP</t>
   </si>
   <si>
-    <t>83f377bdb33260c4ca151c226f670d2e</t>
+    <t>84a1a9aff333a40f7b93ff13f396825b</t>
   </si>
   <si>
     <t>03-030004TM</t>
@@ -2156,7 +2156,7 @@
     <t>915-150015TC</t>
   </si>
   <si>
-    <t>1e80b3d0df570694e83ec8c84bcc78ca</t>
+    <t>363b8da5a43db16b69f56ba299c69d4a</t>
   </si>
   <si>
     <t>04-040009TC</t>
@@ -2207,7 +2207,7 @@
     <t>915-150004TP</t>
   </si>
   <si>
-    <t>ffed5a323c47487b53ac2cadb90868ab</t>
+    <t>19796459bde6467c01113b81816d466f</t>
   </si>
   <si>
     <t>01-010060TP</t>
@@ -2228,7 +2228,7 @@
     <t>915-150004TM</t>
   </si>
   <si>
-    <t>b046fedaf21e139c91af0947c19d4c24</t>
+    <t>2fe5f54c0a0d39a3106d13918c7f78a7</t>
   </si>
   <si>
     <t>01-010060TM</t>
@@ -2237,7 +2237,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>4d90c661e98736dfc9bc7228ed2a11e5</t>
+    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2264,7 +2264,7 @@
     <t>915-150004TC</t>
   </si>
   <si>
-    <t>0fa37d4e516c6457cb1d73aacb9154b7</t>
+    <t>c3d15ba386f49a4a89cff768392ffa95</t>
   </si>
   <si>
     <t>03-030040A</t>
@@ -2285,7 +2285,7 @@
     <t>05-0709-070905BTP</t>
   </si>
   <si>
-    <t>0ace74bd4d5e14e304eb72587aa1e207</t>
+    <t>c3a6bebf959923ce3ad21b967d0b2062</t>
   </si>
   <si>
     <t>01-010007TP</t>
@@ -2408,13 +2408,13 @@
     <t>915-150017TP</t>
   </si>
   <si>
-    <t>0bf208eae38e5873692b84a66f8fb2ca</t>
+    <t>2882a2cb40dba8d87f6ef93f3dc9b3b3</t>
   </si>
   <si>
     <t>915-150017TM</t>
   </si>
   <si>
-    <t>49281bf4f40ead942888b810674ffdb9</t>
+    <t>ec21d5055c8849c0238a64995935b9ac</t>
   </si>
   <si>
     <t>01-010023A</t>
@@ -2441,7 +2441,7 @@
     <t>05-0709-070909TC</t>
   </si>
   <si>
-    <t>b8d747b6a2f4360f473ec24392463b45</t>
+    <t>4e57d31c81b8f0b4e80c3d80a51d4c70</t>
   </si>
   <si>
     <t>05-050204A</t>
@@ -2453,7 +2453,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>ed22506af71d0901f2e012d947ce109b</t>
+    <t>5854519ef399046ca625a71dce515635</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2477,7 +2477,7 @@
     <t>915-150017TC</t>
   </si>
   <si>
-    <t>4370bf2a6c612a26ee49dfc30ab5e233</t>
+    <t>466d1df6ad4f7853fa33b6bca722803d</t>
   </si>
   <si>
     <t>01-010009TC</t>
@@ -2516,7 +2516,7 @@
     <t>03-030016A</t>
   </si>
   <si>
-    <t>a9763d2a082f1a96fc711b79aaf5c6e8</t>
+    <t>2e1cb344bc4c52acae679a96ac27c388</t>
   </si>
   <si>
     <t>03-030036TP</t>
@@ -2552,7 +2552,7 @@
     <t>04-040011TM</t>
   </si>
   <si>
-    <t>c9509a175aee0e574dc1a10d5352122b</t>
+    <t>9c97e798b02676a3ca40e0f0ef22b628</t>
   </si>
   <si>
     <t>05-050314A</t>
@@ -2567,7 +2567,7 @@
     <t>05-0709-070909TM</t>
   </si>
   <si>
-    <t>9f49a98543ca027eb508621e1fb91e3b</t>
+    <t>3dcb045817c3098469dbe3b3069eb83d</t>
   </si>
   <si>
     <t>01-010009TP</t>
@@ -2579,7 +2579,7 @@
     <t>03-030001TC</t>
   </si>
   <si>
-    <t>b160c7ec0a78a8efefbead291473c70e</t>
+    <t>ac5faa7b24db5e3a4281517c9b86466e</t>
   </si>
   <si>
     <t>03-030047TC</t>
@@ -2591,7 +2591,7 @@
     <t>05-0709-070909TP</t>
   </si>
   <si>
-    <t>f32062aa5e28d6309651fc09b2df374b</t>
+    <t>1651e0a559aaee0fdaf68eecd726d95c</t>
   </si>
   <si>
     <t>04-040011TP</t>
@@ -2609,7 +2609,7 @@
     <t>905-9050607-905060701TM</t>
   </si>
   <si>
-    <t>1c8a64a363632393752b560f5a6a2f10</t>
+    <t>e0e5a8781dbac31946c52f46dcd95db7</t>
   </si>
   <si>
     <t>01-010051TP</t>
@@ -2621,7 +2621,7 @@
     <t>905-9050607-905060701TP</t>
   </si>
   <si>
-    <t>6c00b36e0eaa8e4dcd941f8ed587f786</t>
+    <t>1f4766a2be0c799e3c5310f4e0f5c983</t>
   </si>
   <si>
     <t>01-010045A</t>
@@ -2726,7 +2726,7 @@
     <t>905-9050607-905060701TC</t>
   </si>
   <si>
-    <t>b6968f3f8506bbe85976337f02c79a14</t>
+    <t>caf0902acd5e4ab007abd4dbb31c1a66</t>
   </si>
   <si>
     <t>01-010062TC</t>
@@ -2747,7 +2747,7 @@
     <t>01-010068A</t>
   </si>
   <si>
-    <t>381d76a139cbb5b90408aa873647f71b</t>
+    <t>121b6022ca6b23d18bfb7fb505803db0</t>
   </si>
   <si>
     <t>03-030014TP</t>
@@ -2810,7 +2810,7 @@
     <t>05-0709-070903A</t>
   </si>
   <si>
-    <t>4aaa92afb0abaea7fcdadb713098ba12</t>
+    <t>935ef81b9fb805a4be34a828255ed1c9</t>
   </si>
   <si>
     <t>05-050317TP</t>
@@ -2864,7 +2864,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>2f155268974893256ff764d9a39e9335</t>
+    <t>524aacb4580b4166773e582cb0808dbc</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2882,7 +2882,7 @@
     <t>05-0709-070902A</t>
   </si>
   <si>
-    <t>ee108dfa4ade719dfc394066af30f874</t>
+    <t>b28a09c762509387e269714acae243b2</t>
   </si>
   <si>
     <t>03-030013A</t>
@@ -2894,7 +2894,7 @@
     <t>01-010064TP</t>
   </si>
   <si>
-    <t>61af9898f6bd8e9b0b8cc5ef77622c3a</t>
+    <t>d152e0b7e58e4c0a3b12fbe91d962f80</t>
   </si>
   <si>
     <t>03-90205-0205_007A</t>
@@ -2909,7 +2909,7 @@
     <t>915-150008TM</t>
   </si>
   <si>
-    <t>f85e80bd8c13c6c66f07235d826f385f</t>
+    <t>32137b737f73b05333e215fb77c16587</t>
   </si>
   <si>
     <t>01-010064TM</t>
@@ -2957,7 +2957,7 @@
     <t>915-150008TP</t>
   </si>
   <si>
-    <t>ac8cf6c32ece5e43ac3f79ebad48ed51</t>
+    <t>4c36003fcffd031a25a22fbbe3a1ca63</t>
   </si>
   <si>
     <t>01-010075TC</t>
@@ -2969,7 +2969,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>579451a92beef97da558af495ebe8606</t>
+    <t>9908ed097b4574baad512db74f20ff68</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -2981,7 +2981,7 @@
     <t>05-0709-070901A</t>
   </si>
   <si>
-    <t>b46da07bb323bdbffc5d0cfa704f77e6</t>
+    <t>e6ece49d19fe9fdfa605f0790e42ec84</t>
   </si>
   <si>
     <t>03-030012A</t>
@@ -2999,7 +2999,7 @@
     <t>915-150008TC</t>
   </si>
   <si>
-    <t>9518f3d56e3f5e0f6059671e877e498d</t>
+    <t>6e672982fa194296a2efa95bac027c65</t>
   </si>
   <si>
     <t>03-02010301-030100TC</t>
@@ -3020,7 +3020,7 @@
     <t>03-030001TM</t>
   </si>
   <si>
-    <t>ead04ed2740ceb084a3f0ce234470464</t>
+    <t>2f7eb22ff6ad0ca3d69e86974d03036b</t>
   </si>
   <si>
     <t>05-050308TC</t>
@@ -3032,7 +3032,7 @@
     <t>02-020002TC</t>
   </si>
   <si>
-    <t>417016e5a0ec9e73fd288ff16d22d782</t>
+    <t>a3ee29141986a4326417d8abaf0d6c3b</t>
   </si>
   <si>
     <t>03-030047TP</t>
@@ -3050,7 +3050,7 @@
     <t>03-030001TP</t>
   </si>
   <si>
-    <t>c30b13a5f0820e4e3c43214a99090270</t>
+    <t>ce67bdb572db24e4f6a2a30199fbe017</t>
   </si>
   <si>
     <t>03-030047TM</t>
@@ -3104,7 +3104,7 @@
     <t>01-010042TM</t>
   </si>
   <si>
-    <t>842636dc1e868b133495f4c2822e30a8</t>
+    <t>ed9f4b5680ebb02261d1eb6cc016f9a4</t>
   </si>
   <si>
     <t>03-030012TM</t>
@@ -3158,7 +3158,7 @@
     <t>01-080101-010089TM</t>
   </si>
   <si>
-    <t>f6bfb4fdedde97622b8a9058dcdeb57a</t>
+    <t>c557d1831e9be763f4fc83df83adf496</t>
   </si>
   <si>
     <t>03-030058A</t>
@@ -3176,7 +3176,7 @@
     <t>02-020002TM</t>
   </si>
   <si>
-    <t>93d7e9998659a16749e560d868f6e77a</t>
+    <t>918d0f6d00993ac69e708551f5e7e685</t>
   </si>
   <si>
     <t>01-010053TC</t>
@@ -3188,7 +3188,7 @@
     <t>02-020002TP</t>
   </si>
   <si>
-    <t>a306edc42f7ab2f4a339be49a216ffcb</t>
+    <t>64b83428c51981a8982ff0dc2928eeb6</t>
   </si>
   <si>
     <t>01-010031TP</t>
@@ -3227,7 +3227,7 @@
     <t>915-150008A</t>
   </si>
   <si>
-    <t>df19891eae88e9c353acb3c0f9238ac6</t>
+    <t>372abfffb38b2dc96240a099ef34c8d4</t>
   </si>
   <si>
     <t>05-0709-070955TP</t>
@@ -3251,7 +3251,7 @@
     <t>01-010042TC</t>
   </si>
   <si>
-    <t>d678389545d7e835d100ebc2f8ed9cca</t>
+    <t>922fbfeb06bc04374c9b8582e84c655d</t>
   </si>
   <si>
     <t>03-030032TC</t>
@@ -3317,7 +3317,7 @@
     <t>915-150007A</t>
   </si>
   <si>
-    <t>cafd5b65cc2ec420f27ccaa633e56e54</t>
+    <t>8bf4d4b70def7c3e1618c64e37847534</t>
   </si>
   <si>
     <t>05-050204TM</t>
@@ -3476,7 +3476,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>3509aa1997c3bcfb51b1a748dbd724ac</t>
+    <t>5b29ef0d3bf73f26c0132e79d57393cb</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3503,7 +3503,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>e7360a55096f740ab6e9aa80791956d2</t>
+    <t>0dc6f178beadd0b262ab340291e84963</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -3581,7 +3581,7 @@
     <t>01-010022TM</t>
   </si>
   <si>
-    <t>d906ce77b292c21e5f235b858758d7a8</t>
+    <t>656a006cbcf7ec2b05e7d214903ff9f2</t>
   </si>
   <si>
     <t>03-030030TP</t>
@@ -3593,7 +3593,7 @@
     <t>01-010002A</t>
   </si>
   <si>
-    <t>169b297b7fff24b881c52844b61284f0</t>
+    <t>35629bd494fb012622aba1a361a71f50</t>
   </si>
   <si>
     <t>01-010026A</t>
@@ -3614,7 +3614,7 @@
     <t>01-010068TP</t>
   </si>
   <si>
-    <t>6d5a025eee1b238ca18d69b146d7ed69</t>
+    <t>79222eb8a64864ef0957ba4fb2640dfd</t>
   </si>
   <si>
     <t>05-050206TP</t>
@@ -3626,7 +3626,7 @@
     <t>01-010068TM</t>
   </si>
   <si>
-    <t>efb93854e64d76a0082712ec93245e76</t>
+    <t>e1fa09aa78f53496969d261f9f5e7b69</t>
   </si>
   <si>
     <t>03-030076TP</t>
@@ -3635,7 +3635,7 @@
     <t>05-0709-070909A</t>
   </si>
   <si>
-    <t>dfc6091f934fc5044cfda2da5a67bfe3</t>
+    <t>31cfbe580fe6dfa303d681e53f909b80</t>
   </si>
   <si>
     <t>05-050206TM</t>
@@ -3650,7 +3650,7 @@
     <t>04-040013TM</t>
   </si>
   <si>
-    <t>2fe9e38eb071602504cde8eff31fe52e</t>
+    <t>d90a7dff71d15179e07e07d8d49cfe8e</t>
   </si>
   <si>
     <t>03-030041TC</t>
@@ -3662,7 +3662,7 @@
     <t>04-040013TP</t>
   </si>
   <si>
-    <t>2677e6917f5f9c5aa9daaa462655b2df</t>
+    <t>901335dcb975050b3a06ba2bb478fb2d</t>
   </si>
   <si>
     <t>01-010011TM</t>
@@ -3713,7 +3713,7 @@
     <t>04-040013TC</t>
   </si>
   <si>
-    <t>3591178de414aee03e8df5bbfe0638dd</t>
+    <t>5d36b099269766af24b39475fff3e8e3</t>
   </si>
   <si>
     <t>01-010011TP</t>
@@ -3758,25 +3758,25 @@
     <t>05-0709-070908A</t>
   </si>
   <si>
-    <t>a570bf9870c8beb68d7d03210d5b6f2c</t>
+    <t>7392593711ab7bb3250d7e56e6dece16</t>
   </si>
   <si>
     <t>01-010022TC</t>
   </si>
   <si>
-    <t>18fa7188d999ad4ba17761497e898d64</t>
+    <t>e9d235c08e4c1c94c33f933f84de5cef</t>
   </si>
   <si>
     <t>01-010049A</t>
   </si>
   <si>
-    <t>1b165eb937c09f4de7e61b497d3863c7</t>
+    <t>cc393fd4da76289572f103c2edfb820d</t>
   </si>
   <si>
     <t>05-0709-070905AA</t>
   </si>
   <si>
-    <t>6b00962aa51e03e90db15ec9f0d86e8f</t>
+    <t>b63bbf7509084a2b7b03ebc9663565f9</t>
   </si>
   <si>
     <t>01-080101-010110TP</t>
@@ -3791,7 +3791,7 @@
     <t>915-150002A</t>
   </si>
   <si>
-    <t>ae9e80c0c022799a39445a2399c8fe6e</t>
+    <t>74bc5bcce3784988c2080f7367ac96d1</t>
   </si>
   <si>
     <t>03-030054TC</t>
@@ -3827,7 +3827,7 @@
     <t>05-0709-070921ATP</t>
   </si>
   <si>
-    <t>74476aad8ebce81639d2b214aaafd947</t>
+    <t>ea3f030a8a490b970f7da01d292fecd4</t>
   </si>
   <si>
     <t>01-010024A</t>
@@ -3884,13 +3884,13 @@
     <t>02-020006TC</t>
   </si>
   <si>
-    <t>863e39fef68f7fa45e955c21edad39b0</t>
+    <t>2802ab1063279d54146223f696f20eb3</t>
   </si>
   <si>
     <t>05-0709-070921ATC</t>
   </si>
   <si>
-    <t>deab5c160b3856a617105a2bec99a5e9</t>
+    <t>f0e5c24140c9cb41727b2a54e3a260c8</t>
   </si>
   <si>
     <t>05-050207A</t>
@@ -3902,7 +3902,7 @@
     <t>02-020006TM</t>
   </si>
   <si>
-    <t>6a9b8ebe912b307b25cda9cc6184e098</t>
+    <t>fb6579275369feca2249f6a62946d497</t>
   </si>
   <si>
     <t>902-0204-02040101BTM</t>
@@ -3923,19 +3923,19 @@
     <t>05-0709-070905BA</t>
   </si>
   <si>
-    <t>265b93a97a6e7762073090ed8bd68ce6</t>
+    <t>6fcb607af1cb60af2252a39f7d1745de</t>
   </si>
   <si>
     <t>02-020006TP</t>
   </si>
   <si>
-    <t>0cbd0f8fba9b7654d2c9e52df7e20192</t>
+    <t>45cce2fdc22e2cfd7fa5302a2e549dab</t>
   </si>
   <si>
     <t>915-150001A</t>
   </si>
   <si>
-    <t>81d184e5ea89069a9746708c27ba9b3a</t>
+    <t>bbb159c371c7188bcb1da38b8b6d591f</t>
   </si>
   <si>
     <t>03-030065TC</t>
@@ -3965,7 +3965,7 @@
     <t>05-0709-070901TC</t>
   </si>
   <si>
-    <t>01b6ff12abce8f078560254cddfc1627</t>
+    <t>ed8d0f2e534d224e43bcd71563f0f88b</t>
   </si>
   <si>
     <t>03-02010301-030096TC</t>
@@ -3974,19 +3974,19 @@
     <t>05-0709-070901TM</t>
   </si>
   <si>
-    <t>fee68621940ff3e17fd834505ea2331f</t>
+    <t>a7c1dadd7ec65360b7f5725a4cbe5b52</t>
   </si>
   <si>
     <t>01-010035TP</t>
   </si>
   <si>
-    <t>6490fabded0eb05a792536ed212a3e3e</t>
+    <t>edf354052625762b4b29e5510944d1cf</t>
   </si>
   <si>
     <t>01-010035TM</t>
   </si>
   <si>
-    <t>9d4902c0a081edff9aa839214ab773dc</t>
+    <t>e5555af19ade7cb69b3de639b53efbe2</t>
   </si>
   <si>
     <t>03-030073A</t>
@@ -4055,13 +4055,13 @@
     <t>05-0709-070901TP</t>
   </si>
   <si>
-    <t>397ba27f653d891ebe59029a6f0dab43</t>
+    <t>ba34bad9b6e7c800a1ade4e878ae97ca</t>
   </si>
   <si>
     <t>01-010035TC</t>
   </si>
   <si>
-    <t>50f3d5dd6de63f6f2ef93eb78f2564ba</t>
+    <t>535b9101700329efe947e9ed77b67f67</t>
   </si>
   <si>
     <t>03-02010301-030097A</t>
@@ -4076,7 +4076,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>4c26779b04aeb6357d6d674c0a29a362</t>
+    <t>84cab191ff25374b88bc173f93d60944</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4163,7 +4163,7 @@
     <t>03-030075TC</t>
   </si>
   <si>
-    <t>108dc20ead86ac9393e968a56ddbf757</t>
+    <t>1dd2ae8d880542e886ef8a0209785ad8</t>
   </si>
   <si>
     <t>05-050002TC</t>
@@ -4175,13 +4175,13 @@
     <t>03-030075TP</t>
   </si>
   <si>
-    <t>6eeff8e5ccfdab36c3b0a066b9bdbb66</t>
+    <t>4275c97ed1a790378ff8d6467314d457</t>
   </si>
   <si>
     <t>03-030075TM</t>
   </si>
   <si>
-    <t>c8670ec4e105f8c3246ecc1e391e16c4</t>
+    <t>8faee9629b60f43f0634f2f8efb568d4</t>
   </si>
   <si>
     <t>01-010048TC</t>
@@ -4202,13 +4202,13 @@
     <t>01-010002TM</t>
   </si>
   <si>
-    <t>002835f1d5546c3b330e10097ccbdc55</t>
+    <t>b1b88d90fa7d6865d68888cf1e30c1b8</t>
   </si>
   <si>
     <t>01-010002TP</t>
   </si>
   <si>
-    <t>0cca9b1731114d9a37c688f6079a9756</t>
+    <t>1b26a4858ebe756a23b4d8e5281c487e</t>
   </si>
   <si>
     <t>03-030070A</t>
@@ -4241,7 +4241,7 @@
     <t>05-0709-070903TC</t>
   </si>
   <si>
-    <t>655ea82c1cd5f1a39de0c488797ceb33</t>
+    <t>dfb41bc87eb854e2b99e152486144459</t>
   </si>
   <si>
     <t>01-010037TC</t>
@@ -4280,7 +4280,7 @@
     <t>01-010002TC</t>
   </si>
   <si>
-    <t>a7baf553fd3303b88d87616b23993853</t>
+    <t>2367230e0e9179c07dffed373205d81b</t>
   </si>
   <si>
     <t>03-02010301-030094A</t>
@@ -4292,7 +4292,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>235ab4bbe3eaa87649557f3c8ee3781b</t>
+    <t>ee1c195c1c2e0f45c3609111d1ac2f34</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4307,7 +4307,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>54dff1e3570afa76227c826ad2050f2d</t>
+    <t>1e2f02d90578b126e9ea63ac2cfcf96b</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4337,7 +4337,7 @@
     <t>05-0709-070903TM</t>
   </si>
   <si>
-    <t>60bc3633d16921f4896c881995a4e52e</t>
+    <t>b4e3ba5466c57f698549f42028666b21</t>
   </si>
   <si>
     <t>03-02010301-030093A</t>
@@ -4355,7 +4355,7 @@
     <t>05-0709-070903TP</t>
   </si>
   <si>
-    <t>e9530b989030d7acff041a50998e3855</t>
+    <t>d8ef158d83f87a66c3dcaa3efb83d98e</t>
   </si>
   <si>
     <t>04-040017TM</t>
@@ -4403,7 +4403,7 @@
     <t>04-040014A</t>
   </si>
   <si>
-    <t>1b6ed3b3a92747c4d0e386b2f9f87036</t>
+    <t>3bbeda48cc454f005a899945f7dbc5cd</t>
   </si>
   <si>
     <t>03-02010301-030092A</t>
@@ -4448,7 +4448,7 @@
     <t>915-150001TP</t>
   </si>
   <si>
-    <t>0c127b5f0172ed781a509349e6c28409</t>
+    <t>fb8bdd52c88c645604e93c2f67b8f429</t>
   </si>
   <si>
     <t>01-010004TP</t>
@@ -4478,7 +4478,7 @@
     <t>04-040013A</t>
   </si>
   <si>
-    <t>e441fe22d2b6b1f8e98bd23734f91e23</t>
+    <t>97220f71e67f3b425088a394f3a84b22</t>
   </si>
   <si>
     <t>03-02010301-030085TM</t>
@@ -4487,7 +4487,7 @@
     <t>915-150001TC</t>
   </si>
   <si>
-    <t>0ee05b216d187cd84b1366bfd9caf193</t>
+    <t>3c8fe25a6d9290e0a1321791ef223075</t>
   </si>
   <si>
     <t>03-02010301-030091A</t>
@@ -4496,7 +4496,7 @@
     <t>915-150001TM</t>
   </si>
   <si>
-    <t>d3e31586fc0f238413a108d7c84e733b</t>
+    <t>767187267aeb43374fa487d09b04d827</t>
   </si>
   <si>
     <t>03-02010301-030092TC</t>
@@ -4514,7 +4514,7 @@
     <t>01-010039TC</t>
   </si>
   <si>
-    <t>1f91ba663c5d24d29a8a88b3b45b8af5</t>
+    <t>7a5683a1bed4ff3e2674c0c7d869e083</t>
   </si>
   <si>
     <t>03-030029TC</t>
@@ -4535,7 +4535,7 @@
     <t>01-010039TM</t>
   </si>
   <si>
-    <t>7cfd5035d1ebc32c5b2e72d83c64bb55</t>
+    <t>ef898df150aa366cade8df3324848dbf</t>
   </si>
   <si>
     <t>01-080101-010084A</t>
@@ -4568,7 +4568,7 @@
     <t>03-030033A</t>
   </si>
   <si>
-    <t>17762dfdee88730f2873000080b186a2</t>
+    <t>5651ddd7888be309a021eb04eadb21e4</t>
   </si>
   <si>
     <t>03-02010301-030102TC</t>
@@ -4622,13 +4622,13 @@
     <t>915-150014TP</t>
   </si>
   <si>
-    <t>e095021e161529e65617f068d8eacd08</t>
+    <t>ebdec01a6b309e3748d9754a298a2ebb</t>
   </si>
   <si>
     <t>05-0709-070906BTC</t>
   </si>
   <si>
-    <t>948d665e3651e517e7ba26c501a65a10</t>
+    <t>ff0372bf9239fb61a080e87ed3195bd4</t>
   </si>
   <si>
     <t>01-010017TC</t>
@@ -4652,7 +4652,7 @@
     <t>915-150014TM</t>
   </si>
   <si>
-    <t>1ca3c1484e483fc4f4a9f3f57da3afba</t>
+    <t>57e6a5c84dd98419a196f687ba7da1cf</t>
   </si>
   <si>
     <t>901-010202-9010102023TC</t>
@@ -4688,7 +4688,7 @@
     <t>05-0709-070906BTM</t>
   </si>
   <si>
-    <t>dbee2729cb23d5bd7600ef69e57d464b</t>
+    <t>dab242bab5bc7656d6a1f3e354d7d51e</t>
   </si>
   <si>
     <t>03-030071TC</t>
@@ -4700,7 +4700,7 @@
     <t>915-150014TC</t>
   </si>
   <si>
-    <t>aca0e08bd02ff79f804a3d1d3f23c4ec</t>
+    <t>ec565bb99879f865a731ab258df28300</t>
   </si>
   <si>
     <t>01-010115TC</t>
@@ -4712,7 +4712,7 @@
     <t>05-0709-070906BTP</t>
   </si>
   <si>
-    <t>3ed0674e3f47802436055ef0aee8cd25</t>
+    <t>602b4fb729c08f06791474bf1a154eb1</t>
   </si>
   <si>
     <t>03-030007TP</t>
@@ -4748,7 +4748,7 @@
     <t>915-150003TP</t>
   </si>
   <si>
-    <t>fce84300477d16728114d72d4f7f8c5f</t>
+    <t>6c8a48c4793f647ae22e6415d1918f72</t>
   </si>
   <si>
     <t>01-080101-010083TC</t>
@@ -4760,7 +4760,7 @@
     <t>05-0709-070905ATC</t>
   </si>
   <si>
-    <t>059a421cbf7df830f6ac6bf08b052994</t>
+    <t>b2f44d3255fdd42d13a8b4353660a499</t>
   </si>
   <si>
     <t>01-010006TC</t>
@@ -4778,7 +4778,7 @@
     <t>915-150003TM</t>
   </si>
   <si>
-    <t>b7a6d29a9cba82cd87d582fa13a4bd8b</t>
+    <t>b98caff4d64e24b295aa661bef3da148</t>
   </si>
   <si>
     <t>01-080101-010083TM</t>
@@ -4829,13 +4829,13 @@
     <t>915-150003TC</t>
   </si>
   <si>
-    <t>35058e423177b5c2a1d9a3311e909735</t>
+    <t>cba30d7950a13a0c0967661dd8f1ded3</t>
   </si>
   <si>
     <t>05-0709-070905ATP</t>
   </si>
   <si>
-    <t>9d0ae80615e37b264f45d02edcddf360</t>
+    <t>b213c4e2488ad106b7235cb5839dce7a</t>
   </si>
   <si>
     <t>03-030018TP</t>
@@ -4886,7 +4886,7 @@
     <t>05-0709-070921AA</t>
   </si>
   <si>
-    <t>48ceb0bb5e2337ee5eb66697c3577418</t>
+    <t>95060d6e31bc91f2529e80a514b7f8a5</t>
   </si>
   <si>
     <t>03-02010301-030094TP</t>
@@ -4904,7 +4904,7 @@
     <t>03-02010301-030094TM</t>
   </si>
   <si>
-    <t>e803f7f4aa3331ae0d7c50f00e3f9fd8</t>
+    <t>5d277c98d807f951754f80bb69f75730</t>
   </si>
   <si>
     <t>03-030077A</t>
@@ -4913,7 +4913,7 @@
     <t>02-020006A</t>
   </si>
   <si>
-    <t>2369ec9edb1081bafb40644aa89da109</t>
+    <t>0739e4252751d56b83824b70b671b54d</t>
   </si>
   <si>
     <t>03-030053A</t>
@@ -4943,7 +4943,7 @@
     <t>05-0709-070921BA</t>
   </si>
   <si>
-    <t>388219a416373a3bd84b66165eec03cb</t>
+    <t>74ae33be2fdccb45346e846d82e80256</t>
   </si>
   <si>
     <t>03-030076A</t>
@@ -4967,7 +4967,7 @@
     <t>915-150016TP</t>
   </si>
   <si>
-    <t>ce1b21339d84c5b978949d033b30414d</t>
+    <t>252258ccc0477f771cfa7f7fff6e2847</t>
   </si>
   <si>
     <t>03-030005TC</t>
@@ -4979,7 +4979,7 @@
     <t>915-150016TM</t>
   </si>
   <si>
-    <t>22e4bccc3e21839772d7f2ed46a745fe</t>
+    <t>cddf31685c87ea1f10494c5af2604c98</t>
   </si>
   <si>
     <t>901-010202-9010102021TC</t>
@@ -5018,7 +5018,7 @@
     <t>915-150016TC</t>
   </si>
   <si>
-    <t>2a91eeed6df5af4e3324f09910f32329</t>
+    <t>164564ca6182282ff0c3c6b63f6c25c6</t>
   </si>
   <si>
     <t>01-080101-010085TC</t>
@@ -5045,7 +5045,7 @@
     <t>03-030016TC</t>
   </si>
   <si>
-    <t>135b2f3d16f10aadcd7a1e64c383a5b4</t>
+    <t>f74152985e919acc18d24beda95e9ea2</t>
   </si>
   <si>
     <t>915-150005TM</t>
@@ -5069,7 +5069,7 @@
     <t>03-030016TP</t>
   </si>
   <si>
-    <t>e23f0036d392bc5288233b226bb4056b</t>
+    <t>2775c1aca94ef3be5e1cb93e632b9c32</t>
   </si>
   <si>
     <t>03-030050A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie nov 19 01:56:30 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -311,7 +311,7 @@
     <t>01-010063TM</t>
   </si>
   <si>
-    <t>1a6e4967b8ad4e3060d15835ec792907</t>
+    <t>ad89823b30623527e3baef2253bbb1b1</t>
   </si>
   <si>
     <t>01-010056A</t>
@@ -443,7 +443,7 @@
     <t>01-010063TC</t>
   </si>
   <si>
-    <t>8ddcd036d580247e0b740246cf2a0105</t>
+    <t>c4ba01d46b527d0a4e04edce448dd616</t>
   </si>
   <si>
     <t>905-9050607-905060702TC</t>
@@ -1775,7 +1775,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>c90fc8532d13b2b346d3f832d1eadf70</t>
+    <t>07e7ff1786a3adbf9c279a7e4fbc6815</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -2237,7 +2237,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2915,7 +2915,7 @@
     <t>01-010064TM</t>
   </si>
   <si>
-    <t>3b38a9b4f52efd161cab11b028c91cdb</t>
+    <t>282e369444428aa780db634d3867d417</t>
   </si>
   <si>
     <t>01-080101-010087A</t>
@@ -3092,13 +3092,13 @@
     <t>01-010064TC</t>
   </si>
   <si>
-    <t>34d02d95e73aec059411612203a54ca3</t>
+    <t>b7ae7df38ad9ddc0f435e255584d2b1b</t>
   </si>
   <si>
     <t>01-010064A</t>
   </si>
   <si>
-    <t>b50b38e198c71bcf98c0c43aaa9ed33b</t>
+    <t>819a318a42b307090b15e32fe333138c</t>
   </si>
   <si>
     <t>01-010042TM</t>
@@ -4505,7 +4505,7 @@
     <t>01-010063A</t>
   </si>
   <si>
-    <t>ada3adcd7fdb09e539595719cabad321</t>
+    <t>43057fba58fa2f6a9cc65bd8ce502873</t>
   </si>
   <si>
     <t>902-0204-02040101AA</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb nov 20 05:53:44 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -65,7 +65,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>13630f8ea748eb39213fb6ef801fd380</t>
+    <t>c53aca77dd2eb05472af945ce1fab4a0</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -101,7 +101,7 @@
     <t>05-050207TP</t>
   </si>
   <si>
-    <t>6823801810e55ff4c050f38a91e4ee75</t>
+    <t>be277a350cb68cb239874586d866832c</t>
   </si>
   <si>
     <t>915-150012A</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>055fecd33eb5761f774217967e6b2550</t>
+    <t>3016d42d9958a4430e511833cbad6fdb</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -209,7 +209,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>e5cfcd4b711511c2aa6cacf2c915a266</t>
+    <t>cfaa5bf0423f64320f9a9d42bd4cf449</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -659,7 +659,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>d7dc2244dcc7fecc58c0c3f61dbc3c9c</t>
+    <t>8d829c4616cf4b96cdcf731bac392921</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -674,7 +674,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>ffc1acb4f56a9e3a2b0a163ba14a7197</t>
+    <t>cd850b29b88b6ee555efda7d2e1ed0d8</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -692,7 +692,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>736157ad34d20b9c81f8fff54f9a9631</t>
+    <t>e9e3a3273eaea7f1621c414b75cd8e62</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -728,7 +728,7 @@
     <t>05-050312TP</t>
   </si>
   <si>
-    <t>506c015a866fcfd78105d0dad33e5604</t>
+    <t>0b699f43ea4ee38a8ef5af2190d978db</t>
   </si>
   <si>
     <t>05-0709-070954TC</t>
@@ -743,7 +743,7 @@
     <t>05-050312TC</t>
   </si>
   <si>
-    <t>5d72b43503f22b39630f179807bb9baa</t>
+    <t>7cda573046364bdfef778b607b1de319</t>
   </si>
   <si>
     <t>03-030055TP</t>
@@ -863,7 +863,7 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>a8fdbc611b2e9f7c4c152c9ba817869a</t>
+    <t>ec793cf2baa9c1e8e7a640296dc50ce5</t>
   </si>
   <si>
     <t>05-050007TP</t>
@@ -878,7 +878,7 @@
     <t>05-050308A</t>
   </si>
   <si>
-    <t>ec4833957306512adf3cd6b652995fbb</t>
+    <t>5296f8a14708031cbb4605357cefad3c</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -920,7 +920,7 @@
     <t>05-050203TC</t>
   </si>
   <si>
-    <t>3ae605d2b3b9c02b245e347ef8d76cca</t>
+    <t>1c233742bac1e1822da8175ed997895e</t>
   </si>
   <si>
     <t>01-110304-11030404A</t>
@@ -950,7 +950,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>3baf8294f342ef57a23dda7f24b84723</t>
+    <t>dab12adcd4ed49832c26769dfc184eee</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -977,7 +977,7 @@
     <t>05-050303TC</t>
   </si>
   <si>
-    <t>df06acf56eb967b330d5b4c870ed029f</t>
+    <t>c8c118d80a2faed223eb06df3af69849</t>
   </si>
   <si>
     <t>01-010010TP</t>
@@ -995,7 +995,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>f8821589ef5fdd9120fbd2aff304eec0</t>
+    <t>bbf014442ec7342f24a53f458de5ad7e</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1040,7 +1040,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>451d116ee64b5aa6bf3d70e50dc98460</t>
+    <t>2da1fe0de84631b48d3a06e374457a98</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1082,7 +1082,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>7c81ed8327f94681ddb71d7a034dd2ae</t>
+    <t>41f45a9006ca64465dcc261596a96597</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1091,7 +1091,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>781bbd8f0bd4f4011ad0c5aa657b3dfd</t>
+    <t>99e3a3c99b1a18803949cf311cddee9b</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1160,7 +1160,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>f148727e7d1763d473f4e7d50a0d0537</t>
+    <t>3d71c1a01703991aa2e798cd69cc83fd</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1205,7 +1205,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>fef84f93db9651d6600d6c8a708afce2</t>
+    <t>9b9c5ad6d08999ce87b5a3fb29e233e1</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1223,7 +1223,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>0f005e63dde286f8e3058b771f9337b8</t>
+    <t>a8a5934b9fbb7f8a3af7943abe7151a7</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1235,19 +1235,19 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>c980546ac28c1898ef8532c6ac4dd9ad</t>
+    <t>47a95099f630a3c583fbf39b74203835</t>
   </si>
   <si>
     <t>05-050304A</t>
   </si>
   <si>
-    <t>e876d5ecab2c294d26cd82e36841d4e1</t>
+    <t>298f515debba9a5401523ba659a476b7</t>
   </si>
   <si>
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>d10fec61808a7040d47b8ca917d63023</t>
+    <t>b49f57b75c313ea891009b54356d4dc7</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1265,7 +1265,7 @@
     <t>05-050205TC</t>
   </si>
   <si>
-    <t>136010479b81bec4839cd44ca875e0da</t>
+    <t>6ddc9e616f4e07a473378ab68070f8b6</t>
   </si>
   <si>
     <t>04-040014TM</t>
@@ -1334,7 +1334,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>59e2c60c299b11bf1878b7c12928704b</t>
+    <t>ea63104c284ba92d83bc28f5d4b4d0fa</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1493,7 +1493,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>24268ba88e2f55a73e6dcfc6688432f6</t>
+    <t>dec5f47ae10b79faf1426a61aa8f8f71</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1523,7 +1523,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>a35b6184d00322ac983d6e46c8d3b739</t>
+    <t>1ff49cc2cabbac71112c2dd8e1e07df9</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1592,7 +1592,7 @@
     <t>05-050310TC</t>
   </si>
   <si>
-    <t>1adcf6dd01531097255d81652cf0e496</t>
+    <t>c805972242716513bfadad06ca579d42</t>
   </si>
   <si>
     <t>04-040004A</t>
@@ -1628,7 +1628,7 @@
     <t>03-030072TP</t>
   </si>
   <si>
-    <t>4183ab0db7a08c682ce11ed5151a5865</t>
+    <t>350988c015adaef798f9ca27e0db87e2</t>
   </si>
   <si>
     <t>01-080101-010082TC</t>
@@ -1640,7 +1640,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>f38ff71b4069d32deb4b7efc6c9a494b</t>
+    <t>e8a4f4a4c128ff1c4f80285ebd76cd83</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1796,7 +1796,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>a76262f09e2bababef10048b7cf6b52e</t>
+    <t>88c2c435c6884dbc5cd8eee399a772bd</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -1820,7 +1820,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>521a1ea2b471158f05007f3d14e8a0ec</t>
+    <t>ba89fa237d3c1de83be112506073ffef</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2192,7 +2192,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>f32ef20998e148a5e83300b518f8b8aa</t>
+    <t>71eb7d279df1c426c1fd315939e79c4c</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2237,7 +2237,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2375,7 +2375,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>5f3bede9bc5494fbe250853461b17ef7</t>
+    <t>6b59dffa6a9d25921f97bf229d443f9f</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2447,7 +2447,7 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>8457a07139e24db019e8d6df63ad2827</t>
+    <t>a59190224bf106fc2b4489a4cecd3308</t>
   </si>
   <si>
     <t>05-050313A</t>
@@ -2546,7 +2546,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>d1f78befcbb5ec95525e4a7383c40a3d</t>
+    <t>1fae6ea99358972b39c639786ee95090</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2558,7 +2558,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>875fe72072dbc895784a534a5d3e2e28</t>
+    <t>268ccf6c135c07df6ef7a32de07d76ac</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2639,7 +2639,7 @@
     <t>05-050208TC</t>
   </si>
   <si>
-    <t>e4d54b20b5600dd1d55880b751fe0a3b</t>
+    <t>40dbccc2a205d1183f72c8ebda232d7f</t>
   </si>
   <si>
     <t>03-030039A</t>
@@ -2690,7 +2690,7 @@
     <t>05-050311A</t>
   </si>
   <si>
-    <t>78f5ced1ce911714c84b05d6a2f92c45</t>
+    <t>8167a2ba8c125857267cd07e5e751176</t>
   </si>
   <si>
     <t>05-050208TP</t>
@@ -2720,7 +2720,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>d187e98f94589cff4479a0c30e4cbae3</t>
+    <t>3fb67e4334b5f14ec0e6abda6406aea5</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -2759,25 +2759,25 @@
     <t>05-050317TC</t>
   </si>
   <si>
-    <t>de3989494a8d80f0e897ec548840e892</t>
+    <t>247d2893ef57beb94920af4c3a13268b</t>
   </si>
   <si>
     <t>05-050312A</t>
   </si>
   <si>
-    <t>85b414f65cb310bc02d3b5a8d2e6aafa</t>
+    <t>6838da6c280e0c020cdff659201a38a8</t>
   </si>
   <si>
     <t>05-050009A</t>
   </si>
   <si>
-    <t>19ecefd17ffd2ecb988508254d964af1</t>
+    <t>23d15f1cb493200890169d571862b78c</t>
   </si>
   <si>
     <t>05-050203A</t>
   </si>
   <si>
-    <t>6bafa4222fcfa731ffc89cbcf0a38cdd</t>
+    <t>d0635cb66a53dc8f3f496b0b48204ebb</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -2816,7 +2816,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>db8b3e160875855515bd36f32b37d052</t>
+    <t>6db229385d7a332619d838a619ce1f0e</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -2933,7 +2933,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>ce7ffbd88adb00583fb4e8593eff66d7</t>
+    <t>d68016c2360cfba9cc7bb1fa05b2fcc8</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -2951,7 +2951,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>6fcb97b4a576ce03922c3902ff5a16f1</t>
+    <t>6951d41d22924c7ab8b3bf00c598385c</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3026,7 +3026,7 @@
     <t>05-050308TC</t>
   </si>
   <si>
-    <t>bcf4be1647d201974f4b0c9ee489295f</t>
+    <t>dcfb9e42e10397fd09d545a4970f1e03</t>
   </si>
   <si>
     <t>02-020002TC</t>
@@ -3044,7 +3044,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>dfc4f7a6e509488ca6dd55ea25e4f67d</t>
+    <t>39034531c7e1e066474fb27a4e884d31</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3080,7 +3080,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>0fd199be6f4b0c11ad5b1d17d6cf4ee2</t>
+    <t>b7ba5a35fae68f25ce43ece6d5c66757</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3152,7 +3152,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>566462fd282551480d244a97e19df41f</t>
+    <t>c6e78183b43f39189efec6685703a997</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3311,7 +3311,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>04d4a4dde888ace96511377acc86d18e</t>
+    <t>273130e8155c20a2a805533d4dc27d6c</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3365,7 +3365,7 @@
     <t>05-050204TC</t>
   </si>
   <si>
-    <t>339e16d77d46a0c02df06e6b09cd300e</t>
+    <t>4b37fefbeb61c67215325e4cb59935e5</t>
   </si>
   <si>
     <t>04-040015TM</t>
@@ -3401,7 +3401,7 @@
     <t>05-050302TC</t>
   </si>
   <si>
-    <t>8221a623c2222a4c1107cf2575720ec5</t>
+    <t>d7b63d0c5ead8ea370338c4af7bf8d19</t>
   </si>
   <si>
     <t>01-110304-11030403TP</t>
@@ -3554,7 +3554,7 @@
     <t>05-050317A</t>
   </si>
   <si>
-    <t>1120433771da77469c9c1baa4818b120</t>
+    <t>60ada143f9042a8d096218e39f0248a2</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -3620,7 +3620,7 @@
     <t>05-050206TP</t>
   </si>
   <si>
-    <t>5cbdd52c76a3a7656bd66c1706434ebc</t>
+    <t>5c55b7bf12ff4456e1b8aedb2f4c8985</t>
   </si>
   <si>
     <t>01-010068TM</t>
@@ -3644,7 +3644,7 @@
     <t>05-050206TC</t>
   </si>
   <si>
-    <t>2182b10777082951959b97d7584fdc12</t>
+    <t>fe3f06501ddafceab9b092665cc20436</t>
   </si>
   <si>
     <t>04-040013TM</t>
@@ -3728,7 +3728,7 @@
     <t>05-050304TC</t>
   </si>
   <si>
-    <t>1244be0c3cb0fd8401423484ea23db4e</t>
+    <t>22c2b281c13284cc6f284ed199446070</t>
   </si>
   <si>
     <t>03-030043TP</t>
@@ -3740,13 +3740,13 @@
     <t>05-050206A</t>
   </si>
   <si>
-    <t>9b2c0f7d69eb2c153cbc54c17dd014d4</t>
+    <t>46ec2f9ea6517760035a3563ebcad0a2</t>
   </si>
   <si>
     <t>05-050315A</t>
   </si>
   <si>
-    <t>9f197d1576d87a37f72bad3a0091e36e</t>
+    <t>dd9e1c5e0bd7764c6d92dab6d071c342</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -3809,7 +3809,7 @@
     <t>05-050304TP</t>
   </si>
   <si>
-    <t>e325ac58d2c018c05398370c6aa8b454</t>
+    <t>7646562564e2afd2dc47e0c7fdbb92f2</t>
   </si>
   <si>
     <t>04-040002TP</t>
@@ -3857,7 +3857,7 @@
     <t>05-050315TC</t>
   </si>
   <si>
-    <t>18b5b6b7843e3a0c6b5e24f7bb284379</t>
+    <t>5be32278080156c5a60a9623e20d69bc</t>
   </si>
   <si>
     <t>01-010046TM</t>
@@ -3872,7 +3872,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>04737aab45fd06f3fd0b30259466fa71</t>
+    <t>cd44ce05963049fb11b16ca8c418e68f</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -3896,7 +3896,7 @@
     <t>05-050207A</t>
   </si>
   <si>
-    <t>e9fb843323e7e79fdc96daf231e22da8</t>
+    <t>8e89956ea9346583179bddb29fe7a67c</t>
   </si>
   <si>
     <t>02-020006TM</t>
@@ -3947,7 +3947,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>2000fef9b593309d512616c5c0518c00</t>
+    <t>d47eca90d0b1c581bd5adaebabed648f</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4019,7 +4019,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>d7f617917143389b639634a39c04c3ce</t>
+    <t>dccb20dfef28d5ed895d63f8f7e04400</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4040,13 +4040,13 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>f210143051871837bfc6627dd7c56325</t>
+    <t>f18f536e3de80068df632cfe33f3bb03</t>
   </si>
   <si>
     <t>03-030072A</t>
   </si>
   <si>
-    <t>847ed2a86541d7dff12a22c185cc5e4f</t>
+    <t>fdcf1341c4940500bc3314e7d423c93f</t>
   </si>
   <si>
     <t>04-040019TC</t>
@@ -4169,7 +4169,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>c8542c3fc14549a882ce5868fc05d872</t>
+    <t>8a04a9aa62ef3df9bf6a9a7eb767d24e</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4379,7 +4379,7 @@
     <t>05-050202TC</t>
   </si>
   <si>
-    <t>770fdb1cec3a9e3293ed5272c64ca9f1</t>
+    <t>f9c83da9342f98d4e01c32045e4cd7a5</t>
   </si>
   <si>
     <t>03-030062TP</t>
@@ -4397,7 +4397,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>6d6b70f832a931acc0f79c7ea4fa0815</t>
+    <t>95934d6fd05c3c25aef4d88585311d0c</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4424,7 +4424,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>1da3972a2a795ae38fdc7cf064ae3495</t>
+    <t>94f8b627ca292ce8f5f6a87cdbae9a88</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -4523,13 +4523,13 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>3bbb92af73a72d21d7d114abb9b296f8</t>
+    <t>33d9ff0211090157d1fe1c44163c8c81</t>
   </si>
   <si>
     <t>05-050002A</t>
   </si>
   <si>
-    <t>37bc8746756aee4c57f645530b894c71</t>
+    <t>97a4b71c619267fbc7a432e40b572498</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4559,7 +4559,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>471f5dcc4254d33acd91db30453b5cd5</t>
+    <t>dc081dbe79b68938b1d983e668aeb2a0</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -4586,7 +4586,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>35f46cc2fe6a73572aca4c48470db552</t>
+    <t>ca5323dc83c80c367335e59fb001f277</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4790,7 +4790,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>48240156f8a81f6de60a53a6f7fafed1</t>
+    <t>41db3c4839784cf4d3b168511e209381</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -4925,7 +4925,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>202098ad51d2c394cf99d44d4e81b2b5</t>
+    <t>3e9e213a9d032a3e59a0992b563250a8</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar nov 23 05:24:47 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -152,7 +152,7 @@
     <t>05-050316TC</t>
   </si>
   <si>
-    <t>3962fd7b709886f150bd31bb3b07ca9e</t>
+    <t>7174e6b3cf9fa37bacae7ad6c81246c8</t>
   </si>
   <si>
     <t>03-030059TP</t>
@@ -182,7 +182,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>3ab600f8362b7bcfde638b88e63a8edf</t>
+    <t>9768a0c89cf9a4d0e4eb049cf1e10e50</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -2684,7 +2684,7 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>0469b64bb08b560959c1a4b120224755</t>
+    <t>1f1fee98b33e14a4c767eea7088d4d1a</t>
   </si>
   <si>
     <t>05-050311A</t>
@@ -2696,7 +2696,7 @@
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>4eedab6b746da735ee74177a709f6dbe</t>
+    <t>efbd23f4219cad75c5dcd48237a79503</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -3374,7 +3374,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>83753fff470acdb2d7675839e5d94a25</t>
+    <t>f91da0bd70bc4b36583b401d3391f1a5</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3548,7 +3548,7 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>32af589514444a64350b4c5fbc8493d6</t>
+    <t>03b7accc98cca16374adda1ddc340b24</t>
   </si>
   <si>
     <t>05-050317A</t>
@@ -4331,7 +4331,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>a32272aa3859c328aa744788c8f65243</t>
+    <t>8ca78fda18656c861cebf50c49ec0829</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>

</xml_diff>